<commit_message>
Sorvete: variacao passa a ser de um dia para o outro
Era primeiro dia da serie contra o ultimo, o que respondia "mudou quanto em
14 dias". O que interessa e o que mudou de ontem para hoje, entao agora a
coluna compara sempre os DOIS ULTIMOS dias. O titulo diz quais sao.

Exemplo do efeito: RJ aparecia como +8 (58 em 25/09 contra 66 em 08/10) e
agora aparece como -5 (71 em 07/10 contra 66 em 08/10). O segundo e o numero
que importa no dia a dia.

Tirei tambem o bloco de resumo embaixo da tabela (SOS, ALTO, fechados,
abertos, saldo, provaveis resolvidos, lojas paradas): o Christian pediu so a
tabela por regional. Sai do gerador, entao some do painel e do xlsx ao mesmo
tempo -- uma fonte so.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -284,7 +284,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 08/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 08/10 · variação 07/10 → 08/10</t>
         </is>
       </c>
     </row>
@@ -419,8 +419,8 @@
       <c r="O4" s="37">
         <v>66</v>
       </c>
-      <c r="P4" s="34">
-        <v>8</v>
+      <c r="P4" s="35">
+        <v>-5</v>
       </c>
     </row>
     <row r="5">
@@ -472,7 +472,7 @@
         <v>39</v>
       </c>
       <c r="P5" s="35">
-        <v>-12</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="6">
@@ -524,7 +524,7 @@
         <v>28</v>
       </c>
       <c r="P6" s="34">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -575,8 +575,8 @@
       <c r="O7" s="37">
         <v>28</v>
       </c>
-      <c r="P7" s="35">
-        <v>-9</v>
+      <c r="P7" s="34">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -627,8 +627,8 @@
       <c r="O8" s="37">
         <v>18</v>
       </c>
-      <c r="P8" s="35">
-        <v>-14</v>
+      <c r="P8" s="36">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -679,8 +679,8 @@
       <c r="O9" s="37">
         <v>18</v>
       </c>
-      <c r="P9" s="35">
-        <v>-14</v>
+      <c r="P9" s="36">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -732,7 +732,7 @@
         <v>11</v>
       </c>
       <c r="P10" s="34">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -784,7 +784,7 @@
         <v>7</v>
       </c>
       <c r="P11" s="35">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="12">
@@ -836,7 +836,7 @@
         <v>7</v>
       </c>
       <c r="P12" s="35">
-        <v>-6</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="13">
@@ -887,8 +887,8 @@
       <c r="O13" s="37">
         <v>6</v>
       </c>
-      <c r="P13" s="35">
-        <v>-15</v>
+      <c r="P13" s="34">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -939,8 +939,8 @@
       <c r="O14" s="37">
         <v>4</v>
       </c>
-      <c r="P14" s="35">
-        <v>-2</v>
+      <c r="P14" s="34">
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -992,467 +992,7 @@
         <v>232</v>
       </c>
       <c r="P15" s="35">
-        <v>-56</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="B16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="L16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="P16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOS abertos</t>
-        </is>
-      </c>
-      <c r="B17" s="36">
-        <v>177</v>
-      </c>
-      <c r="C17" s="36">
-        <v>169</v>
-      </c>
-      <c r="D17" s="36">
-        <v>157</v>
-      </c>
-      <c r="E17" s="36">
-        <v>151</v>
-      </c>
-      <c r="F17" s="36">
-        <v>145</v>
-      </c>
-      <c r="G17" s="36">
-        <v>143</v>
-      </c>
-      <c r="H17" s="36">
-        <v>146</v>
-      </c>
-      <c r="I17" s="36">
-        <v>142</v>
-      </c>
-      <c r="J17" s="36">
-        <v>142</v>
-      </c>
-      <c r="K17" s="36">
-        <v>153</v>
-      </c>
-      <c r="L17" s="36">
-        <v>156</v>
-      </c>
-      <c r="M17" s="36">
-        <v>149</v>
-      </c>
-      <c r="N17" s="36">
-        <v>147</v>
-      </c>
-      <c r="O17" s="37">
-        <v>150</v>
-      </c>
-      <c r="P17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTO abertos</t>
-        </is>
-      </c>
-      <c r="B18" s="36">
-        <v>111</v>
-      </c>
-      <c r="C18" s="36">
-        <v>112</v>
-      </c>
-      <c r="D18" s="36">
-        <v>111</v>
-      </c>
-      <c r="E18" s="36">
-        <v>108</v>
-      </c>
-      <c r="F18" s="36">
-        <v>103</v>
-      </c>
-      <c r="G18" s="36">
-        <v>104</v>
-      </c>
-      <c r="H18" s="36">
-        <v>96</v>
-      </c>
-      <c r="I18" s="36">
-        <v>90</v>
-      </c>
-      <c r="J18" s="36">
-        <v>93</v>
-      </c>
-      <c r="K18" s="36">
-        <v>94</v>
-      </c>
-      <c r="L18" s="36">
-        <v>92</v>
-      </c>
-      <c r="M18" s="36">
-        <v>88</v>
-      </c>
-      <c r="N18" s="36">
-        <v>89</v>
-      </c>
-      <c r="O18" s="37">
-        <v>82</v>
-      </c>
-      <c r="P18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fechados no dia</t>
-        </is>
-      </c>
-      <c r="B19" s="36">
-        <v>29</v>
-      </c>
-      <c r="C19" s="36">
-        <v>38</v>
-      </c>
-      <c r="D19" s="36">
-        <v>21</v>
-      </c>
-      <c r="E19" s="36">
-        <v>32</v>
-      </c>
-      <c r="F19" s="36">
-        <v>43</v>
-      </c>
-      <c r="G19" s="36">
-        <v>36</v>
-      </c>
-      <c r="H19" s="36">
-        <v>40</v>
-      </c>
-      <c r="I19" s="36">
-        <v>36</v>
-      </c>
-      <c r="J19" s="36">
-        <v>25</v>
-      </c>
-      <c r="K19" s="36">
-        <v>9</v>
-      </c>
-      <c r="L19" s="36">
-        <v>30</v>
-      </c>
-      <c r="M19" s="36">
-        <v>31</v>
-      </c>
-      <c r="N19" s="36">
-        <v>34</v>
-      </c>
-      <c r="O19" s="37">
-        <v>38</v>
-      </c>
-      <c r="P19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Abertos no dia</t>
-        </is>
-      </c>
-      <c r="B20" s="36">
-        <v>30</v>
-      </c>
-      <c r="C20" s="36">
-        <v>31</v>
-      </c>
-      <c r="D20" s="36">
-        <v>8</v>
-      </c>
-      <c r="E20" s="36">
-        <v>23</v>
-      </c>
-      <c r="F20" s="36">
-        <v>32</v>
-      </c>
-      <c r="G20" s="36">
-        <v>35</v>
-      </c>
-      <c r="H20" s="36">
-        <v>35</v>
-      </c>
-      <c r="I20" s="36">
-        <v>26</v>
-      </c>
-      <c r="J20" s="36">
-        <v>28</v>
-      </c>
-      <c r="K20" s="36">
-        <v>21</v>
-      </c>
-      <c r="L20" s="36">
-        <v>31</v>
-      </c>
-      <c r="M20" s="36">
-        <v>20</v>
-      </c>
-      <c r="N20" s="36">
-        <v>33</v>
-      </c>
-      <c r="O20" s="37">
-        <v>34</v>
-      </c>
-      <c r="P20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saldo do dia</t>
-        </is>
-      </c>
-      <c r="B21" s="36">
-        <v>-1</v>
-      </c>
-      <c r="C21" s="36">
-        <v>7</v>
-      </c>
-      <c r="D21" s="36">
-        <v>13</v>
-      </c>
-      <c r="E21" s="36">
-        <v>9</v>
-      </c>
-      <c r="F21" s="36">
-        <v>11</v>
-      </c>
-      <c r="G21" s="36">
-        <v>1</v>
-      </c>
-      <c r="H21" s="36">
-        <v>5</v>
-      </c>
-      <c r="I21" s="36">
-        <v>10</v>
-      </c>
-      <c r="J21" s="36">
-        <v>-3</v>
-      </c>
-      <c r="K21" s="36">
-        <v>-12</v>
-      </c>
-      <c r="L21" s="36">
-        <v>-1</v>
-      </c>
-      <c r="M21" s="36">
-        <v>11</v>
-      </c>
-      <c r="N21" s="36">
-        <v>1</v>
-      </c>
-      <c r="O21" s="37">
-        <v>4</v>
-      </c>
-      <c r="P21" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Provavelmente resolvidos</t>
-        </is>
-      </c>
-      <c r="B22" s="36">
-        <v>148</v>
-      </c>
-      <c r="C22" s="36">
-        <v>137</v>
-      </c>
-      <c r="D22" s="36">
-        <v>128</v>
-      </c>
-      <c r="E22" s="36">
-        <v>123</v>
-      </c>
-      <c r="F22" s="36">
-        <v>117</v>
-      </c>
-      <c r="G22" s="36">
-        <v>117</v>
-      </c>
-      <c r="H22" s="36">
-        <v>116</v>
-      </c>
-      <c r="I22" s="36">
-        <v>112</v>
-      </c>
-      <c r="J22" s="36">
-        <v>109</v>
-      </c>
-      <c r="K22" s="36">
-        <v>115</v>
-      </c>
-      <c r="L22" s="36">
-        <v>116</v>
-      </c>
-      <c r="M22" s="36">
-        <v>115</v>
-      </c>
-      <c r="N22" s="36">
-        <v>114</v>
-      </c>
-      <c r="O22" s="37">
-        <v>116</v>
-      </c>
-      <c r="P22" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lojas 100% paradas</t>
-        </is>
-      </c>
-      <c r="B23" s="36">
-        <v>18</v>
-      </c>
-      <c r="C23" s="36">
-        <v>17</v>
-      </c>
-      <c r="D23" s="36">
-        <v>16</v>
-      </c>
-      <c r="E23" s="36">
-        <v>17</v>
-      </c>
-      <c r="F23" s="36">
-        <v>16</v>
-      </c>
-      <c r="G23" s="36">
-        <v>14</v>
-      </c>
-      <c r="H23" s="36">
-        <v>14</v>
-      </c>
-      <c r="I23" s="36">
-        <v>13</v>
-      </c>
-      <c r="J23" s="36">
-        <v>15</v>
-      </c>
-      <c r="K23" s="36">
-        <v>15</v>
-      </c>
-      <c r="L23" s="36">
-        <v>15</v>
-      </c>
-      <c r="M23" s="36">
-        <v>13</v>
-      </c>
-      <c r="N23" s="36">
-        <v>13</v>
-      </c>
-      <c r="O23" s="37">
-        <v>10</v>
-      </c>
-      <c r="P23" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+        <v>-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sorvete: Variacao vira formula e o bloco de resumo volta
Formula, nao numero: a coluna Variacao agora e =O{linha}-N{linha}, entre as
duas ultimas colunas de dia. Assim, se alguem mexer num valor, a variacao
acompanha. Pedido do Christian.

Armadilha paga aqui: no xlsx o elemento <f> guarda SO a expressao. Gravei
"=O4-N4" na primeira tentativa e o Excel recusaria a formula. Agora vai
"O4-N4".

O bloco de resumo (SOS, ALTO, fechados, abertos, saldo, provaveis resolvidos,
lojas paradas) voltou -- eu tinha tirado por ter lido mal um pedido. Ele
esconde no Excel as linhas que nao usa; esconder e decisao dele.

Dois estilos novos para a Variacao na linha do TOTAL: cor de texto com fundo
cinza, senao a faixa cinza do total quebrava bem na celula que ele mais olha.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf xfId="0" borderId="1" applyBorder="1"/>
     <xf xfId="0" fontId="1" fillId="2" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -247,6 +247,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" fontId="4" fillId="7" borderId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf xfId="0" fontId="14" fillId="7" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" fontId="15" fillId="7" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
@@ -420,7 +426,7 @@
         <v>66</v>
       </c>
       <c r="P4" s="35">
-        <v>-5</v>
+        <f>O4-N4</f>
       </c>
     </row>
     <row r="5">
@@ -472,7 +478,7 @@
         <v>39</v>
       </c>
       <c r="P5" s="35">
-        <v>-2</v>
+        <f>O5-N5</f>
       </c>
     </row>
     <row r="6">
@@ -524,7 +530,7 @@
         <v>28</v>
       </c>
       <c r="P6" s="34">
-        <v>4</v>
+        <f>O6-N6</f>
       </c>
     </row>
     <row r="7">
@@ -576,7 +582,7 @@
         <v>28</v>
       </c>
       <c r="P7" s="34">
-        <v>2</v>
+        <f>O7-N7</f>
       </c>
     </row>
     <row r="8">
@@ -628,7 +634,7 @@
         <v>18</v>
       </c>
       <c r="P8" s="36">
-        <v>0</v>
+        <f>O8-N8</f>
       </c>
     </row>
     <row r="9">
@@ -680,7 +686,7 @@
         <v>18</v>
       </c>
       <c r="P9" s="36">
-        <v>0</v>
+        <f>O9-N9</f>
       </c>
     </row>
     <row r="10">
@@ -732,7 +738,7 @@
         <v>11</v>
       </c>
       <c r="P10" s="34">
-        <v>3</v>
+        <f>O10-N10</f>
       </c>
     </row>
     <row r="11">
@@ -784,7 +790,7 @@
         <v>7</v>
       </c>
       <c r="P11" s="35">
-        <v>-4</v>
+        <f>O11-N11</f>
       </c>
     </row>
     <row r="12">
@@ -836,7 +842,7 @@
         <v>7</v>
       </c>
       <c r="P12" s="35">
-        <v>-5</v>
+        <f>O12-N12</f>
       </c>
     </row>
     <row r="13">
@@ -888,7 +894,7 @@
         <v>6</v>
       </c>
       <c r="P13" s="34">
-        <v>1</v>
+        <f>O13-N13</f>
       </c>
     </row>
     <row r="14">
@@ -940,7 +946,7 @@
         <v>4</v>
       </c>
       <c r="P14" s="34">
-        <v>2</v>
+        <f>O14-N14</f>
       </c>
     </row>
     <row r="15">
@@ -991,8 +997,468 @@
       <c r="O15" s="38">
         <v>232</v>
       </c>
-      <c r="P15" s="35">
-        <v>-4</v>
+      <c r="P15" s="41">
+        <f>O15-N15</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SOS abertos</t>
+        </is>
+      </c>
+      <c r="B17" s="36">
+        <v>177</v>
+      </c>
+      <c r="C17" s="36">
+        <v>169</v>
+      </c>
+      <c r="D17" s="36">
+        <v>157</v>
+      </c>
+      <c r="E17" s="36">
+        <v>151</v>
+      </c>
+      <c r="F17" s="36">
+        <v>145</v>
+      </c>
+      <c r="G17" s="36">
+        <v>143</v>
+      </c>
+      <c r="H17" s="36">
+        <v>146</v>
+      </c>
+      <c r="I17" s="36">
+        <v>142</v>
+      </c>
+      <c r="J17" s="36">
+        <v>142</v>
+      </c>
+      <c r="K17" s="36">
+        <v>153</v>
+      </c>
+      <c r="L17" s="36">
+        <v>156</v>
+      </c>
+      <c r="M17" s="36">
+        <v>149</v>
+      </c>
+      <c r="N17" s="36">
+        <v>147</v>
+      </c>
+      <c r="O17" s="37">
+        <v>150</v>
+      </c>
+      <c r="P17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTO abertos</t>
+        </is>
+      </c>
+      <c r="B18" s="36">
+        <v>111</v>
+      </c>
+      <c r="C18" s="36">
+        <v>112</v>
+      </c>
+      <c r="D18" s="36">
+        <v>111</v>
+      </c>
+      <c r="E18" s="36">
+        <v>108</v>
+      </c>
+      <c r="F18" s="36">
+        <v>103</v>
+      </c>
+      <c r="G18" s="36">
+        <v>104</v>
+      </c>
+      <c r="H18" s="36">
+        <v>96</v>
+      </c>
+      <c r="I18" s="36">
+        <v>90</v>
+      </c>
+      <c r="J18" s="36">
+        <v>93</v>
+      </c>
+      <c r="K18" s="36">
+        <v>94</v>
+      </c>
+      <c r="L18" s="36">
+        <v>92</v>
+      </c>
+      <c r="M18" s="36">
+        <v>88</v>
+      </c>
+      <c r="N18" s="36">
+        <v>89</v>
+      </c>
+      <c r="O18" s="37">
+        <v>82</v>
+      </c>
+      <c r="P18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fechados no dia</t>
+        </is>
+      </c>
+      <c r="B19" s="36">
+        <v>29</v>
+      </c>
+      <c r="C19" s="36">
+        <v>38</v>
+      </c>
+      <c r="D19" s="36">
+        <v>21</v>
+      </c>
+      <c r="E19" s="36">
+        <v>32</v>
+      </c>
+      <c r="F19" s="36">
+        <v>43</v>
+      </c>
+      <c r="G19" s="36">
+        <v>36</v>
+      </c>
+      <c r="H19" s="36">
+        <v>40</v>
+      </c>
+      <c r="I19" s="36">
+        <v>36</v>
+      </c>
+      <c r="J19" s="36">
+        <v>25</v>
+      </c>
+      <c r="K19" s="36">
+        <v>9</v>
+      </c>
+      <c r="L19" s="36">
+        <v>30</v>
+      </c>
+      <c r="M19" s="36">
+        <v>31</v>
+      </c>
+      <c r="N19" s="36">
+        <v>34</v>
+      </c>
+      <c r="O19" s="37">
+        <v>38</v>
+      </c>
+      <c r="P19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abertos no dia</t>
+        </is>
+      </c>
+      <c r="B20" s="36">
+        <v>30</v>
+      </c>
+      <c r="C20" s="36">
+        <v>31</v>
+      </c>
+      <c r="D20" s="36">
+        <v>8</v>
+      </c>
+      <c r="E20" s="36">
+        <v>23</v>
+      </c>
+      <c r="F20" s="36">
+        <v>32</v>
+      </c>
+      <c r="G20" s="36">
+        <v>35</v>
+      </c>
+      <c r="H20" s="36">
+        <v>35</v>
+      </c>
+      <c r="I20" s="36">
+        <v>26</v>
+      </c>
+      <c r="J20" s="36">
+        <v>28</v>
+      </c>
+      <c r="K20" s="36">
+        <v>21</v>
+      </c>
+      <c r="L20" s="36">
+        <v>31</v>
+      </c>
+      <c r="M20" s="36">
+        <v>20</v>
+      </c>
+      <c r="N20" s="36">
+        <v>33</v>
+      </c>
+      <c r="O20" s="37">
+        <v>34</v>
+      </c>
+      <c r="P20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saldo do dia</t>
+        </is>
+      </c>
+      <c r="B21" s="36">
+        <v>-1</v>
+      </c>
+      <c r="C21" s="36">
+        <v>7</v>
+      </c>
+      <c r="D21" s="36">
+        <v>13</v>
+      </c>
+      <c r="E21" s="36">
+        <v>9</v>
+      </c>
+      <c r="F21" s="36">
+        <v>11</v>
+      </c>
+      <c r="G21" s="36">
+        <v>1</v>
+      </c>
+      <c r="H21" s="36">
+        <v>5</v>
+      </c>
+      <c r="I21" s="36">
+        <v>10</v>
+      </c>
+      <c r="J21" s="36">
+        <v>-3</v>
+      </c>
+      <c r="K21" s="36">
+        <v>-12</v>
+      </c>
+      <c r="L21" s="36">
+        <v>-1</v>
+      </c>
+      <c r="M21" s="36">
+        <v>11</v>
+      </c>
+      <c r="N21" s="36">
+        <v>1</v>
+      </c>
+      <c r="O21" s="37">
+        <v>4</v>
+      </c>
+      <c r="P21" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provavelmente resolvidos</t>
+        </is>
+      </c>
+      <c r="B22" s="36">
+        <v>148</v>
+      </c>
+      <c r="C22" s="36">
+        <v>137</v>
+      </c>
+      <c r="D22" s="36">
+        <v>128</v>
+      </c>
+      <c r="E22" s="36">
+        <v>123</v>
+      </c>
+      <c r="F22" s="36">
+        <v>117</v>
+      </c>
+      <c r="G22" s="36">
+        <v>117</v>
+      </c>
+      <c r="H22" s="36">
+        <v>116</v>
+      </c>
+      <c r="I22" s="36">
+        <v>112</v>
+      </c>
+      <c r="J22" s="36">
+        <v>109</v>
+      </c>
+      <c r="K22" s="36">
+        <v>115</v>
+      </c>
+      <c r="L22" s="36">
+        <v>116</v>
+      </c>
+      <c r="M22" s="36">
+        <v>115</v>
+      </c>
+      <c r="N22" s="36">
+        <v>114</v>
+      </c>
+      <c r="O22" s="37">
+        <v>116</v>
+      </c>
+      <c r="P22" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lojas 100% paradas</t>
+        </is>
+      </c>
+      <c r="B23" s="36">
+        <v>18</v>
+      </c>
+      <c r="C23" s="36">
+        <v>17</v>
+      </c>
+      <c r="D23" s="36">
+        <v>16</v>
+      </c>
+      <c r="E23" s="36">
+        <v>17</v>
+      </c>
+      <c r="F23" s="36">
+        <v>16</v>
+      </c>
+      <c r="G23" s="36">
+        <v>14</v>
+      </c>
+      <c r="H23" s="36">
+        <v>14</v>
+      </c>
+      <c r="I23" s="36">
+        <v>13</v>
+      </c>
+      <c r="J23" s="36">
+        <v>15</v>
+      </c>
+      <c r="K23" s="36">
+        <v>15</v>
+      </c>
+      <c r="L23" s="36">
+        <v>15</v>
+      </c>
+      <c r="M23" s="36">
+        <v>13</v>
+      </c>
+      <c r="N23" s="36">
+        <v>13</v>
+      </c>
+      <c r="O23" s="37">
+        <v>10</v>
+      </c>
+      <c r="P23" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sorvete: formula em tudo que soma, e 3 linhas a menos
TOTAL BRASIL agora e =SUM(B4:B14) em cada coluna de dia, nao numero cravado.
"Saldo do dia" virou =B17-B18 (fechados menos abertos). Total cravado e
divergencia esperando acontecer: se alguem corrige uma regional, o total
ficava mentindo sem avisar.

Fora, a pedido: "SOS abertos", "ALTO abertos" e "Provavelmente resolvidos".
O bloco de resumo fica com fechados no dia, abertos no dia, saldo do dia e
lojas 100% paradas.

Sai do gerador, entao some do painel e do xlsx junto -- uma fonte so.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -956,46 +956,46 @@
         </is>
       </c>
       <c r="B15" s="38">
-        <v>288</v>
+        <f>SUM(B4:B14)</f>
       </c>
       <c r="C15" s="38">
-        <v>281</v>
+        <f>SUM(C4:C14)</f>
       </c>
       <c r="D15" s="38">
-        <v>268</v>
+        <f>SUM(D4:D14)</f>
       </c>
       <c r="E15" s="38">
-        <v>259</v>
+        <f>SUM(E4:E14)</f>
       </c>
       <c r="F15" s="38">
-        <v>248</v>
+        <f>SUM(F4:F14)</f>
       </c>
       <c r="G15" s="38">
-        <v>247</v>
+        <f>SUM(G4:G14)</f>
       </c>
       <c r="H15" s="38">
-        <v>242</v>
+        <f>SUM(H4:H14)</f>
       </c>
       <c r="I15" s="38">
-        <v>232</v>
+        <f>SUM(I4:I14)</f>
       </c>
       <c r="J15" s="38">
-        <v>235</v>
+        <f>SUM(J4:J14)</f>
       </c>
       <c r="K15" s="38">
-        <v>247</v>
+        <f>SUM(K4:K14)</f>
       </c>
       <c r="L15" s="38">
-        <v>248</v>
+        <f>SUM(L4:L14)</f>
       </c>
       <c r="M15" s="38">
-        <v>237</v>
+        <f>SUM(M4:M14)</f>
       </c>
       <c r="N15" s="38">
-        <v>236</v>
+        <f>SUM(N4:N14)</f>
       </c>
       <c r="O15" s="38">
-        <v>232</v>
+        <f>SUM(O4:O14)</f>
       </c>
       <c r="P15" s="41">
         <f>O15-N15</f>
@@ -1086,50 +1086,50 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOS abertos</t>
+          <t xml:space="preserve">Fechados no dia</t>
         </is>
       </c>
       <c r="B17" s="36">
-        <v>177</v>
+        <v>29</v>
       </c>
       <c r="C17" s="36">
-        <v>169</v>
+        <v>38</v>
       </c>
       <c r="D17" s="36">
-        <v>157</v>
+        <v>21</v>
       </c>
       <c r="E17" s="36">
-        <v>151</v>
+        <v>32</v>
       </c>
       <c r="F17" s="36">
-        <v>145</v>
+        <v>43</v>
       </c>
       <c r="G17" s="36">
-        <v>143</v>
+        <v>36</v>
       </c>
       <c r="H17" s="36">
-        <v>146</v>
+        <v>40</v>
       </c>
       <c r="I17" s="36">
-        <v>142</v>
+        <v>36</v>
       </c>
       <c r="J17" s="36">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="K17" s="36">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="L17" s="36">
-        <v>156</v>
+        <v>30</v>
       </c>
       <c r="M17" s="36">
-        <v>149</v>
+        <v>31</v>
       </c>
       <c r="N17" s="36">
-        <v>147</v>
+        <v>34</v>
       </c>
       <c r="O17" s="37">
-        <v>150</v>
+        <v>38</v>
       </c>
       <c r="P17" s="36" t="inlineStr">
         <is>
@@ -1140,50 +1140,50 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTO abertos</t>
+          <t xml:space="preserve">Abertos no dia</t>
         </is>
       </c>
       <c r="B18" s="36">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="C18" s="36">
-        <v>112</v>
+        <v>31</v>
       </c>
       <c r="D18" s="36">
-        <v>111</v>
+        <v>8</v>
       </c>
       <c r="E18" s="36">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="F18" s="36">
-        <v>103</v>
+        <v>32</v>
       </c>
       <c r="G18" s="36">
-        <v>104</v>
+        <v>35</v>
       </c>
       <c r="H18" s="36">
-        <v>96</v>
+        <v>35</v>
       </c>
       <c r="I18" s="36">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="J18" s="36">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="K18" s="36">
-        <v>94</v>
+        <v>21</v>
       </c>
       <c r="L18" s="36">
-        <v>92</v>
+        <v>31</v>
       </c>
       <c r="M18" s="36">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="N18" s="36">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="O18" s="37">
-        <v>82</v>
+        <v>34</v>
       </c>
       <c r="P18" s="36" t="inlineStr">
         <is>
@@ -1194,50 +1194,50 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fechados no dia</t>
+          <t xml:space="preserve">Saldo do dia</t>
         </is>
       </c>
       <c r="B19" s="36">
-        <v>29</v>
+        <f>B17-B18</f>
       </c>
       <c r="C19" s="36">
-        <v>38</v>
+        <f>C17-C18</f>
       </c>
       <c r="D19" s="36">
-        <v>21</v>
+        <f>D17-D18</f>
       </c>
       <c r="E19" s="36">
-        <v>32</v>
+        <f>E17-E18</f>
       </c>
       <c r="F19" s="36">
-        <v>43</v>
+        <f>F17-F18</f>
       </c>
       <c r="G19" s="36">
-        <v>36</v>
+        <f>G17-G18</f>
       </c>
       <c r="H19" s="36">
-        <v>40</v>
+        <f>H17-H18</f>
       </c>
       <c r="I19" s="36">
-        <v>36</v>
+        <f>I17-I18</f>
       </c>
       <c r="J19" s="36">
-        <v>25</v>
+        <f>J17-J18</f>
       </c>
       <c r="K19" s="36">
-        <v>9</v>
+        <f>K17-K18</f>
       </c>
       <c r="L19" s="36">
-        <v>30</v>
+        <f>L17-L18</f>
       </c>
       <c r="M19" s="36">
-        <v>31</v>
+        <f>M17-M18</f>
       </c>
       <c r="N19" s="36">
-        <v>34</v>
+        <f>N17-N18</f>
       </c>
       <c r="O19" s="37">
-        <v>38</v>
+        <f>O17-O18</f>
       </c>
       <c r="P19" s="36" t="inlineStr">
         <is>
@@ -1248,214 +1248,52 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abertos no dia</t>
+          <t xml:space="preserve">Lojas 100% paradas</t>
         </is>
       </c>
       <c r="B20" s="36">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C20" s="36">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D20" s="36">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E20" s="36">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F20" s="36">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G20" s="36">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H20" s="36">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="I20" s="36">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="J20" s="36">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="K20" s="36">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="L20" s="36">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="M20" s="36">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="N20" s="36">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="O20" s="37">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="P20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saldo do dia</t>
-        </is>
-      </c>
-      <c r="B21" s="36">
-        <v>-1</v>
-      </c>
-      <c r="C21" s="36">
-        <v>7</v>
-      </c>
-      <c r="D21" s="36">
-        <v>13</v>
-      </c>
-      <c r="E21" s="36">
-        <v>9</v>
-      </c>
-      <c r="F21" s="36">
-        <v>11</v>
-      </c>
-      <c r="G21" s="36">
-        <v>1</v>
-      </c>
-      <c r="H21" s="36">
-        <v>5</v>
-      </c>
-      <c r="I21" s="36">
-        <v>10</v>
-      </c>
-      <c r="J21" s="36">
-        <v>-3</v>
-      </c>
-      <c r="K21" s="36">
-        <v>-12</v>
-      </c>
-      <c r="L21" s="36">
-        <v>-1</v>
-      </c>
-      <c r="M21" s="36">
-        <v>11</v>
-      </c>
-      <c r="N21" s="36">
-        <v>1</v>
-      </c>
-      <c r="O21" s="37">
-        <v>4</v>
-      </c>
-      <c r="P21" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Provavelmente resolvidos</t>
-        </is>
-      </c>
-      <c r="B22" s="36">
-        <v>148</v>
-      </c>
-      <c r="C22" s="36">
-        <v>137</v>
-      </c>
-      <c r="D22" s="36">
-        <v>128</v>
-      </c>
-      <c r="E22" s="36">
-        <v>123</v>
-      </c>
-      <c r="F22" s="36">
-        <v>117</v>
-      </c>
-      <c r="G22" s="36">
-        <v>117</v>
-      </c>
-      <c r="H22" s="36">
-        <v>116</v>
-      </c>
-      <c r="I22" s="36">
-        <v>112</v>
-      </c>
-      <c r="J22" s="36">
-        <v>109</v>
-      </c>
-      <c r="K22" s="36">
-        <v>115</v>
-      </c>
-      <c r="L22" s="36">
-        <v>116</v>
-      </c>
-      <c r="M22" s="36">
-        <v>115</v>
-      </c>
-      <c r="N22" s="36">
-        <v>114</v>
-      </c>
-      <c r="O22" s="37">
-        <v>116</v>
-      </c>
-      <c r="P22" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lojas 100% paradas</t>
-        </is>
-      </c>
-      <c r="B23" s="36">
-        <v>18</v>
-      </c>
-      <c r="C23" s="36">
-        <v>17</v>
-      </c>
-      <c r="D23" s="36">
-        <v>16</v>
-      </c>
-      <c r="E23" s="36">
-        <v>17</v>
-      </c>
-      <c r="F23" s="36">
-        <v>16</v>
-      </c>
-      <c r="G23" s="36">
-        <v>14</v>
-      </c>
-      <c r="H23" s="36">
-        <v>14</v>
-      </c>
-      <c r="I23" s="36">
-        <v>13</v>
-      </c>
-      <c r="J23" s="36">
-        <v>15</v>
-      </c>
-      <c r="K23" s="36">
-        <v>15</v>
-      </c>
-      <c r="L23" s="36">
-        <v>15</v>
-      </c>
-      <c r="M23" s="36">
-        <v>13</v>
-      </c>
-      <c r="N23" s="36">
-        <v>13</v>
-      </c>
-      <c r="O23" s="37">
-        <v>10</v>
-      </c>
-      <c r="P23" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: exclui 4 chamados do SUL abertos por engano em 08/10
Decisao do Christian em 09/10: WO0066460, WO0066314, WO0066287 e WO0066283
foram abertos indevidamente e nao representam equipamento parado. Ficam fora
da contagem ate alguem corrigir na origem.

Efeito: SUL 26 -> 24 (variacao -2, era +2). TOTAL BRASIL 236 -> 228 (-8).

COMO foi feito importa tanto quanto o que: a exclusao vive em exclusoes.json,
com numero, loja, motivo, quem decidiu e a data. NAO entra na formula. Numero
ajustado dentro de formula some de vista, contamina o SUM do total e nao deixa
rastro -- daqui a uma semana ninguem sabe qual coluna e real.

E ela APARECE: o titulo da aba lista os 4 numeros excluidos. Corte que nao se
ve e corte que engana.

O gerador reverifica a cada execucao e diz se o chamado continua aberto no
SOMA. Os 4 ainda estao "Pronto para Expedicao". Quando forem cancelados ou
fechados na origem, e so tirar da lista.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -290,7 +290,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 08/10 · variação 07/10 → 08/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 08/10 · variação 07/10 → 08/10 · 4 chamado(s) fora da conta por abertura indevida (WO0066460, WO0066314, WO0066287, WO0066283)</t>
         </is>
       </c>
     </row>
@@ -579,9 +579,9 @@
         <v>26</v>
       </c>
       <c r="O7" s="37">
-        <v>28</v>
-      </c>
-      <c r="P7" s="34">
+        <v>24</v>
+      </c>
+      <c r="P7" s="35">
         <f>O7-N7</f>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
         <v>33</v>
       </c>
       <c r="O18" s="37">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="P18" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sorvete: Saldo do dia passa a ter o mesmo sinal da Variacao
Estava como fechados menos abertos (38-30 = +8, positivo = bom), enquanto a
coluna Variacao logo acima e estoque de hoje menos o de ontem (228-236 = -8,
negativo = bom). Dois numeros do mesmo fato, com sinais opostos, um debaixo
do outro. O Christian tropecou nisso e tinha razao.

Agora e abertos menos fechados, com o rotulo dizendo a conta. Em 08/10 da -8,
igual a Variacao do TOTAL -- e isso vira conferencia embutida: se os dois
discordarem, tem erro em algum lugar.

A formula acompanhou: =O18-O17.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -1194,50 +1194,50 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saldo do dia</t>
+          <t xml:space="preserve">Saldo do dia (abertos − fechados)</t>
         </is>
       </c>
       <c r="B19" s="36">
-        <f>B17-B18</f>
+        <f>B18-B17</f>
       </c>
       <c r="C19" s="36">
-        <f>C17-C18</f>
+        <f>C18-C17</f>
       </c>
       <c r="D19" s="36">
-        <f>D17-D18</f>
+        <f>D18-D17</f>
       </c>
       <c r="E19" s="36">
-        <f>E17-E18</f>
+        <f>E18-E17</f>
       </c>
       <c r="F19" s="36">
-        <f>F17-F18</f>
+        <f>F18-F17</f>
       </c>
       <c r="G19" s="36">
-        <f>G17-G18</f>
+        <f>G18-G17</f>
       </c>
       <c r="H19" s="36">
-        <f>H17-H18</f>
+        <f>H18-H17</f>
       </c>
       <c r="I19" s="36">
-        <f>I17-I18</f>
+        <f>I18-I17</f>
       </c>
       <c r="J19" s="36">
-        <f>J17-J18</f>
+        <f>J18-J17</f>
       </c>
       <c r="K19" s="36">
-        <f>K17-K18</f>
+        <f>K18-K17</f>
       </c>
       <c r="L19" s="36">
-        <f>L17-L18</f>
+        <f>L18-L17</f>
       </c>
       <c r="M19" s="36">
-        <f>M17-M18</f>
+        <f>M18-M17</f>
       </c>
       <c r="N19" s="36">
-        <f>N17-N18</f>
+        <f>N18-N17</f>
       </c>
       <c r="O19" s="37">
-        <f>O17-O18</f>
+        <f>O18-O17</f>
       </c>
       <c r="P19" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sorvete: serie comeca no dia 1 do mes e ganha Variacao MES
Pedido do Christian. A tabela passa a cobrir o mes corrente (01/10 em diante)
em vez de 14 dias corridos, e sao duas colunas:

  Variacao DIA = ultimo dia menos o anterior      (=I4-H4)
  Variacao MES = ultimo dia menos o dia 1 do mes  (=I4-B4)

Quando o mes virar, a serie recomeca sozinha no novo dia 1 e a Variacao MES
passa a comparar com ele.

CONSERTO JUNTO: o gerador decidia o ultimo dia fechado como "ontem". A tarefa
roda as 23:59, entao nessa hora ela fechava 07/10 em vez de 08/10 -- a serie
ficaria um dia atrasada toda noite, sem erro nenhum aparecendo. Agora o
wrapper passa a data explicitamente, e o gerador so' chuta quando ninguem
informa (e aí usa a hora: >= 23h fecha o dia corrente).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -278,13 +278,7 @@
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="10" customWidth="1"/>
-    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -303,77 +297,52 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">25/09</t>
+          <t xml:space="preserve">01/10</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">26/09</t>
+          <t xml:space="preserve">02/10</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">27/09</t>
+          <t xml:space="preserve">03/10</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">28/09</t>
+          <t xml:space="preserve">04/10</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">29/09</t>
+          <t xml:space="preserve">05/10</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">30/09</t>
+          <t xml:space="preserve">06/10</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">01/10</t>
+          <t xml:space="preserve">07/10</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">02/10</t>
+          <t xml:space="preserve">08/10</t>
         </is>
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">03/10</t>
+          <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">04/10</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05/10</t>
-        </is>
-      </c>
-      <c r="M3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06/10</t>
-        </is>
-      </c>
-      <c r="N3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07/10</t>
-        </is>
-      </c>
-      <c r="O3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08/10</t>
-        </is>
-      </c>
-      <c r="P3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Variação</t>
+          <t xml:space="preserve">Variação MÊS</t>
         </is>
       </c>
     </row>
@@ -384,49 +353,34 @@
         </is>
       </c>
       <c r="B4" s="36">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C4" s="36">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="D4" s="36">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="E4" s="36">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="F4" s="36">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G4" s="36">
         <v>64</v>
       </c>
       <c r="H4" s="36">
-        <v>63</v>
-      </c>
-      <c r="I4" s="36">
-        <v>63</v>
-      </c>
-      <c r="J4" s="36">
-        <v>59</v>
-      </c>
-      <c r="K4" s="36">
-        <v>61</v>
-      </c>
-      <c r="L4" s="36">
+        <v>71</v>
+      </c>
+      <c r="I4" s="37">
         <v>66</v>
       </c>
-      <c r="M4" s="36">
-        <v>64</v>
-      </c>
-      <c r="N4" s="36">
-        <v>71</v>
-      </c>
-      <c r="O4" s="37">
-        <v>66</v>
-      </c>
-      <c r="P4" s="35">
-        <f>O4-N4</f>
+      <c r="J4" s="35">
+        <f>I4-H4</f>
+      </c>
+      <c r="K4" s="34">
+        <f>I4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -436,49 +390,34 @@
         </is>
       </c>
       <c r="B5" s="36">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C5" s="36">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D5" s="36">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E5" s="36">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F5" s="36">
         <v>42</v>
       </c>
       <c r="G5" s="36">
+        <v>45</v>
+      </c>
+      <c r="H5" s="36">
         <v>41</v>
       </c>
-      <c r="H5" s="36">
+      <c r="I5" s="37">
         <v>39</v>
       </c>
-      <c r="I5" s="36">
-        <v>39</v>
-      </c>
-      <c r="J5" s="36">
-        <v>44</v>
+      <c r="J5" s="35">
+        <f>I5-H5</f>
       </c>
       <c r="K5" s="36">
-        <v>43</v>
-      </c>
-      <c r="L5" s="36">
-        <v>42</v>
-      </c>
-      <c r="M5" s="36">
-        <v>45</v>
-      </c>
-      <c r="N5" s="36">
-        <v>41</v>
-      </c>
-      <c r="O5" s="37">
-        <v>39</v>
-      </c>
-      <c r="P5" s="35">
-        <f>O5-N5</f>
+        <f>I5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -488,49 +427,34 @@
         </is>
       </c>
       <c r="B6" s="36">
+        <v>23</v>
+      </c>
+      <c r="C6" s="36">
         <v>22</v>
       </c>
-      <c r="C6" s="36">
-        <v>21</v>
-      </c>
       <c r="D6" s="36">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" s="36">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" s="36">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G6" s="36">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H6" s="36">
-        <v>23</v>
-      </c>
-      <c r="I6" s="36">
-        <v>22</v>
-      </c>
-      <c r="J6" s="36">
-        <v>22</v>
-      </c>
-      <c r="K6" s="36">
-        <v>22</v>
-      </c>
-      <c r="L6" s="36">
-        <v>23</v>
-      </c>
-      <c r="M6" s="36">
-        <v>25</v>
-      </c>
-      <c r="N6" s="36">
         <v>24</v>
       </c>
-      <c r="O6" s="37">
+      <c r="I6" s="37">
         <v>28</v>
       </c>
-      <c r="P6" s="34">
-        <f>O6-N6</f>
+      <c r="J6" s="34">
+        <f>I6-H6</f>
+      </c>
+      <c r="K6" s="34">
+        <f>I6-B6</f>
       </c>
     </row>
     <row r="7">
@@ -540,49 +464,34 @@
         </is>
       </c>
       <c r="B7" s="36">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C7" s="36">
+        <v>32</v>
+      </c>
+      <c r="D7" s="36">
+        <v>32</v>
+      </c>
+      <c r="E7" s="36">
+        <v>34</v>
+      </c>
+      <c r="F7" s="36">
         <v>38</v>
       </c>
-      <c r="D7" s="36">
-        <v>35</v>
-      </c>
-      <c r="E7" s="36">
+      <c r="G7" s="36">
         <v>31</v>
       </c>
-      <c r="F7" s="36">
-        <v>32</v>
-      </c>
-      <c r="G7" s="36">
-        <v>34</v>
-      </c>
       <c r="H7" s="36">
-        <v>34</v>
-      </c>
-      <c r="I7" s="36">
-        <v>32</v>
-      </c>
-      <c r="J7" s="36">
-        <v>32</v>
-      </c>
-      <c r="K7" s="36">
-        <v>34</v>
-      </c>
-      <c r="L7" s="36">
-        <v>38</v>
-      </c>
-      <c r="M7" s="36">
-        <v>31</v>
-      </c>
-      <c r="N7" s="36">
         <v>26</v>
       </c>
-      <c r="O7" s="37">
+      <c r="I7" s="37">
         <v>24</v>
       </c>
-      <c r="P7" s="35">
-        <f>O7-N7</f>
+      <c r="J7" s="35">
+        <f>I7-H7</f>
+      </c>
+      <c r="K7" s="35">
+        <f>I7-B7</f>
       </c>
     </row>
     <row r="8">
@@ -592,49 +501,34 @@
         </is>
       </c>
       <c r="B8" s="36">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="C8" s="36">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D8" s="36">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E8" s="36">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F8" s="36">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G8" s="36">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="H8" s="36">
-        <v>21</v>
-      </c>
-      <c r="I8" s="36">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="I8" s="37">
+        <v>18</v>
       </c>
       <c r="J8" s="36">
-        <v>18</v>
-      </c>
-      <c r="K8" s="36">
-        <v>20</v>
-      </c>
-      <c r="L8" s="36">
-        <v>17</v>
-      </c>
-      <c r="M8" s="36">
-        <v>17</v>
-      </c>
-      <c r="N8" s="36">
-        <v>18</v>
-      </c>
-      <c r="O8" s="37">
-        <v>18</v>
-      </c>
-      <c r="P8" s="36">
-        <f>O8-N8</f>
+        <f>I8-H8</f>
+      </c>
+      <c r="K8" s="35">
+        <f>I8-B8</f>
       </c>
     </row>
     <row r="9">
@@ -644,49 +538,34 @@
         </is>
       </c>
       <c r="B9" s="36">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C9" s="36">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D9" s="36">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E9" s="36">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F9" s="36">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G9" s="36">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H9" s="36">
         <v>18</v>
       </c>
-      <c r="I9" s="36">
-        <v>16</v>
+      <c r="I9" s="37">
+        <v>18</v>
       </c>
       <c r="J9" s="36">
-        <v>20</v>
+        <f>I9-H9</f>
       </c>
       <c r="K9" s="36">
-        <v>22</v>
-      </c>
-      <c r="L9" s="36">
-        <v>23</v>
-      </c>
-      <c r="M9" s="36">
-        <v>20</v>
-      </c>
-      <c r="N9" s="36">
-        <v>18</v>
-      </c>
-      <c r="O9" s="37">
-        <v>18</v>
-      </c>
-      <c r="P9" s="36">
-        <f>O9-N9</f>
+        <f>I9-B9</f>
       </c>
     </row>
     <row r="10">
@@ -696,49 +575,34 @@
         </is>
       </c>
       <c r="B10" s="36">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10" s="36">
         <v>7</v>
       </c>
       <c r="D10" s="36">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E10" s="36">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F10" s="36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G10" s="36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H10" s="36">
         <v>8</v>
       </c>
-      <c r="I10" s="36">
-        <v>7</v>
-      </c>
-      <c r="J10" s="36">
-        <v>9</v>
-      </c>
-      <c r="K10" s="36">
-        <v>14</v>
-      </c>
-      <c r="L10" s="36">
-        <v>7</v>
-      </c>
-      <c r="M10" s="36">
-        <v>6</v>
-      </c>
-      <c r="N10" s="36">
-        <v>8</v>
-      </c>
-      <c r="O10" s="37">
+      <c r="I10" s="37">
         <v>11</v>
       </c>
-      <c r="P10" s="34">
-        <f>O10-N10</f>
+      <c r="J10" s="34">
+        <f>I10-H10</f>
+      </c>
+      <c r="K10" s="34">
+        <f>I10-B10</f>
       </c>
     </row>
     <row r="11">
@@ -748,49 +612,34 @@
         </is>
       </c>
       <c r="B11" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D11" s="36">
         <v>9</v>
       </c>
       <c r="E11" s="36">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F11" s="36">
+        <v>13</v>
+      </c>
+      <c r="G11" s="36">
+        <v>9</v>
+      </c>
+      <c r="H11" s="36">
+        <v>11</v>
+      </c>
+      <c r="I11" s="37">
         <v>7</v>
       </c>
-      <c r="G11" s="36">
-        <v>8</v>
-      </c>
-      <c r="H11" s="36">
-        <v>9</v>
-      </c>
-      <c r="I11" s="36">
-        <v>7</v>
-      </c>
-      <c r="J11" s="36">
-        <v>9</v>
-      </c>
-      <c r="K11" s="36">
-        <v>12</v>
-      </c>
-      <c r="L11" s="36">
-        <v>13</v>
-      </c>
-      <c r="M11" s="36">
-        <v>9</v>
-      </c>
-      <c r="N11" s="36">
-        <v>11</v>
-      </c>
-      <c r="O11" s="37">
-        <v>7</v>
-      </c>
-      <c r="P11" s="35">
-        <f>O11-N11</f>
+      <c r="J11" s="35">
+        <f>I11-H11</f>
+      </c>
+      <c r="K11" s="35">
+        <f>I11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -800,49 +649,34 @@
         </is>
       </c>
       <c r="B12" s="36">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="36">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D12" s="36">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E12" s="36">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F12" s="36">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G12" s="36">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H12" s="36">
         <v>12</v>
       </c>
-      <c r="I12" s="36">
-        <v>11</v>
-      </c>
-      <c r="J12" s="36">
-        <v>10</v>
-      </c>
-      <c r="K12" s="36">
-        <v>10</v>
-      </c>
-      <c r="L12" s="36">
-        <v>12</v>
-      </c>
-      <c r="M12" s="36">
-        <v>11</v>
-      </c>
-      <c r="N12" s="36">
-        <v>12</v>
-      </c>
-      <c r="O12" s="37">
+      <c r="I12" s="37">
         <v>7</v>
       </c>
-      <c r="P12" s="35">
-        <f>O12-N12</f>
+      <c r="J12" s="35">
+        <f>I12-H12</f>
+      </c>
+      <c r="K12" s="35">
+        <f>I12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -852,49 +686,34 @@
         </is>
       </c>
       <c r="B13" s="36">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C13" s="36">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D13" s="36">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E13" s="36">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F13" s="36">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G13" s="36">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H13" s="36">
-        <v>11</v>
-      </c>
-      <c r="I13" s="36">
-        <v>10</v>
-      </c>
-      <c r="J13" s="36">
-        <v>9</v>
-      </c>
-      <c r="K13" s="36">
+        <v>5</v>
+      </c>
+      <c r="I13" s="37">
         <v>6</v>
       </c>
-      <c r="L13" s="36">
-        <v>5</v>
-      </c>
-      <c r="M13" s="36">
-        <v>5</v>
-      </c>
-      <c r="N13" s="36">
-        <v>5</v>
-      </c>
-      <c r="O13" s="37">
-        <v>6</v>
-      </c>
-      <c r="P13" s="34">
-        <f>O13-N13</f>
+      <c r="J13" s="34">
+        <f>I13-H13</f>
+      </c>
+      <c r="K13" s="35">
+        <f>I13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -904,49 +723,34 @@
         </is>
       </c>
       <c r="B14" s="36">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C14" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14" s="36">
+        <v>3</v>
+      </c>
+      <c r="F14" s="36">
         <v>2</v>
       </c>
-      <c r="F14" s="36">
-        <v>3</v>
-      </c>
       <c r="G14" s="36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="36">
+        <v>2</v>
+      </c>
+      <c r="I14" s="37">
         <v>4</v>
       </c>
-      <c r="I14" s="36">
-        <v>4</v>
-      </c>
-      <c r="J14" s="36">
-        <v>3</v>
+      <c r="J14" s="34">
+        <f>I14-H14</f>
       </c>
       <c r="K14" s="36">
-        <v>3</v>
-      </c>
-      <c r="L14" s="36">
-        <v>2</v>
-      </c>
-      <c r="M14" s="36">
-        <v>4</v>
-      </c>
-      <c r="N14" s="36">
-        <v>2</v>
-      </c>
-      <c r="O14" s="37">
-        <v>4</v>
-      </c>
-      <c r="P14" s="34">
-        <f>O14-N14</f>
+        <f>I14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -979,26 +783,11 @@
       <c r="I15" s="38">
         <f>SUM(I4:I14)</f>
       </c>
-      <c r="J15" s="38">
-        <f>SUM(J4:J14)</f>
-      </c>
-      <c r="K15" s="38">
-        <f>SUM(K4:K14)</f>
-      </c>
-      <c r="L15" s="38">
-        <f>SUM(L4:L14)</f>
-      </c>
-      <c r="M15" s="38">
-        <f>SUM(M4:M14)</f>
-      </c>
-      <c r="N15" s="38">
-        <f>SUM(N4:N14)</f>
-      </c>
-      <c r="O15" s="38">
-        <f>SUM(O4:O14)</f>
-      </c>
-      <c r="P15" s="41">
-        <f>O15-N15</f>
+      <c r="J15" s="41">
+        <f>I15-H15</f>
+      </c>
+      <c r="K15" s="41">
+        <f>I15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1057,31 +846,6 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="L16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="P16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1090,48 +854,35 @@
         </is>
       </c>
       <c r="B17" s="36">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C17" s="36">
+        <v>36</v>
+      </c>
+      <c r="D17" s="36">
+        <v>25</v>
+      </c>
+      <c r="E17" s="36">
+        <v>9</v>
+      </c>
+      <c r="F17" s="36">
+        <v>30</v>
+      </c>
+      <c r="G17" s="36">
+        <v>31</v>
+      </c>
+      <c r="H17" s="36">
+        <v>34</v>
+      </c>
+      <c r="I17" s="37">
         <v>38</v>
       </c>
-      <c r="D17" s="36">
-        <v>21</v>
-      </c>
-      <c r="E17" s="36">
-        <v>32</v>
-      </c>
-      <c r="F17" s="36">
-        <v>43</v>
-      </c>
-      <c r="G17" s="36">
-        <v>36</v>
-      </c>
-      <c r="H17" s="36">
-        <v>40</v>
-      </c>
-      <c r="I17" s="36">
-        <v>36</v>
-      </c>
-      <c r="J17" s="36">
-        <v>25</v>
-      </c>
-      <c r="K17" s="36">
-        <v>9</v>
-      </c>
-      <c r="L17" s="36">
-        <v>30</v>
-      </c>
-      <c r="M17" s="36">
-        <v>31</v>
-      </c>
-      <c r="N17" s="36">
-        <v>34</v>
-      </c>
-      <c r="O17" s="37">
-        <v>38</v>
-      </c>
-      <c r="P17" s="36" t="inlineStr">
+      <c r="J17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1144,48 +895,35 @@
         </is>
       </c>
       <c r="B18" s="36">
+        <v>35</v>
+      </c>
+      <c r="C18" s="36">
+        <v>26</v>
+      </c>
+      <c r="D18" s="36">
+        <v>28</v>
+      </c>
+      <c r="E18" s="36">
+        <v>21</v>
+      </c>
+      <c r="F18" s="36">
+        <v>31</v>
+      </c>
+      <c r="G18" s="36">
+        <v>20</v>
+      </c>
+      <c r="H18" s="36">
+        <v>33</v>
+      </c>
+      <c r="I18" s="37">
         <v>30</v>
       </c>
-      <c r="C18" s="36">
-        <v>31</v>
-      </c>
-      <c r="D18" s="36">
-        <v>8</v>
-      </c>
-      <c r="E18" s="36">
-        <v>23</v>
-      </c>
-      <c r="F18" s="36">
-        <v>32</v>
-      </c>
-      <c r="G18" s="36">
-        <v>35</v>
-      </c>
-      <c r="H18" s="36">
-        <v>35</v>
-      </c>
-      <c r="I18" s="36">
-        <v>26</v>
-      </c>
-      <c r="J18" s="36">
-        <v>28</v>
-      </c>
-      <c r="K18" s="36">
-        <v>21</v>
-      </c>
-      <c r="L18" s="36">
-        <v>31</v>
-      </c>
-      <c r="M18" s="36">
-        <v>20</v>
-      </c>
-      <c r="N18" s="36">
-        <v>33</v>
-      </c>
-      <c r="O18" s="37">
-        <v>30</v>
-      </c>
-      <c r="P18" s="36" t="inlineStr">
+      <c r="J18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1218,28 +956,15 @@
       <c r="H19" s="36">
         <f>H18-H17</f>
       </c>
-      <c r="I19" s="36">
+      <c r="I19" s="37">
         <f>I18-I17</f>
       </c>
-      <c r="J19" s="36">
-        <f>J18-J17</f>
-      </c>
-      <c r="K19" s="36">
-        <f>K18-K17</f>
-      </c>
-      <c r="L19" s="36">
-        <f>L18-L17</f>
-      </c>
-      <c r="M19" s="36">
-        <f>M18-M17</f>
-      </c>
-      <c r="N19" s="36">
-        <f>N18-N17</f>
-      </c>
-      <c r="O19" s="37">
-        <f>O18-O17</f>
-      </c>
-      <c r="P19" s="36" t="inlineStr">
+      <c r="J19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1252,48 +977,35 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C20" s="36">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D20" s="36">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E20" s="36">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F20" s="36">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G20" s="36">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H20" s="36">
-        <v>14</v>
-      </c>
-      <c r="I20" s="36">
         <v>13</v>
       </c>
-      <c r="J20" s="36">
-        <v>15</v>
-      </c>
-      <c r="K20" s="36">
-        <v>15</v>
-      </c>
-      <c r="L20" s="36">
-        <v>15</v>
-      </c>
-      <c r="M20" s="36">
-        <v>13</v>
-      </c>
-      <c r="N20" s="36">
-        <v>13</v>
-      </c>
-      <c r="O20" s="37">
+      <c r="I20" s="37">
         <v>10</v>
       </c>
-      <c r="P20" s="36" t="inlineStr">
+      <c r="J20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-09 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -278,13 +278,14 @@
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 08/10 · variação 07/10 → 08/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 09/10 · variação 08/10 → 09/10</t>
         </is>
       </c>
     </row>
@@ -337,10 +338,15 @@
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">09/10</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -373,199 +379,217 @@
       <c r="H4" s="36">
         <v>71</v>
       </c>
-      <c r="I4" s="37">
+      <c r="I4" s="36">
         <v>66</v>
       </c>
-      <c r="J4" s="35">
-        <f>I4-H4</f>
-      </c>
-      <c r="K4" s="34">
-        <f>I4-B4</f>
+      <c r="J4" s="37">
+        <v>63</v>
+      </c>
+      <c r="K4" s="35">
+        <f>J4-I4</f>
+      </c>
+      <c r="L4" s="36">
+        <f>J4-B4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B5" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="C5" s="36">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D5" s="36">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="E5" s="36">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="F5" s="36">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="G5" s="36">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H5" s="36">
-        <v>41</v>
-      </c>
-      <c r="I5" s="37">
-        <v>39</v>
-      </c>
-      <c r="J5" s="35">
-        <f>I5-H5</f>
-      </c>
-      <c r="K5" s="36">
-        <f>I5-B5</f>
+        <v>24</v>
+      </c>
+      <c r="I5" s="36">
+        <v>28</v>
+      </c>
+      <c r="J5" s="37">
+        <v>30</v>
+      </c>
+      <c r="K5" s="34">
+        <f>J5-I5</f>
+      </c>
+      <c r="L5" s="34">
+        <f>J5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" s="36">
+        <v>21</v>
+      </c>
+      <c r="D6" s="36">
+        <v>18</v>
+      </c>
+      <c r="E6" s="36">
+        <v>20</v>
+      </c>
+      <c r="F6" s="36">
+        <v>17</v>
+      </c>
+      <c r="G6" s="36">
+        <v>17</v>
+      </c>
+      <c r="H6" s="36">
+        <v>18</v>
+      </c>
+      <c r="I6" s="36">
+        <v>18</v>
+      </c>
+      <c r="J6" s="37">
         <v>22</v>
       </c>
-      <c r="D6" s="36">
-        <v>22</v>
-      </c>
-      <c r="E6" s="36">
-        <v>22</v>
-      </c>
-      <c r="F6" s="36">
-        <v>23</v>
-      </c>
-      <c r="G6" s="36">
-        <v>25</v>
-      </c>
-      <c r="H6" s="36">
-        <v>24</v>
-      </c>
-      <c r="I6" s="37">
-        <v>28</v>
-      </c>
-      <c r="J6" s="34">
-        <f>I6-H6</f>
-      </c>
       <c r="K6" s="34">
-        <f>I6-B6</f>
+        <f>J6-I6</f>
+      </c>
+      <c r="L6" s="34">
+        <f>J6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="C7" s="36">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D7" s="36">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E7" s="36">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="F7" s="36">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G7" s="36">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H7" s="36">
-        <v>26</v>
-      </c>
-      <c r="I7" s="37">
-        <v>24</v>
-      </c>
-      <c r="J7" s="35">
-        <f>I7-H7</f>
-      </c>
-      <c r="K7" s="35">
-        <f>I7-B7</f>
+        <v>18</v>
+      </c>
+      <c r="I7" s="36">
+        <v>18</v>
+      </c>
+      <c r="J7" s="37">
+        <v>19</v>
+      </c>
+      <c r="K7" s="34">
+        <f>J7-I7</f>
+      </c>
+      <c r="L7" s="34">
+        <f>J7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="C8" s="36">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D8" s="36">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E8" s="36">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="F8" s="36">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G8" s="36">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="H8" s="36">
-        <v>18</v>
-      </c>
-      <c r="I8" s="37">
-        <v>18</v>
-      </c>
-      <c r="J8" s="36">
-        <f>I8-H8</f>
+        <v>26</v>
+      </c>
+      <c r="I8" s="36">
+        <v>24</v>
+      </c>
+      <c r="J8" s="37">
+        <v>19</v>
       </c>
       <c r="K8" s="35">
-        <f>I8-B8</f>
+        <f>J8-I8</f>
+      </c>
+      <c r="L8" s="35">
+        <f>J8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="C9" s="36">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D9" s="36">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E9" s="36">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F9" s="36">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="G9" s="36">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H9" s="36">
-        <v>18</v>
-      </c>
-      <c r="I9" s="37">
-        <v>18</v>
-      </c>
-      <c r="J9" s="36">
-        <f>I9-H9</f>
-      </c>
-      <c r="K9" s="36">
-        <f>I9-B9</f>
+        <v>41</v>
+      </c>
+      <c r="I9" s="36">
+        <v>39</v>
+      </c>
+      <c r="J9" s="37">
+        <v>14</v>
+      </c>
+      <c r="K9" s="35">
+        <f>J9-I9</f>
+      </c>
+      <c r="L9" s="35">
+        <f>J9-B9</f>
       </c>
     </row>
     <row r="10">
@@ -595,14 +619,17 @@
       <c r="H10" s="36">
         <v>8</v>
       </c>
-      <c r="I10" s="37">
+      <c r="I10" s="36">
         <v>11</v>
       </c>
-      <c r="J10" s="34">
-        <f>I10-H10</f>
-      </c>
-      <c r="K10" s="34">
-        <f>I10-B10</f>
+      <c r="J10" s="37">
+        <v>11</v>
+      </c>
+      <c r="K10" s="36">
+        <f>J10-I10</f>
+      </c>
+      <c r="L10" s="34">
+        <f>J10-B10</f>
       </c>
     </row>
     <row r="11">
@@ -632,14 +659,17 @@
       <c r="H11" s="36">
         <v>11</v>
       </c>
-      <c r="I11" s="37">
+      <c r="I11" s="36">
         <v>7</v>
       </c>
-      <c r="J11" s="35">
-        <f>I11-H11</f>
+      <c r="J11" s="37">
+        <v>6</v>
       </c>
       <c r="K11" s="35">
-        <f>I11-B11</f>
+        <f>J11-I11</f>
+      </c>
+      <c r="L11" s="35">
+        <f>J11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -669,14 +699,17 @@
       <c r="H12" s="36">
         <v>12</v>
       </c>
-      <c r="I12" s="37">
+      <c r="I12" s="36">
         <v>7</v>
       </c>
-      <c r="J12" s="35">
-        <f>I12-H12</f>
+      <c r="J12" s="37">
+        <v>6</v>
       </c>
       <c r="K12" s="35">
-        <f>I12-B12</f>
+        <f>J12-I12</f>
+      </c>
+      <c r="L12" s="35">
+        <f>J12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -706,14 +739,17 @@
       <c r="H13" s="36">
         <v>5</v>
       </c>
-      <c r="I13" s="37">
+      <c r="I13" s="36">
         <v>6</v>
       </c>
-      <c r="J13" s="34">
-        <f>I13-H13</f>
+      <c r="J13" s="37">
+        <v>5</v>
       </c>
       <c r="K13" s="35">
-        <f>I13-B13</f>
+        <f>J13-I13</f>
+      </c>
+      <c r="L13" s="35">
+        <f>J13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -743,14 +779,17 @@
       <c r="H14" s="36">
         <v>2</v>
       </c>
-      <c r="I14" s="37">
+      <c r="I14" s="36">
         <v>4</v>
       </c>
-      <c r="J14" s="34">
-        <f>I14-H14</f>
-      </c>
-      <c r="K14" s="36">
-        <f>I14-B14</f>
+      <c r="J14" s="37">
+        <v>3</v>
+      </c>
+      <c r="K14" s="35">
+        <f>J14-I14</f>
+      </c>
+      <c r="L14" s="35">
+        <f>J14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -783,11 +822,14 @@
       <c r="I15" s="38">
         <f>SUM(I4:I14)</f>
       </c>
-      <c r="J15" s="41">
-        <f>I15-H15</f>
+      <c r="J15" s="38">
+        <f>SUM(J4:J14)</f>
       </c>
       <c r="K15" s="41">
-        <f>I15-B15</f>
+        <f>J15-I15</f>
+      </c>
+      <c r="L15" s="41">
+        <f>J15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -846,6 +888,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="L16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -874,15 +921,18 @@
       <c r="H17" s="36">
         <v>34</v>
       </c>
-      <c r="I17" s="37">
+      <c r="I17" s="36">
         <v>38</v>
       </c>
-      <c r="J17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="J17" s="37">
+        <v>61</v>
       </c>
       <c r="K17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -915,15 +965,18 @@
       <c r="H18" s="36">
         <v>33</v>
       </c>
-      <c r="I18" s="37">
+      <c r="I18" s="36">
         <v>30</v>
       </c>
-      <c r="J18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="J18" s="37">
+        <v>31</v>
       </c>
       <c r="K18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -956,15 +1009,18 @@
       <c r="H19" s="36">
         <f>H18-H17</f>
       </c>
-      <c r="I19" s="37">
+      <c r="I19" s="36">
         <f>I18-I17</f>
       </c>
-      <c r="J19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="J19" s="37">
+        <f>J18-J17</f>
       </c>
       <c r="K19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -997,15 +1053,18 @@
       <c r="H20" s="36">
         <v>13</v>
       </c>
-      <c r="I20" s="37">
+      <c r="I20" s="36">
         <v>10</v>
       </c>
-      <c r="J20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="J20" s="37">
+        <v>10</v>
       </c>
       <c r="K20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-10 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -279,13 +279,14 @@
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 09/10 · variação 08/10 → 09/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 10/10 · variação 09/10 → 10/10</t>
         </is>
       </c>
     </row>
@@ -343,10 +344,15 @@
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">10/10</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -382,14 +388,17 @@
       <c r="I4" s="36">
         <v>66</v>
       </c>
-      <c r="J4" s="37">
+      <c r="J4" s="36">
         <v>63</v>
       </c>
-      <c r="K4" s="35">
-        <f>J4-I4</f>
-      </c>
-      <c r="L4" s="36">
-        <f>J4-B4</f>
+      <c r="K4" s="37">
+        <v>51</v>
+      </c>
+      <c r="L4" s="35">
+        <f>K4-J4</f>
+      </c>
+      <c r="M4" s="35">
+        <f>K4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -422,14 +431,17 @@
       <c r="I5" s="36">
         <v>28</v>
       </c>
-      <c r="J5" s="37">
+      <c r="J5" s="36">
         <v>30</v>
       </c>
-      <c r="K5" s="34">
-        <f>J5-I5</f>
+      <c r="K5" s="37">
+        <v>32</v>
       </c>
       <c r="L5" s="34">
-        <f>J5-B5</f>
+        <f>K5-J5</f>
+      </c>
+      <c r="M5" s="34">
+        <f>K5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -462,94 +474,103 @@
       <c r="I6" s="36">
         <v>18</v>
       </c>
-      <c r="J6" s="37">
+      <c r="J6" s="36">
         <v>22</v>
       </c>
-      <c r="K6" s="34">
-        <f>J6-I6</f>
-      </c>
-      <c r="L6" s="34">
-        <f>J6-B6</f>
+      <c r="K6" s="37">
+        <v>17</v>
+      </c>
+      <c r="L6" s="35">
+        <f>K6-J6</f>
+      </c>
+      <c r="M6" s="35">
+        <f>K6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C7" s="36">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D7" s="36">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="E7" s="36">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F7" s="36">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="G7" s="36">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H7" s="36">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I7" s="36">
-        <v>18</v>
-      </c>
-      <c r="J7" s="37">
+        <v>24</v>
+      </c>
+      <c r="J7" s="36">
         <v>19</v>
       </c>
-      <c r="K7" s="34">
-        <f>J7-I7</f>
-      </c>
-      <c r="L7" s="34">
-        <f>J7-B7</f>
+      <c r="K7" s="37">
+        <v>17</v>
+      </c>
+      <c r="L7" s="35">
+        <f>K7-J7</f>
+      </c>
+      <c r="M7" s="35">
+        <f>K7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="C8" s="36">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D8" s="36">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E8" s="36">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="F8" s="36">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G8" s="36">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H8" s="36">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="I8" s="36">
-        <v>24</v>
-      </c>
-      <c r="J8" s="37">
+        <v>18</v>
+      </c>
+      <c r="J8" s="36">
         <v>19</v>
       </c>
-      <c r="K8" s="35">
-        <f>J8-I8</f>
+      <c r="K8" s="37">
+        <v>16</v>
       </c>
       <c r="L8" s="35">
-        <f>J8-B8</f>
+        <f>K8-J8</f>
+      </c>
+      <c r="M8" s="35">
+        <f>K8-B8</f>
       </c>
     </row>
     <row r="9">
@@ -582,14 +603,17 @@
       <c r="I9" s="36">
         <v>39</v>
       </c>
-      <c r="J9" s="37">
+      <c r="J9" s="36">
         <v>14</v>
       </c>
-      <c r="K9" s="35">
-        <f>J9-I9</f>
-      </c>
-      <c r="L9" s="35">
-        <f>J9-B9</f>
+      <c r="K9" s="37">
+        <v>15</v>
+      </c>
+      <c r="L9" s="34">
+        <f>K9-J9</f>
+      </c>
+      <c r="M9" s="35">
+        <f>K9-B9</f>
       </c>
     </row>
     <row r="10">
@@ -622,94 +646,103 @@
       <c r="I10" s="36">
         <v>11</v>
       </c>
-      <c r="J10" s="37">
+      <c r="J10" s="36">
         <v>11</v>
       </c>
-      <c r="K10" s="36">
-        <f>J10-I10</f>
+      <c r="K10" s="37">
+        <v>13</v>
       </c>
       <c r="L10" s="34">
-        <f>J10-B10</f>
+        <f>K10-J10</f>
+      </c>
+      <c r="M10" s="34">
+        <f>K10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C11" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D11" s="36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11" s="36">
+        <v>10</v>
+      </c>
+      <c r="F11" s="36">
         <v>12</v>
       </c>
-      <c r="F11" s="36">
-        <v>13</v>
-      </c>
       <c r="G11" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H11" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I11" s="36">
         <v>7</v>
       </c>
-      <c r="J11" s="37">
+      <c r="J11" s="36">
         <v>6</v>
       </c>
-      <c r="K11" s="35">
-        <f>J11-I11</f>
-      </c>
-      <c r="L11" s="35">
-        <f>J11-B11</f>
+      <c r="K11" s="37">
+        <v>7</v>
+      </c>
+      <c r="L11" s="34">
+        <f>K11-J11</f>
+      </c>
+      <c r="M11" s="35">
+        <f>K11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B12" s="36">
+        <v>9</v>
+      </c>
+      <c r="C12" s="36">
+        <v>7</v>
+      </c>
+      <c r="D12" s="36">
+        <v>9</v>
+      </c>
+      <c r="E12" s="36">
         <v>12</v>
       </c>
-      <c r="C12" s="36">
+      <c r="F12" s="36">
+        <v>13</v>
+      </c>
+      <c r="G12" s="36">
+        <v>9</v>
+      </c>
+      <c r="H12" s="36">
         <v>11</v>
-      </c>
-      <c r="D12" s="36">
-        <v>10</v>
-      </c>
-      <c r="E12" s="36">
-        <v>10</v>
-      </c>
-      <c r="F12" s="36">
-        <v>12</v>
-      </c>
-      <c r="G12" s="36">
-        <v>11</v>
-      </c>
-      <c r="H12" s="36">
-        <v>12</v>
       </c>
       <c r="I12" s="36">
         <v>7</v>
       </c>
-      <c r="J12" s="37">
+      <c r="J12" s="36">
         <v>6</v>
       </c>
-      <c r="K12" s="35">
-        <f>J12-I12</f>
-      </c>
-      <c r="L12" s="35">
-        <f>J12-B12</f>
+      <c r="K12" s="37">
+        <v>6</v>
+      </c>
+      <c r="L12" s="36">
+        <f>K12-J12</f>
+      </c>
+      <c r="M12" s="35">
+        <f>K12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -742,14 +775,17 @@
       <c r="I13" s="36">
         <v>6</v>
       </c>
-      <c r="J13" s="37">
+      <c r="J13" s="36">
         <v>5</v>
       </c>
-      <c r="K13" s="35">
-        <f>J13-I13</f>
+      <c r="K13" s="37">
+        <v>4</v>
       </c>
       <c r="L13" s="35">
-        <f>J13-B13</f>
+        <f>K13-J13</f>
+      </c>
+      <c r="M13" s="35">
+        <f>K13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -782,14 +818,17 @@
       <c r="I14" s="36">
         <v>4</v>
       </c>
-      <c r="J14" s="37">
+      <c r="J14" s="36">
         <v>3</v>
       </c>
-      <c r="K14" s="35">
-        <f>J14-I14</f>
+      <c r="K14" s="37">
+        <v>0</v>
       </c>
       <c r="L14" s="35">
-        <f>J14-B14</f>
+        <f>K14-J14</f>
+      </c>
+      <c r="M14" s="35">
+        <f>K14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -825,11 +864,14 @@
       <c r="J15" s="38">
         <f>SUM(J4:J14)</f>
       </c>
-      <c r="K15" s="41">
-        <f>J15-I15</f>
+      <c r="K15" s="38">
+        <f>SUM(K4:K14)</f>
       </c>
       <c r="L15" s="41">
-        <f>J15-B15</f>
+        <f>K15-J15</f>
+      </c>
+      <c r="M15" s="41">
+        <f>K15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -893,6 +935,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="M16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -924,15 +971,18 @@
       <c r="I17" s="36">
         <v>38</v>
       </c>
-      <c r="J17" s="37">
+      <c r="J17" s="36">
         <v>61</v>
       </c>
-      <c r="K17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="K17" s="37">
+        <v>54</v>
       </c>
       <c r="L17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -968,15 +1018,18 @@
       <c r="I18" s="36">
         <v>30</v>
       </c>
-      <c r="J18" s="37">
+      <c r="J18" s="36">
         <v>31</v>
       </c>
-      <c r="K18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="K18" s="37">
+        <v>34</v>
       </c>
       <c r="L18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1012,15 +1065,18 @@
       <c r="I19" s="36">
         <f>I18-I17</f>
       </c>
-      <c r="J19" s="37">
+      <c r="J19" s="36">
         <f>J18-J17</f>
       </c>
-      <c r="K19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="K19" s="37">
+        <f>K18-K17</f>
       </c>
       <c r="L19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1056,15 +1112,18 @@
       <c r="I20" s="36">
         <v>10</v>
       </c>
-      <c r="J20" s="37">
+      <c r="J20" s="36">
         <v>10</v>
       </c>
-      <c r="K20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="K20" s="37">
+        <v>8</v>
       </c>
       <c r="L20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-11 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -280,13 +280,14 @@
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 10/10 · variação 09/10 → 10/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 11/10 · variação 10/10 → 11/10</t>
         </is>
       </c>
     </row>
@@ -349,10 +350,15 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">11/10</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="N3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -391,14 +397,17 @@
       <c r="J4" s="36">
         <v>63</v>
       </c>
-      <c r="K4" s="37">
+      <c r="K4" s="36">
         <v>51</v>
       </c>
-      <c r="L4" s="35">
-        <f>K4-J4</f>
+      <c r="L4" s="37">
+        <v>50</v>
       </c>
       <c r="M4" s="35">
-        <f>K4-B4</f>
+        <f>L4-K4</f>
+      </c>
+      <c r="N4" s="35">
+        <f>L4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -434,14 +443,17 @@
       <c r="J5" s="36">
         <v>30</v>
       </c>
-      <c r="K5" s="37">
+      <c r="K5" s="36">
         <v>31</v>
       </c>
-      <c r="L5" s="34">
-        <f>K5-J5</f>
-      </c>
-      <c r="M5" s="34">
-        <f>K5-B5</f>
+      <c r="L5" s="37">
+        <v>31</v>
+      </c>
+      <c r="M5" s="36">
+        <f>L5-K5</f>
+      </c>
+      <c r="N5" s="34">
+        <f>L5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -477,14 +489,17 @@
       <c r="J6" s="36">
         <v>19</v>
       </c>
-      <c r="K6" s="37">
+      <c r="K6" s="36">
         <v>17</v>
       </c>
-      <c r="L6" s="35">
-        <f>K6-J6</f>
+      <c r="L6" s="37">
+        <v>16</v>
       </c>
       <c r="M6" s="35">
-        <f>K6-B6</f>
+        <f>L6-K6</f>
+      </c>
+      <c r="N6" s="35">
+        <f>L6-B6</f>
       </c>
     </row>
     <row r="7">
@@ -520,14 +535,17 @@
       <c r="J7" s="36">
         <v>19</v>
       </c>
-      <c r="K7" s="37">
+      <c r="K7" s="36">
         <v>17</v>
       </c>
-      <c r="L7" s="35">
-        <f>K7-J7</f>
+      <c r="L7" s="37">
+        <v>14</v>
       </c>
       <c r="M7" s="35">
-        <f>K7-B7</f>
+        <f>L7-K7</f>
+      </c>
+      <c r="N7" s="35">
+        <f>L7-B7</f>
       </c>
     </row>
     <row r="8">
@@ -563,128 +581,137 @@
       <c r="J8" s="36">
         <v>22</v>
       </c>
-      <c r="K8" s="37">
+      <c r="K8" s="36">
         <v>16</v>
       </c>
-      <c r="L8" s="35">
-        <f>K8-J8</f>
+      <c r="L8" s="37">
+        <v>13</v>
       </c>
       <c r="M8" s="35">
-        <f>K8-B8</f>
+        <f>L8-K8</f>
+      </c>
+      <c r="N8" s="35">
+        <f>L8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="C9" s="36">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="D9" s="36">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E9" s="36">
+        <v>43</v>
+      </c>
+      <c r="F9" s="36">
+        <v>42</v>
+      </c>
+      <c r="G9" s="36">
+        <v>45</v>
+      </c>
+      <c r="H9" s="36">
+        <v>41</v>
+      </c>
+      <c r="I9" s="36">
+        <v>39</v>
+      </c>
+      <c r="J9" s="36">
         <v>14</v>
       </c>
-      <c r="F9" s="36">
-        <v>7</v>
-      </c>
-      <c r="G9" s="36">
-        <v>6</v>
-      </c>
-      <c r="H9" s="36">
-        <v>8</v>
-      </c>
-      <c r="I9" s="36">
-        <v>11</v>
-      </c>
-      <c r="J9" s="36">
-        <v>11</v>
-      </c>
-      <c r="K9" s="37">
+      <c r="K9" s="36">
         <v>12</v>
       </c>
-      <c r="L9" s="34">
-        <f>K9-J9</f>
-      </c>
-      <c r="M9" s="34">
-        <f>K9-B9</f>
+      <c r="L9" s="37">
+        <v>12</v>
+      </c>
+      <c r="M9" s="36">
+        <f>L9-K9</f>
+      </c>
+      <c r="N9" s="35">
+        <f>L9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C10" s="36">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E10" s="36">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="F10" s="36">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="G10" s="36">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="H10" s="36">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="I10" s="36">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="J10" s="36">
-        <v>14</v>
-      </c>
-      <c r="K10" s="37">
-        <v>12</v>
-      </c>
-      <c r="L10" s="35">
-        <f>K10-J10</f>
-      </c>
-      <c r="M10" s="35">
-        <f>K10-B10</f>
+        <v>6</v>
+      </c>
+      <c r="K10" s="36">
+        <v>7</v>
+      </c>
+      <c r="L10" s="37">
+        <v>7</v>
+      </c>
+      <c r="M10" s="36">
+        <f>L10-K10</f>
+      </c>
+      <c r="N10" s="35">
+        <f>L10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B11" s="36">
+        <v>9</v>
+      </c>
+      <c r="C11" s="36">
+        <v>7</v>
+      </c>
+      <c r="D11" s="36">
+        <v>9</v>
+      </c>
+      <c r="E11" s="36">
         <v>12</v>
       </c>
-      <c r="C11" s="36">
+      <c r="F11" s="36">
+        <v>13</v>
+      </c>
+      <c r="G11" s="36">
+        <v>9</v>
+      </c>
+      <c r="H11" s="36">
         <v>11</v>
-      </c>
-      <c r="D11" s="36">
-        <v>10</v>
-      </c>
-      <c r="E11" s="36">
-        <v>10</v>
-      </c>
-      <c r="F11" s="36">
-        <v>12</v>
-      </c>
-      <c r="G11" s="36">
-        <v>11</v>
-      </c>
-      <c r="H11" s="36">
-        <v>12</v>
       </c>
       <c r="I11" s="36">
         <v>7</v>
@@ -692,100 +719,109 @@
       <c r="J11" s="36">
         <v>6</v>
       </c>
-      <c r="K11" s="37">
-        <v>7</v>
-      </c>
-      <c r="L11" s="34">
-        <f>K11-J11</f>
-      </c>
-      <c r="M11" s="35">
-        <f>K11-B11</f>
+      <c r="K11" s="36">
+        <v>6</v>
+      </c>
+      <c r="L11" s="37">
+        <v>6</v>
+      </c>
+      <c r="M11" s="36">
+        <f>L11-K11</f>
+      </c>
+      <c r="N11" s="35">
+        <f>L11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C12" s="36">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D12" s="36">
         <v>9</v>
       </c>
       <c r="E12" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F12" s="36">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G12" s="36">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H12" s="36">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I12" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J12" s="36">
-        <v>6</v>
-      </c>
-      <c r="K12" s="37">
-        <v>6</v>
-      </c>
-      <c r="L12" s="36">
-        <f>K12-J12</f>
-      </c>
-      <c r="M12" s="35">
-        <f>K12-B12</f>
+        <v>5</v>
+      </c>
+      <c r="K12" s="36">
+        <v>4</v>
+      </c>
+      <c r="L12" s="37">
+        <v>4</v>
+      </c>
+      <c r="M12" s="36">
+        <f>L12-K12</f>
+      </c>
+      <c r="N12" s="35">
+        <f>L12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C13" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D13" s="36">
         <v>9</v>
       </c>
       <c r="E13" s="36">
+        <v>14</v>
+      </c>
+      <c r="F13" s="36">
+        <v>7</v>
+      </c>
+      <c r="G13" s="36">
         <v>6</v>
       </c>
-      <c r="F13" s="36">
-        <v>5</v>
-      </c>
-      <c r="G13" s="36">
-        <v>5</v>
-      </c>
       <c r="H13" s="36">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I13" s="36">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J13" s="36">
-        <v>5</v>
-      </c>
-      <c r="K13" s="37">
-        <v>4</v>
-      </c>
-      <c r="L13" s="35">
-        <f>K13-J13</f>
+        <v>11</v>
+      </c>
+      <c r="K13" s="36">
+        <v>12</v>
+      </c>
+      <c r="L13" s="37">
+        <v>3</v>
       </c>
       <c r="M13" s="35">
-        <f>K13-B13</f>
+        <f>L13-K13</f>
+      </c>
+      <c r="N13" s="35">
+        <f>L13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -821,14 +857,17 @@
       <c r="J14" s="36">
         <v>3</v>
       </c>
-      <c r="K14" s="37">
+      <c r="K14" s="36">
         <v>0</v>
       </c>
-      <c r="L14" s="35">
-        <f>K14-J14</f>
-      </c>
-      <c r="M14" s="35">
-        <f>K14-B14</f>
+      <c r="L14" s="37">
+        <v>0</v>
+      </c>
+      <c r="M14" s="36">
+        <f>L14-K14</f>
+      </c>
+      <c r="N14" s="35">
+        <f>L14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -867,11 +906,14 @@
       <c r="K15" s="38">
         <f>SUM(K4:K14)</f>
       </c>
-      <c r="L15" s="41">
-        <f>K15-J15</f>
+      <c r="L15" s="38">
+        <f>SUM(L4:L14)</f>
       </c>
       <c r="M15" s="41">
-        <f>K15-B15</f>
+        <f>L15-K15</f>
+      </c>
+      <c r="N15" s="41">
+        <f>L15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -940,6 +982,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="N16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -974,15 +1021,18 @@
       <c r="J17" s="36">
         <v>61</v>
       </c>
-      <c r="K17" s="37">
+      <c r="K17" s="36">
         <v>61</v>
       </c>
-      <c r="L17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="L17" s="37">
+        <v>19</v>
       </c>
       <c r="M17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1021,15 +1071,18 @@
       <c r="J18" s="36">
         <v>31</v>
       </c>
-      <c r="K18" s="37">
+      <c r="K18" s="36">
         <v>36</v>
       </c>
-      <c r="L18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="L18" s="37">
+        <v>2</v>
       </c>
       <c r="M18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1068,15 +1121,18 @@
       <c r="J19" s="36">
         <f>J18-J17</f>
       </c>
-      <c r="K19" s="37">
+      <c r="K19" s="36">
         <f>K18-K17</f>
       </c>
-      <c r="L19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="L19" s="37">
+        <f>L18-L17</f>
       </c>
       <c r="M19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1115,15 +1171,18 @@
       <c r="J20" s="36">
         <v>10</v>
       </c>
-      <c r="K20" s="37">
+      <c r="K20" s="36">
         <v>8</v>
       </c>
-      <c r="L20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="L20" s="37">
+        <v>7</v>
       </c>
       <c r="M20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-12 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -281,13 +281,14 @@
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 11/10 · variação 10/10 → 11/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 12/10 · variação 11/10 → 12/10</t>
         </is>
       </c>
     </row>
@@ -355,10 +356,15 @@
       </c>
       <c r="M3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">12/10</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="N3" s="1" t="inlineStr">
+      <c r="O3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -400,14 +406,17 @@
       <c r="K4" s="36">
         <v>51</v>
       </c>
-      <c r="L4" s="37">
-        <v>50</v>
-      </c>
-      <c r="M4" s="35">
-        <f>L4-K4</f>
+      <c r="L4" s="36">
+        <v>41</v>
+      </c>
+      <c r="M4" s="37">
+        <v>38</v>
       </c>
       <c r="N4" s="35">
-        <f>L4-B4</f>
+        <f>M4-L4</f>
+      </c>
+      <c r="O4" s="35">
+        <f>M4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -446,14 +455,17 @@
       <c r="K5" s="36">
         <v>31</v>
       </c>
-      <c r="L5" s="37">
-        <v>31</v>
-      </c>
-      <c r="M5" s="36">
-        <f>L5-K5</f>
-      </c>
-      <c r="N5" s="34">
-        <f>L5-B5</f>
+      <c r="L5" s="36">
+        <v>26</v>
+      </c>
+      <c r="M5" s="37">
+        <v>24</v>
+      </c>
+      <c r="N5" s="35">
+        <f>M5-L5</f>
+      </c>
+      <c r="O5" s="34">
+        <f>M5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -492,14 +504,17 @@
       <c r="K6" s="36">
         <v>17</v>
       </c>
-      <c r="L6" s="37">
-        <v>16</v>
-      </c>
-      <c r="M6" s="35">
-        <f>L6-K6</f>
-      </c>
-      <c r="N6" s="35">
-        <f>L6-B6</f>
+      <c r="L6" s="36">
+        <v>13</v>
+      </c>
+      <c r="M6" s="37">
+        <v>14</v>
+      </c>
+      <c r="N6" s="34">
+        <f>M6-L6</f>
+      </c>
+      <c r="O6" s="35">
+        <f>M6-B6</f>
       </c>
     </row>
     <row r="7">
@@ -509,43 +524,46 @@
         </is>
       </c>
       <c r="B7" s="36">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7" s="36">
+        <v>33</v>
+      </c>
+      <c r="D7" s="36">
+        <v>33</v>
+      </c>
+      <c r="E7" s="36">
+        <v>35</v>
+      </c>
+      <c r="F7" s="36">
+        <v>39</v>
+      </c>
+      <c r="G7" s="36">
         <v>32</v>
       </c>
-      <c r="D7" s="36">
-        <v>32</v>
-      </c>
-      <c r="E7" s="36">
-        <v>34</v>
-      </c>
-      <c r="F7" s="36">
-        <v>38</v>
-      </c>
-      <c r="G7" s="36">
-        <v>31</v>
-      </c>
       <c r="H7" s="36">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I7" s="36">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J7" s="36">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K7" s="36">
-        <v>17</v>
-      </c>
-      <c r="L7" s="37">
+        <v>18</v>
+      </c>
+      <c r="L7" s="36">
         <v>14</v>
       </c>
-      <c r="M7" s="35">
-        <f>L7-K7</f>
-      </c>
-      <c r="N7" s="35">
-        <f>L7-B7</f>
+      <c r="M7" s="37">
+        <v>14</v>
+      </c>
+      <c r="N7" s="36">
+        <f>M7-L7</f>
+      </c>
+      <c r="O7" s="35">
+        <f>M7-B7</f>
       </c>
     </row>
     <row r="8">
@@ -584,14 +602,17 @@
       <c r="K8" s="36">
         <v>16</v>
       </c>
-      <c r="L8" s="37">
-        <v>13</v>
-      </c>
-      <c r="M8" s="35">
-        <f>L8-K8</f>
-      </c>
-      <c r="N8" s="35">
-        <f>L8-B8</f>
+      <c r="L8" s="36">
+        <v>12</v>
+      </c>
+      <c r="M8" s="37">
+        <v>12</v>
+      </c>
+      <c r="N8" s="36">
+        <f>M8-L8</f>
+      </c>
+      <c r="O8" s="35">
+        <f>M8-B8</f>
       </c>
     </row>
     <row r="9">
@@ -630,42 +651,45 @@
       <c r="K9" s="36">
         <v>12</v>
       </c>
-      <c r="L9" s="37">
-        <v>12</v>
-      </c>
-      <c r="M9" s="36">
-        <f>L9-K9</f>
-      </c>
-      <c r="N9" s="35">
-        <f>L9-B9</f>
+      <c r="L9" s="36">
+        <v>10</v>
+      </c>
+      <c r="M9" s="37">
+        <v>10</v>
+      </c>
+      <c r="N9" s="36">
+        <f>M9-L9</f>
+      </c>
+      <c r="O9" s="35">
+        <f>M9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B10" s="36">
+        <v>9</v>
+      </c>
+      <c r="C10" s="36">
+        <v>7</v>
+      </c>
+      <c r="D10" s="36">
+        <v>9</v>
+      </c>
+      <c r="E10" s="36">
         <v>12</v>
       </c>
-      <c r="C10" s="36">
+      <c r="F10" s="36">
+        <v>13</v>
+      </c>
+      <c r="G10" s="36">
+        <v>9</v>
+      </c>
+      <c r="H10" s="36">
         <v>11</v>
-      </c>
-      <c r="D10" s="36">
-        <v>10</v>
-      </c>
-      <c r="E10" s="36">
-        <v>10</v>
-      </c>
-      <c r="F10" s="36">
-        <v>12</v>
-      </c>
-      <c r="G10" s="36">
-        <v>11</v>
-      </c>
-      <c r="H10" s="36">
-        <v>12</v>
       </c>
       <c r="I10" s="36">
         <v>7</v>
@@ -674,44 +698,47 @@
         <v>6</v>
       </c>
       <c r="K10" s="36">
+        <v>6</v>
+      </c>
+      <c r="L10" s="36">
         <v>7</v>
       </c>
-      <c r="L10" s="37">
+      <c r="M10" s="37">
         <v>7</v>
       </c>
-      <c r="M10" s="36">
-        <f>L10-K10</f>
-      </c>
-      <c r="N10" s="35">
-        <f>L10-B10</f>
+      <c r="N10" s="36">
+        <f>M10-L10</f>
+      </c>
+      <c r="O10" s="35">
+        <f>M10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C11" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D11" s="36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11" s="36">
+        <v>10</v>
+      </c>
+      <c r="F11" s="36">
         <v>12</v>
       </c>
-      <c r="F11" s="36">
-        <v>13</v>
-      </c>
       <c r="G11" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H11" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I11" s="36">
         <v>7</v>
@@ -720,16 +747,19 @@
         <v>6</v>
       </c>
       <c r="K11" s="36">
-        <v>6</v>
-      </c>
-      <c r="L11" s="37">
-        <v>6</v>
-      </c>
-      <c r="M11" s="36">
-        <f>L11-K11</f>
-      </c>
-      <c r="N11" s="35">
-        <f>L11-B11</f>
+        <v>7</v>
+      </c>
+      <c r="L11" s="36">
+        <v>7</v>
+      </c>
+      <c r="M11" s="37">
+        <v>7</v>
+      </c>
+      <c r="N11" s="36">
+        <f>M11-L11</f>
+      </c>
+      <c r="O11" s="35">
+        <f>M11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -768,14 +798,17 @@
       <c r="K12" s="36">
         <v>4</v>
       </c>
-      <c r="L12" s="37">
+      <c r="L12" s="36">
         <v>4</v>
       </c>
-      <c r="M12" s="36">
-        <f>L12-K12</f>
-      </c>
-      <c r="N12" s="35">
-        <f>L12-B12</f>
+      <c r="M12" s="37">
+        <v>5</v>
+      </c>
+      <c r="N12" s="34">
+        <f>M12-L12</f>
+      </c>
+      <c r="O12" s="35">
+        <f>M12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -814,14 +847,17 @@
       <c r="K13" s="36">
         <v>12</v>
       </c>
-      <c r="L13" s="37">
-        <v>3</v>
-      </c>
-      <c r="M13" s="35">
-        <f>L13-K13</f>
-      </c>
-      <c r="N13" s="35">
-        <f>L13-B13</f>
+      <c r="L13" s="36">
+        <v>4</v>
+      </c>
+      <c r="M13" s="37">
+        <v>4</v>
+      </c>
+      <c r="N13" s="36">
+        <f>M13-L13</f>
+      </c>
+      <c r="O13" s="35">
+        <f>M13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -860,14 +896,17 @@
       <c r="K14" s="36">
         <v>0</v>
       </c>
-      <c r="L14" s="37">
+      <c r="L14" s="36">
         <v>0</v>
       </c>
-      <c r="M14" s="36">
-        <f>L14-K14</f>
-      </c>
-      <c r="N14" s="35">
-        <f>L14-B14</f>
+      <c r="M14" s="37">
+        <v>0</v>
+      </c>
+      <c r="N14" s="36">
+        <f>M14-L14</f>
+      </c>
+      <c r="O14" s="35">
+        <f>M14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -909,11 +948,14 @@
       <c r="L15" s="38">
         <f>SUM(L4:L14)</f>
       </c>
-      <c r="M15" s="41">
-        <f>L15-K15</f>
+      <c r="M15" s="38">
+        <f>SUM(M4:M14)</f>
       </c>
       <c r="N15" s="41">
-        <f>L15-B15</f>
+        <f>M15-L15</f>
+      </c>
+      <c r="O15" s="41">
+        <f>M15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -987,6 +1029,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="O16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1024,15 +1071,18 @@
       <c r="K17" s="36">
         <v>61</v>
       </c>
-      <c r="L17" s="37">
-        <v>19</v>
-      </c>
-      <c r="M17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="L17" s="36">
+        <v>61</v>
+      </c>
+      <c r="M17" s="37">
+        <v>8</v>
       </c>
       <c r="N17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1074,15 +1124,18 @@
       <c r="K18" s="36">
         <v>36</v>
       </c>
-      <c r="L18" s="37">
-        <v>2</v>
-      </c>
-      <c r="M18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="L18" s="36">
+        <v>25</v>
+      </c>
+      <c r="M18" s="37">
+        <v>5</v>
       </c>
       <c r="N18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1124,15 +1177,18 @@
       <c r="K19" s="36">
         <f>K18-K17</f>
       </c>
-      <c r="L19" s="37">
+      <c r="L19" s="36">
         <f>L18-L17</f>
       </c>
-      <c r="M19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="M19" s="37">
+        <f>M18-M17</f>
       </c>
       <c r="N19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1174,15 +1230,18 @@
       <c r="K20" s="36">
         <v>8</v>
       </c>
-      <c r="L20" s="37">
+      <c r="L20" s="36">
         <v>7</v>
       </c>
-      <c r="M20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="M20" s="37">
+        <v>7</v>
       </c>
       <c r="N20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-14 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -282,13 +282,15 @@
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 12/10 · variação 11/10 → 12/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 14/10 · variação 13/10 → 14/10</t>
         </is>
       </c>
     </row>
@@ -361,10 +363,20 @@
       </c>
       <c r="N3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">13/10</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14/10</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="O3" s="1" t="inlineStr">
+      <c r="Q3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -377,371 +389,413 @@
         </is>
       </c>
       <c r="B4" s="36">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="C4" s="36">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="D4" s="36">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E4" s="36">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="F4" s="36">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="G4" s="36">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="H4" s="36">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="I4" s="36">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="J4" s="36">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="K4" s="36">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="L4" s="36">
-        <v>41</v>
-      </c>
-      <c r="M4" s="37">
-        <v>38</v>
-      </c>
-      <c r="N4" s="35">
-        <f>M4-L4</f>
-      </c>
-      <c r="O4" s="35">
-        <f>M4-B4</f>
+        <v>26</v>
+      </c>
+      <c r="M4" s="36">
+        <v>27</v>
+      </c>
+      <c r="N4" s="36">
+        <v>35</v>
+      </c>
+      <c r="O4" s="37">
+        <v>35</v>
+      </c>
+      <c r="P4" s="36">
+        <f>O4-N4</f>
+      </c>
+      <c r="Q4" s="34">
+        <f>O4-B4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B5" s="36">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C5" s="36">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="D5" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E5" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F5" s="36">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G5" s="36">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H5" s="36">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="I5" s="36">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="J5" s="36">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="K5" s="36">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="L5" s="36">
-        <v>26</v>
-      </c>
-      <c r="M5" s="37">
-        <v>24</v>
-      </c>
-      <c r="N5" s="35">
-        <f>M5-L5</f>
-      </c>
-      <c r="O5" s="34">
-        <f>M5-B5</f>
+        <v>11</v>
+      </c>
+      <c r="M5" s="36">
+        <v>11</v>
+      </c>
+      <c r="N5" s="36">
+        <v>17</v>
+      </c>
+      <c r="O5" s="37">
+        <v>17</v>
+      </c>
+      <c r="P5" s="36">
+        <f>O5-N5</f>
+      </c>
+      <c r="Q5" s="34">
+        <f>O5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C6" s="36">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D6" s="36">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E6" s="36">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="F6" s="36">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="G6" s="36">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H6" s="36">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="I6" s="36">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="J6" s="36">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="K6" s="36">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="L6" s="36">
+        <v>5</v>
+      </c>
+      <c r="M6" s="36">
+        <v>8</v>
+      </c>
+      <c r="N6" s="36">
         <v>13</v>
       </c>
-      <c r="M6" s="37">
+      <c r="O6" s="37">
         <v>14</v>
       </c>
-      <c r="N6" s="34">
-        <f>M6-L6</f>
-      </c>
-      <c r="O6" s="35">
-        <f>M6-B6</f>
+      <c r="P6" s="34">
+        <f>O6-N6</f>
+      </c>
+      <c r="Q6" s="34">
+        <f>O6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="C7" s="36">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D7" s="36">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E7" s="36">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="F7" s="36">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="G7" s="36">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="H7" s="36">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="I7" s="36">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="J7" s="36">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="K7" s="36">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="L7" s="36">
-        <v>14</v>
-      </c>
-      <c r="M7" s="37">
-        <v>14</v>
+        <v>5</v>
+      </c>
+      <c r="M7" s="36">
+        <v>9</v>
       </c>
       <c r="N7" s="36">
-        <f>M7-L7</f>
-      </c>
-      <c r="O7" s="35">
-        <f>M7-B7</f>
+        <v>13</v>
+      </c>
+      <c r="O7" s="37">
+        <v>13</v>
+      </c>
+      <c r="P7" s="36">
+        <f>O7-N7</f>
+      </c>
+      <c r="Q7" s="34">
+        <f>O7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="C8" s="36">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D8" s="36">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E8" s="36">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="F8" s="36">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="G8" s="36">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="H8" s="36">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="I8" s="36">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J8" s="36">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="K8" s="36">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L8" s="36">
-        <v>12</v>
-      </c>
-      <c r="M8" s="37">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="M8" s="36">
+        <v>11</v>
       </c>
       <c r="N8" s="36">
-        <f>M8-L8</f>
-      </c>
-      <c r="O8" s="35">
-        <f>M8-B8</f>
+        <v>11</v>
+      </c>
+      <c r="O8" s="37">
+        <v>11</v>
+      </c>
+      <c r="P8" s="36">
+        <f>O8-N8</f>
+      </c>
+      <c r="Q8" s="34">
+        <f>O8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="C9" s="36">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="D9" s="36">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="E9" s="36">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="F9" s="36">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="G9" s="36">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="H9" s="36">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="I9" s="36">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="J9" s="36">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="K9" s="36">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L9" s="36">
-        <v>10</v>
-      </c>
-      <c r="M9" s="37">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="M9" s="36">
+        <v>11</v>
       </c>
       <c r="N9" s="36">
-        <f>M9-L9</f>
-      </c>
-      <c r="O9" s="35">
-        <f>M9-B9</f>
+        <v>11</v>
+      </c>
+      <c r="O9" s="37">
+        <v>11</v>
+      </c>
+      <c r="P9" s="36">
+        <f>O9-N9</f>
+      </c>
+      <c r="Q9" s="34">
+        <f>O9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C10" s="36">
+        <v>1</v>
+      </c>
+      <c r="D10" s="36">
+        <v>1</v>
+      </c>
+      <c r="E10" s="36">
+        <v>1</v>
+      </c>
+      <c r="F10" s="36">
+        <v>3</v>
+      </c>
+      <c r="G10" s="36">
+        <v>3</v>
+      </c>
+      <c r="H10" s="36">
+        <v>6</v>
+      </c>
+      <c r="I10" s="36">
+        <v>6</v>
+      </c>
+      <c r="J10" s="36">
+        <v>6</v>
+      </c>
+      <c r="K10" s="36">
         <v>7</v>
-      </c>
-      <c r="D10" s="36">
-        <v>9</v>
-      </c>
-      <c r="E10" s="36">
-        <v>12</v>
-      </c>
-      <c r="F10" s="36">
-        <v>13</v>
-      </c>
-      <c r="G10" s="36">
-        <v>9</v>
-      </c>
-      <c r="H10" s="36">
-        <v>11</v>
-      </c>
-      <c r="I10" s="36">
-        <v>7</v>
-      </c>
-      <c r="J10" s="36">
-        <v>6</v>
-      </c>
-      <c r="K10" s="36">
-        <v>6</v>
       </c>
       <c r="L10" s="36">
         <v>7</v>
       </c>
-      <c r="M10" s="37">
-        <v>7</v>
+      <c r="M10" s="36">
+        <v>9</v>
       </c>
       <c r="N10" s="36">
-        <f>M10-L10</f>
-      </c>
-      <c r="O10" s="35">
-        <f>M10-B10</f>
+        <v>10</v>
+      </c>
+      <c r="O10" s="37">
+        <v>10</v>
+      </c>
+      <c r="P10" s="36">
+        <f>O10-N10</f>
+      </c>
+      <c r="Q10" s="34">
+        <f>O10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C11" s="36">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D11" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E11" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F11" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G11" s="36">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H11" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I11" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J11" s="36">
         <v>6</v>
@@ -752,14 +806,20 @@
       <c r="L11" s="36">
         <v>7</v>
       </c>
-      <c r="M11" s="37">
-        <v>7</v>
+      <c r="M11" s="36">
+        <v>9</v>
       </c>
       <c r="N11" s="36">
-        <f>M11-L11</f>
-      </c>
-      <c r="O11" s="35">
-        <f>M11-B11</f>
+        <v>9</v>
+      </c>
+      <c r="O11" s="37">
+        <v>9</v>
+      </c>
+      <c r="P11" s="36">
+        <f>O11-N11</f>
+      </c>
+      <c r="Q11" s="34">
+        <f>O11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -769,31 +829,31 @@
         </is>
       </c>
       <c r="B12" s="36">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C12" s="36">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D12" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E12" s="36">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F12" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G12" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H12" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I12" s="36">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J12" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K12" s="36">
         <v>4</v>
@@ -801,14 +861,20 @@
       <c r="L12" s="36">
         <v>4</v>
       </c>
-      <c r="M12" s="37">
+      <c r="M12" s="36">
         <v>5</v>
       </c>
-      <c r="N12" s="34">
-        <f>M12-L12</f>
-      </c>
-      <c r="O12" s="35">
-        <f>M12-B12</f>
+      <c r="N12" s="36">
+        <v>8</v>
+      </c>
+      <c r="O12" s="37">
+        <v>8</v>
+      </c>
+      <c r="P12" s="36">
+        <f>O12-N12</f>
+      </c>
+      <c r="Q12" s="34">
+        <f>O12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -818,46 +884,52 @@
         </is>
       </c>
       <c r="B13" s="36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C13" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D13" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E13" s="36">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F13" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G13" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H13" s="36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I13" s="36">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J13" s="36">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K13" s="36">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L13" s="36">
-        <v>4</v>
-      </c>
-      <c r="M13" s="37">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="M13" s="36">
+        <v>1</v>
       </c>
       <c r="N13" s="36">
-        <f>M13-L13</f>
-      </c>
-      <c r="O13" s="35">
-        <f>M13-B13</f>
+        <v>2</v>
+      </c>
+      <c r="O13" s="37">
+        <v>3</v>
+      </c>
+      <c r="P13" s="34">
+        <f>O13-N13</f>
+      </c>
+      <c r="Q13" s="34">
+        <f>O13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -867,31 +939,31 @@
         </is>
       </c>
       <c r="B14" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C14" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D14" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E14" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F14" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G14" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H14" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I14" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J14" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K14" s="36">
         <v>0</v>
@@ -899,14 +971,20 @@
       <c r="L14" s="36">
         <v>0</v>
       </c>
-      <c r="M14" s="37">
+      <c r="M14" s="36">
         <v>0</v>
       </c>
       <c r="N14" s="36">
-        <f>M14-L14</f>
-      </c>
-      <c r="O14" s="35">
-        <f>M14-B14</f>
+        <v>1</v>
+      </c>
+      <c r="O14" s="37">
+        <v>1</v>
+      </c>
+      <c r="P14" s="36">
+        <f>O14-N14</f>
+      </c>
+      <c r="Q14" s="34">
+        <f>O14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -951,11 +1029,17 @@
       <c r="M15" s="38">
         <f>SUM(M4:M14)</f>
       </c>
-      <c r="N15" s="41">
-        <f>M15-L15</f>
-      </c>
-      <c r="O15" s="41">
-        <f>M15-B15</f>
+      <c r="N15" s="38">
+        <f>SUM(N4:N14)</f>
+      </c>
+      <c r="O15" s="38">
+        <f>SUM(O4:O14)</f>
+      </c>
+      <c r="P15" s="40">
+        <f>O15-N15</f>
+      </c>
+      <c r="Q15" s="40">
+        <f>O15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1034,6 +1118,16 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="P16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1042,47 +1136,53 @@
         </is>
       </c>
       <c r="B17" s="36">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C17" s="36">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="D17" s="36">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E17" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F17" s="36">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G17" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H17" s="36">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="I17" s="36">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="J17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="K17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="L17" s="36">
-        <v>61</v>
-      </c>
-      <c r="M17" s="37">
-        <v>8</v>
-      </c>
-      <c r="N17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O17" s="36" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="M17" s="36">
+        <v>0</v>
+      </c>
+      <c r="N17" s="36">
+        <v>0</v>
+      </c>
+      <c r="O17" s="37">
+        <v>0</v>
+      </c>
+      <c r="P17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1095,47 +1195,53 @@
         </is>
       </c>
       <c r="B18" s="36">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="C18" s="36">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="D18" s="36">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E18" s="36">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F18" s="36">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="G18" s="36">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H18" s="36">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="I18" s="36">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="J18" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K18" s="36">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="L18" s="36">
-        <v>25</v>
-      </c>
-      <c r="M18" s="37">
-        <v>5</v>
-      </c>
-      <c r="N18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O18" s="36" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="M18" s="36">
+        <v>14</v>
+      </c>
+      <c r="N18" s="36">
+        <v>29</v>
+      </c>
+      <c r="O18" s="37">
+        <v>2</v>
+      </c>
+      <c r="P18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1180,15 +1286,21 @@
       <c r="L19" s="36">
         <f>L18-L17</f>
       </c>
-      <c r="M19" s="37">
+      <c r="M19" s="36">
         <f>M18-M17</f>
       </c>
-      <c r="N19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O19" s="36" t="inlineStr">
+      <c r="N19" s="36">
+        <f>N18-N17</f>
+      </c>
+      <c r="O19" s="37">
+        <f>O18-O17</f>
+      </c>
+      <c r="P19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1201,47 +1313,53 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C20" s="36">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D20" s="36">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E20" s="36">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F20" s="36">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="G20" s="36">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H20" s="36">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I20" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J20" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K20" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L20" s="36">
+        <v>5</v>
+      </c>
+      <c r="M20" s="36">
+        <v>6</v>
+      </c>
+      <c r="N20" s="36">
         <v>7</v>
       </c>
-      <c r="M20" s="37">
+      <c r="O20" s="37">
         <v>7</v>
       </c>
-      <c r="N20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O20" s="36" t="inlineStr">
+      <c r="P20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
fix(sorvete): relatorio xlsx regenerado terminando em 13/10 (nao 14/10) A planilha baixavel ainda mostrava ate 14/10 porque foi gerada antes da correcao do painel_sorvete.cjs (serie sempre ate o dia anterior). Regenerada agora a partir do sorvete.json corrigido: 13 dias (01/10 a 13/10), ultimo dia 13/10, TOTAL BRASIL 13/10=130. Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -283,14 +283,13 @@
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="10" customWidth="1"/>
-    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 14/10 · variação 13/10 → 14/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 13/10 · variação 12/10 → 13/10</t>
         </is>
       </c>
     </row>
@@ -368,15 +367,10 @@
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">14/10</t>
+          <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
       <c r="P3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Variação DIA</t>
-        </is>
-      </c>
-      <c r="Q3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -389,52 +383,49 @@
         </is>
       </c>
       <c r="B4" s="36">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="C4" s="36">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="D4" s="36">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="E4" s="36">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="F4" s="36">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="G4" s="36">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="H4" s="36">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="I4" s="36">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="J4" s="36">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="K4" s="36">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L4" s="36">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="M4" s="36">
-        <v>27</v>
-      </c>
-      <c r="N4" s="36">
+        <v>38</v>
+      </c>
+      <c r="N4" s="37">
         <v>35</v>
       </c>
-      <c r="O4" s="37">
-        <v>35</v>
-      </c>
-      <c r="P4" s="36">
-        <f>O4-N4</f>
-      </c>
-      <c r="Q4" s="34">
-        <f>O4-B4</f>
+      <c r="O4" s="35">
+        <f>N4-M4</f>
+      </c>
+      <c r="P4" s="35">
+        <f>N4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -444,162 +435,153 @@
         </is>
       </c>
       <c r="B5" s="36">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C5" s="36">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D5" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E5" s="36">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F5" s="36">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G5" s="36">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="H5" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I5" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="J5" s="36">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="K5" s="36">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="L5" s="36">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="M5" s="36">
-        <v>11</v>
-      </c>
-      <c r="N5" s="36">
+        <v>12</v>
+      </c>
+      <c r="N5" s="37">
         <v>17</v>
       </c>
-      <c r="O5" s="37">
-        <v>17</v>
-      </c>
-      <c r="P5" s="36">
-        <f>O5-N5</f>
-      </c>
-      <c r="Q5" s="34">
-        <f>O5-B5</f>
+      <c r="O5" s="34">
+        <f>N5-M5</f>
+      </c>
+      <c r="P5" s="35">
+        <f>N5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C6" s="36">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D6" s="36">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E6" s="36">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F6" s="36">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G6" s="36">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H6" s="36">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I6" s="36">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J6" s="36">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K6" s="36">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L6" s="36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" s="36">
-        <v>8</v>
-      </c>
-      <c r="N6" s="36">
+        <v>7</v>
+      </c>
+      <c r="N6" s="37">
         <v>13</v>
       </c>
-      <c r="O6" s="37">
-        <v>14</v>
+      <c r="O6" s="34">
+        <f>N6-M6</f>
       </c>
       <c r="P6" s="34">
-        <f>O6-N6</f>
-      </c>
-      <c r="Q6" s="34">
-        <f>O6-B6</f>
+        <f>N6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="C7" s="36">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="D7" s="36">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="E7" s="36">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="F7" s="36">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="G7" s="36">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H7" s="36">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="I7" s="36">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="J7" s="36">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="K7" s="36">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="L7" s="36">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="M7" s="36">
-        <v>9</v>
-      </c>
-      <c r="N7" s="36">
+        <v>10</v>
+      </c>
+      <c r="N7" s="37">
         <v>13</v>
       </c>
-      <c r="O7" s="37">
-        <v>13</v>
-      </c>
-      <c r="P7" s="36">
-        <f>O7-N7</f>
-      </c>
-      <c r="Q7" s="34">
-        <f>O7-B7</f>
+      <c r="O7" s="34">
+        <f>N7-M7</f>
+      </c>
+      <c r="P7" s="35">
+        <f>N7-B7</f>
       </c>
     </row>
     <row r="8">
@@ -609,52 +591,49 @@
         </is>
       </c>
       <c r="B8" s="36">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C8" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D8" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E8" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F8" s="36">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="G8" s="36">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H8" s="36">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="I8" s="36">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="J8" s="36">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="K8" s="36">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="L8" s="36">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="M8" s="36">
+        <v>24</v>
+      </c>
+      <c r="N8" s="37">
         <v>11</v>
       </c>
-      <c r="N8" s="36">
-        <v>11</v>
-      </c>
-      <c r="O8" s="37">
-        <v>11</v>
-      </c>
-      <c r="P8" s="36">
-        <f>O8-N8</f>
-      </c>
-      <c r="Q8" s="34">
-        <f>O8-B8</f>
+      <c r="O8" s="35">
+        <f>N8-M8</f>
+      </c>
+      <c r="P8" s="35">
+        <f>N8-B8</f>
       </c>
     </row>
     <row r="9">
@@ -664,52 +643,49 @@
         </is>
       </c>
       <c r="B9" s="36">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="C9" s="36">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D9" s="36">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E9" s="36">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F9" s="36">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="G9" s="36">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="H9" s="36">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="I9" s="36">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="J9" s="36">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="K9" s="36">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="L9" s="36">
+        <v>14</v>
+      </c>
+      <c r="M9" s="36">
+        <v>14</v>
+      </c>
+      <c r="N9" s="37">
         <v>11</v>
       </c>
-      <c r="M9" s="36">
-        <v>11</v>
-      </c>
-      <c r="N9" s="36">
-        <v>11</v>
-      </c>
-      <c r="O9" s="37">
-        <v>11</v>
-      </c>
-      <c r="P9" s="36">
-        <f>O9-N9</f>
-      </c>
-      <c r="Q9" s="34">
-        <f>O9-B9</f>
+      <c r="O9" s="35">
+        <f>N9-M9</f>
+      </c>
+      <c r="P9" s="35">
+        <f>N9-B9</f>
       </c>
     </row>
     <row r="10">
@@ -719,28 +695,28 @@
         </is>
       </c>
       <c r="B10" s="36">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C10" s="36">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E10" s="36">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F10" s="36">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G10" s="36">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="H10" s="36">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I10" s="36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J10" s="36">
         <v>6</v>
@@ -752,19 +728,16 @@
         <v>7</v>
       </c>
       <c r="M10" s="36">
-        <v>9</v>
-      </c>
-      <c r="N10" s="36">
+        <v>7</v>
+      </c>
+      <c r="N10" s="37">
         <v>10</v>
       </c>
-      <c r="O10" s="37">
-        <v>10</v>
-      </c>
-      <c r="P10" s="36">
-        <f>O10-N10</f>
-      </c>
-      <c r="Q10" s="34">
-        <f>O10-B10</f>
+      <c r="O10" s="34">
+        <f>N10-M10</f>
+      </c>
+      <c r="P10" s="35">
+        <f>N10-B10</f>
       </c>
     </row>
     <row r="11">
@@ -774,52 +747,49 @@
         </is>
       </c>
       <c r="B11" s="36">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C11" s="36">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D11" s="36">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E11" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F11" s="36">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="G11" s="36">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H11" s="36">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="I11" s="36">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="J11" s="36">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="K11" s="36">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="L11" s="36">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="M11" s="36">
+        <v>14</v>
+      </c>
+      <c r="N11" s="37">
         <v>9</v>
       </c>
-      <c r="N11" s="36">
-        <v>9</v>
-      </c>
-      <c r="O11" s="37">
-        <v>9</v>
-      </c>
-      <c r="P11" s="36">
-        <f>O11-N11</f>
-      </c>
-      <c r="Q11" s="34">
-        <f>O11-B11</f>
+      <c r="O11" s="35">
+        <f>N11-M11</f>
+      </c>
+      <c r="P11" s="35">
+        <f>N11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -829,31 +799,31 @@
         </is>
       </c>
       <c r="B12" s="36">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C12" s="36">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D12" s="36">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E12" s="36">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I12" s="36">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12" s="36">
         <v>4</v>
@@ -864,17 +834,14 @@
       <c r="M12" s="36">
         <v>5</v>
       </c>
-      <c r="N12" s="36">
+      <c r="N12" s="37">
         <v>8</v>
       </c>
-      <c r="O12" s="37">
-        <v>8</v>
-      </c>
-      <c r="P12" s="36">
-        <f>O12-N12</f>
-      </c>
-      <c r="Q12" s="34">
-        <f>O12-B12</f>
+      <c r="O12" s="34">
+        <f>N12-M12</f>
+      </c>
+      <c r="P12" s="35">
+        <f>N12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -884,52 +851,49 @@
         </is>
       </c>
       <c r="B13" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C13" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D13" s="36">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E13" s="36">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F13" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G13" s="36">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H13" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I13" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J13" s="36">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K13" s="36">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L13" s="36">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M13" s="36">
-        <v>1</v>
-      </c>
-      <c r="N13" s="36">
+        <v>4</v>
+      </c>
+      <c r="N13" s="37">
         <v>2</v>
       </c>
-      <c r="O13" s="37">
-        <v>3</v>
-      </c>
-      <c r="P13" s="34">
-        <f>O13-N13</f>
-      </c>
-      <c r="Q13" s="34">
-        <f>O13-B13</f>
+      <c r="O13" s="35">
+        <f>N13-M13</f>
+      </c>
+      <c r="P13" s="35">
+        <f>N13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -939,31 +903,31 @@
         </is>
       </c>
       <c r="B14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H14" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K14" s="36">
         <v>0</v>
@@ -974,17 +938,14 @@
       <c r="M14" s="36">
         <v>0</v>
       </c>
-      <c r="N14" s="36">
+      <c r="N14" s="37">
         <v>1</v>
       </c>
-      <c r="O14" s="37">
-        <v>1</v>
-      </c>
-      <c r="P14" s="36">
-        <f>O14-N14</f>
-      </c>
-      <c r="Q14" s="34">
-        <f>O14-B14</f>
+      <c r="O14" s="34">
+        <f>N14-M14</f>
+      </c>
+      <c r="P14" s="35">
+        <f>N14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1032,14 +993,11 @@
       <c r="N15" s="38">
         <f>SUM(N4:N14)</f>
       </c>
-      <c r="O15" s="38">
-        <f>SUM(O4:O14)</f>
-      </c>
-      <c r="P15" s="40">
-        <f>O15-N15</f>
-      </c>
-      <c r="Q15" s="40">
-        <f>O15-B15</f>
+      <c r="O15" s="41">
+        <f>N15-M15</f>
+      </c>
+      <c r="P15" s="41">
+        <f>N15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1123,11 +1081,6 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="Q16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1136,53 +1089,50 @@
         </is>
       </c>
       <c r="B17" s="36">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C17" s="36">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="D17" s="36">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E17" s="36">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F17" s="36">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G17" s="36">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H17" s="36">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I17" s="36">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J17" s="36">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="K17" s="36">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="L17" s="36">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="M17" s="36">
-        <v>0</v>
-      </c>
-      <c r="N17" s="36">
-        <v>0</v>
-      </c>
-      <c r="O17" s="37">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="N17" s="37">
+        <v>22</v>
+      </c>
+      <c r="O17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="P17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1195,53 +1145,50 @@
         </is>
       </c>
       <c r="B18" s="36">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="C18" s="36">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D18" s="36">
+        <v>28</v>
+      </c>
+      <c r="E18" s="36">
+        <v>21</v>
+      </c>
+      <c r="F18" s="36">
+        <v>31</v>
+      </c>
+      <c r="G18" s="36">
+        <v>20</v>
+      </c>
+      <c r="H18" s="36">
+        <v>33</v>
+      </c>
+      <c r="I18" s="36">
         <v>2</v>
       </c>
-      <c r="E18" s="36">
-        <v>0</v>
-      </c>
-      <c r="F18" s="36">
-        <v>4</v>
-      </c>
-      <c r="G18" s="36">
-        <v>1</v>
-      </c>
-      <c r="H18" s="36">
-        <v>6</v>
-      </c>
-      <c r="I18" s="36">
-        <v>3</v>
-      </c>
       <c r="J18" s="36">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="K18" s="36">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="L18" s="36">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="M18" s="36">
-        <v>14</v>
-      </c>
-      <c r="N18" s="36">
-        <v>29</v>
-      </c>
-      <c r="O18" s="37">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="N18" s="37">
+        <v>37</v>
+      </c>
+      <c r="O18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="P18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1289,18 +1236,15 @@
       <c r="M19" s="36">
         <f>M18-M17</f>
       </c>
-      <c r="N19" s="36">
+      <c r="N19" s="37">
         <f>N18-N17</f>
       </c>
-      <c r="O19" s="37">
-        <f>O18-O17</f>
+      <c r="O19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="P19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1313,53 +1257,50 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C20" s="36">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D20" s="36">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E20" s="36">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F20" s="36">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G20" s="36">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H20" s="36">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I20" s="36">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="J20" s="36">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K20" s="36">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L20" s="36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M20" s="36">
-        <v>6</v>
-      </c>
-      <c r="N20" s="36">
         <v>7</v>
       </c>
-      <c r="O20" s="37">
+      <c r="N20" s="37">
         <v>7</v>
       </c>
+      <c r="O20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
       <c r="P20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
fix(sorvete): historico 01-12/10 hardcodado (fonte verdade) + dia 13 calculado Correcao definitiva apos multiplas iteracoes: 1. Dias 01/10 a 12/10: valores HARDCODADOS da planilha/imagem validada pelo Christian (fonte de verdade absoluta). A logica automatica falhava porque as fotos diarias sao snapshots de horarios arbitrarios (ex: foto 12/10 foi 11:42, nao 23:59), causando sub/supercontagem. Hardcodar garante que o historico nunca mude. TOTAL 12/10=135 (RJ=38, MINAS BAHIA=24, SP SUL=14, SUL=14, CENTRO OESTE=12, NE=10, etc.). 2. Dia 13/10: calculado automaticamente com logica nova (state nao-fechado + prioridade 1-Critica/2-Alta) usando a ultima foto disponivel, na janela 12/10 23:40 ate 13/10 23:49. TOTAL 13/10=130. 3. Serie termina SEMPRE no dia anterior ao argumento (nunca inclui hoje). Rodando com 2026-10-14, termina em 13/10. Regenerado sorvete.json e relatorio_sorvete.xlsx (13 dias, ultimo 13/10). Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -383,48 +383,48 @@
         </is>
       </c>
       <c r="B4" s="36">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="C4" s="36">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="D4" s="36">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="E4" s="36">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="F4" s="36">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="G4" s="36">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="H4" s="36">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="I4" s="36">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="J4" s="36">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="K4" s="36">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="L4" s="36">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="M4" s="36">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N4" s="37">
         <v>35</v>
       </c>
-      <c r="O4" s="34">
+      <c r="O4" s="35">
         <f>N4-M4</f>
       </c>
-      <c r="P4" s="34">
+      <c r="P4" s="35">
         <f>N4-B4</f>
       </c>
     </row>
@@ -435,40 +435,40 @@
         </is>
       </c>
       <c r="B5" s="36">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C5" s="36">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D5" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E5" s="36">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F5" s="36">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G5" s="36">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="H5" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I5" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="J5" s="36">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="K5" s="36">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="L5" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M5" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N5" s="37">
         <v>17</v>
@@ -476,7 +476,7 @@
       <c r="O5" s="34">
         <f>N5-M5</f>
       </c>
-      <c r="P5" s="34">
+      <c r="P5" s="35">
         <f>N5-B5</f>
       </c>
     </row>
@@ -487,40 +487,40 @@
         </is>
       </c>
       <c r="B6" s="36">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C6" s="36">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D6" s="36">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E6" s="36">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F6" s="36">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G6" s="36">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H6" s="36">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I6" s="36">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J6" s="36">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K6" s="36">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" s="36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M6" s="36">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N6" s="37">
         <v>13</v>
@@ -539,40 +539,40 @@
         </is>
       </c>
       <c r="B7" s="36">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="C7" s="36">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="D7" s="36">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="E7" s="36">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="F7" s="36">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="G7" s="36">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="H7" s="36">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="I7" s="36">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J7" s="36">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="K7" s="36">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="L7" s="36">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="M7" s="36">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N7" s="37">
         <v>13</v>
@@ -580,7 +580,7 @@
       <c r="O7" s="34">
         <f>N7-M7</f>
       </c>
-      <c r="P7" s="34">
+      <c r="P7" s="35">
         <f>N7-B7</f>
       </c>
     </row>
@@ -591,48 +591,48 @@
         </is>
       </c>
       <c r="B8" s="36">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C8" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D8" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E8" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F8" s="36">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="G8" s="36">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H8" s="36">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="I8" s="36">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J8" s="36">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="K8" s="36">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="L8" s="36">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="M8" s="36">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="N8" s="37">
         <v>11</v>
       </c>
-      <c r="O8" s="36">
+      <c r="O8" s="35">
         <f>N8-M8</f>
       </c>
-      <c r="P8" s="34">
+      <c r="P8" s="35">
         <f>N8-B8</f>
       </c>
     </row>
@@ -643,48 +643,48 @@
         </is>
       </c>
       <c r="B9" s="36">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="C9" s="36">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D9" s="36">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E9" s="36">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F9" s="36">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="G9" s="36">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="H9" s="36">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="I9" s="36">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="J9" s="36">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="K9" s="36">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="L9" s="36">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M9" s="36">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="N9" s="37">
         <v>11</v>
       </c>
-      <c r="O9" s="36">
+      <c r="O9" s="35">
         <f>N9-M9</f>
       </c>
-      <c r="P9" s="34">
+      <c r="P9" s="35">
         <f>N9-B9</f>
       </c>
     </row>
@@ -695,28 +695,28 @@
         </is>
       </c>
       <c r="B10" s="36">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C10" s="36">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E10" s="36">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F10" s="36">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G10" s="36">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="H10" s="36">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I10" s="36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J10" s="36">
         <v>6</v>
@@ -728,7 +728,7 @@
         <v>7</v>
       </c>
       <c r="M10" s="36">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N10" s="37">
         <v>10</v>
@@ -736,7 +736,7 @@
       <c r="O10" s="34">
         <f>N10-M10</f>
       </c>
-      <c r="P10" s="34">
+      <c r="P10" s="35">
         <f>N10-B10</f>
       </c>
     </row>
@@ -747,48 +747,48 @@
         </is>
       </c>
       <c r="B11" s="36">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C11" s="36">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D11" s="36">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E11" s="36">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F11" s="36">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="G11" s="36">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H11" s="36">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="I11" s="36">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="J11" s="36">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="K11" s="36">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="L11" s="36">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M11" s="36">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N11" s="37">
         <v>9</v>
       </c>
-      <c r="O11" s="36">
+      <c r="O11" s="35">
         <f>N11-M11</f>
       </c>
-      <c r="P11" s="34">
+      <c r="P11" s="35">
         <f>N11-B11</f>
       </c>
     </row>
@@ -799,31 +799,31 @@
         </is>
       </c>
       <c r="B12" s="36">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C12" s="36">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D12" s="36">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E12" s="36">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I12" s="36">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J12" s="36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12" s="36">
         <v>4</v>
@@ -840,7 +840,7 @@
       <c r="O12" s="34">
         <f>N12-M12</f>
       </c>
-      <c r="P12" s="34">
+      <c r="P12" s="35">
         <f>N12-B12</f>
       </c>
     </row>
@@ -851,48 +851,48 @@
         </is>
       </c>
       <c r="B13" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C13" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D13" s="36">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E13" s="36">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F13" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G13" s="36">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H13" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I13" s="36">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J13" s="36">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K13" s="36">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L13" s="36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M13" s="36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N13" s="37">
         <v>2</v>
       </c>
-      <c r="O13" s="34">
+      <c r="O13" s="35">
         <f>N13-M13</f>
       </c>
-      <c r="P13" s="34">
+      <c r="P13" s="35">
         <f>N13-B13</f>
       </c>
     </row>
@@ -903,31 +903,31 @@
         </is>
       </c>
       <c r="B14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H14" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I14" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K14" s="36">
         <v>0</v>
@@ -944,7 +944,7 @@
       <c r="O14" s="34">
         <f>N14-M14</f>
       </c>
-      <c r="P14" s="34">
+      <c r="P14" s="35">
         <f>N14-B14</f>
       </c>
     </row>
@@ -993,10 +993,10 @@
       <c r="N15" s="38">
         <f>SUM(N4:N14)</f>
       </c>
-      <c r="O15" s="40">
+      <c r="O15" s="41">
         <f>N15-M15</f>
       </c>
-      <c r="P15" s="40">
+      <c r="P15" s="41">
         <f>N15-B15</f>
       </c>
     </row>
@@ -1089,43 +1089,43 @@
         </is>
       </c>
       <c r="B17" s="36">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C17" s="36">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="D17" s="36">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E17" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F17" s="36">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G17" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H17" s="36">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="I17" s="36">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="J17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="K17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="L17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="M17" s="36">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="N17" s="37">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="O17" s="36" t="inlineStr">
         <is>
@@ -1145,43 +1145,43 @@
         </is>
       </c>
       <c r="B18" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C18" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D18" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E18" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G18" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H18" s="36">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I18" s="36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J18" s="36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K18" s="36">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="L18" s="36">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="M18" s="36">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="N18" s="37">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="O18" s="36" t="inlineStr">
         <is>
@@ -1257,40 +1257,40 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L20" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M20" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N20" s="37">
         <v>7</v>

</xml_diff>

<commit_message>
fix(sorvete): restaura historico 01-13/10 da imagem de ontem + calcula so o dia 14
Pedido Christian 15/10/2026: manter EXATAMENTE o mesmo historico
apresentado ontem (imagem 33), so mudando o ultimo dia (14/10).
Antes eu tinha alterado o 13/10 para TOTAL=106 (imagem 34) -- errado,
deveria seguir a imagem de ontem onde 13/10=130.

Restaurado:
- 01-12/10: hardcodado conforme imagem original (TOTAL 12/10=135)
- 13/10: RESTAURADO para TOTAL=130 (RJ=35, CENTRO OESTE=17,
  BK FOGO LESTE=13, NE=13, MINAS BAHIA=11, SUL=11, SP INT SUL=10,
  SP SUL=9, SP INT NORTE=8, BK FOGO NORTE=2, BK FOGO CL=1)
- 14/10: UNICO dia calculado automaticamente (state+prioridade 1-2,
  janela 13/10 23:40->14/10 23:49). TOTAL 14/10=125.

Serie termina em 14/10 (ontem, hoje eh 15/10). Sem coluna 15/10.
Regenerado sorvete.json e relatorio_sorvete.xlsx (14 dias).
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -425,7 +425,7 @@
         <v>38</v>
       </c>
       <c r="N4" s="36">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O4" s="37">
         <v>38</v>
@@ -480,12 +480,12 @@
         <v>12</v>
       </c>
       <c r="N5" s="36">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="O5" s="37">
         <v>16</v>
       </c>
-      <c r="P5" s="34">
+      <c r="P5" s="35">
         <f>O5-N5</f>
       </c>
       <c r="Q5" s="35">
@@ -535,12 +535,12 @@
         <v>7</v>
       </c>
       <c r="N6" s="36">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O6" s="37">
         <v>13</v>
       </c>
-      <c r="P6" s="34">
+      <c r="P6" s="36">
         <f>O6-N6</f>
       </c>
       <c r="Q6" s="34">
@@ -590,12 +590,12 @@
         <v>10</v>
       </c>
       <c r="N7" s="36">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O7" s="37">
         <v>12</v>
       </c>
-      <c r="P7" s="34">
+      <c r="P7" s="35">
         <f>O7-N7</f>
       </c>
       <c r="Q7" s="35">
@@ -645,12 +645,12 @@
         <v>14</v>
       </c>
       <c r="N8" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O8" s="37">
         <v>10</v>
       </c>
-      <c r="P8" s="34">
+      <c r="P8" s="35">
         <f>O8-N8</f>
       </c>
       <c r="Q8" s="35">
@@ -700,12 +700,12 @@
         <v>14</v>
       </c>
       <c r="N9" s="36">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O9" s="37">
         <v>9</v>
       </c>
-      <c r="P9" s="34">
+      <c r="P9" s="36">
         <f>O9-N9</f>
       </c>
       <c r="Q9" s="35">
@@ -755,12 +755,12 @@
         <v>24</v>
       </c>
       <c r="N10" s="36">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O10" s="37">
         <v>8</v>
       </c>
-      <c r="P10" s="36">
+      <c r="P10" s="35">
         <f>O10-N10</f>
       </c>
       <c r="Q10" s="35">
@@ -810,12 +810,12 @@
         <v>7</v>
       </c>
       <c r="N11" s="36">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O11" s="37">
         <v>7</v>
       </c>
-      <c r="P11" s="34">
+      <c r="P11" s="35">
         <f>O11-N11</f>
       </c>
       <c r="Q11" s="35">
@@ -865,12 +865,12 @@
         <v>5</v>
       </c>
       <c r="N12" s="36">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O12" s="37">
         <v>6</v>
       </c>
-      <c r="P12" s="36">
+      <c r="P12" s="35">
         <f>O12-N12</f>
       </c>
       <c r="Q12" s="35">
@@ -1035,7 +1035,7 @@
       <c r="O15" s="38">
         <f>SUM(O4:O14)</f>
       </c>
-      <c r="P15" s="40">
+      <c r="P15" s="41">
         <f>O15-N15</f>
       </c>
       <c r="Q15" s="41">

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-15 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -428,9 +428,9 @@
         <v>35</v>
       </c>
       <c r="O4" s="37">
-        <v>38</v>
-      </c>
-      <c r="P4" s="34">
+        <v>33</v>
+      </c>
+      <c r="P4" s="35">
         <f>O4-N4</f>
       </c>
       <c r="Q4" s="35">
@@ -483,7 +483,7 @@
         <v>17</v>
       </c>
       <c r="O5" s="37">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P5" s="35">
         <f>O5-N5</f>
@@ -495,160 +495,160 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="C6" s="36">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="D6" s="36">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="E6" s="36">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="F6" s="36">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="G6" s="36">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H6" s="36">
+        <v>27</v>
+      </c>
+      <c r="I6" s="36">
+        <v>25</v>
+      </c>
+      <c r="J6" s="36">
+        <v>20</v>
+      </c>
+      <c r="K6" s="36">
+        <v>18</v>
+      </c>
+      <c r="L6" s="36">
+        <v>14</v>
+      </c>
+      <c r="M6" s="36">
+        <v>14</v>
+      </c>
+      <c r="N6" s="36">
         <v>11</v>
       </c>
-      <c r="I6" s="36">
-        <v>7</v>
-      </c>
-      <c r="J6" s="36">
-        <v>6</v>
-      </c>
-      <c r="K6" s="36">
-        <v>6</v>
-      </c>
-      <c r="L6" s="36">
-        <v>7</v>
-      </c>
-      <c r="M6" s="36">
-        <v>7</v>
-      </c>
-      <c r="N6" s="36">
-        <v>13</v>
-      </c>
       <c r="O6" s="37">
-        <v>13</v>
-      </c>
-      <c r="P6" s="36">
+        <v>10</v>
+      </c>
+      <c r="P6" s="35">
         <f>O6-N6</f>
       </c>
-      <c r="Q6" s="34">
+      <c r="Q6" s="35">
         <f>O6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="C7" s="36">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="D7" s="36">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="E7" s="36">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="F7" s="36">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="G7" s="36">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="H7" s="36">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="I7" s="36">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="J7" s="36">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K7" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L7" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="M7" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N7" s="36">
         <v>13</v>
       </c>
       <c r="O7" s="37">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="P7" s="35">
         <f>O7-N7</f>
       </c>
-      <c r="Q7" s="35">
+      <c r="Q7" s="36">
         <f>O7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C8" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D8" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="E8" s="36">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F8" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G8" s="36">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H8" s="36">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I8" s="36">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J8" s="36">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K8" s="36">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="L8" s="36">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="M8" s="36">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N8" s="36">
         <v>11</v>
       </c>
       <c r="O8" s="37">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P8" s="35">
         <f>O8-N8</f>
@@ -660,52 +660,52 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="C9" s="36">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D9" s="36">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E9" s="36">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F9" s="36">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="G9" s="36">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H9" s="36">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="I9" s="36">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="J9" s="36">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K9" s="36">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="L9" s="36">
+        <v>10</v>
+      </c>
+      <c r="M9" s="36">
+        <v>10</v>
+      </c>
+      <c r="N9" s="36">
         <v>13</v>
       </c>
-      <c r="M9" s="36">
-        <v>14</v>
-      </c>
-      <c r="N9" s="36">
-        <v>9</v>
-      </c>
       <c r="O9" s="37">
-        <v>9</v>
-      </c>
-      <c r="P9" s="36">
+        <v>8</v>
+      </c>
+      <c r="P9" s="35">
         <f>O9-N9</f>
       </c>
       <c r="Q9" s="35">
@@ -715,50 +715,50 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C10" s="36">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D10" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E10" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F10" s="36">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="G10" s="36">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H10" s="36">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="I10" s="36">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J10" s="36">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="K10" s="36">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="L10" s="36">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="M10" s="36">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="N10" s="36">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O10" s="37">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P10" s="35">
         <f>O10-N10</f>
@@ -770,47 +770,47 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C11" s="36">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D11" s="36">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E11" s="36">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F11" s="36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G11" s="36">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H11" s="36">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="I11" s="36">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="J11" s="36">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="K11" s="36">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="L11" s="36">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M11" s="36">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="N11" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O11" s="37">
         <v>7</v>
@@ -868,7 +868,7 @@
         <v>8</v>
       </c>
       <c r="O12" s="37">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P12" s="35">
         <f>O12-N12</f>
@@ -923,7 +923,7 @@
         <v>1</v>
       </c>
       <c r="O13" s="37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P13" s="34">
         <f>O13-N13</f>
@@ -978,9 +978,9 @@
         <v>2</v>
       </c>
       <c r="O14" s="37">
-        <v>3</v>
-      </c>
-      <c r="P14" s="34">
+        <v>0</v>
+      </c>
+      <c r="P14" s="35">
         <f>O14-N14</f>
       </c>
       <c r="Q14" s="35">
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="37">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="P18" s="36" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="37">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P20" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(sorvete): corrige 14/10 para TOTAL=125 (fonte verdade) + acrescenta dia 15
Pedido Christian 16/10/2026: a imagem apresentada ontem (37.png) eh
a fonte da verdade. Manter EXATAMENTE o historico 01-14/10 dela e
acrescentar so o dia 15/10.

Correcao no HISTORICO_FIXO do dia 14/10 (estava TOTAL=103, errado):
- 14/10: TOTAL=125 (RJ=38, CENTRO OESTE=16, BK FOGO LESTE=13, NE=12,
SUL=10, SP SUL=9, MINAS BAHIA=8, SP INT SUL=7, SP INT NORTE=6,
BK FOGO CL=3, BK FOGO NORTE=3) -- bate com a imagem fonte de verdade.

Historico 01-13/10 mantido intacto (12/10=135, 13/10=130).
Dia 15/10: UNICO dia calculado automaticamente (state+prioridade 1-2,
janela 14/10 23:40->15/10 23:49). TOTAL 15/10=124.
Serie termina em 15/10 (ontem, hoje eh 16/10). Sem coluna 16/10.
Regenerado sorvete.json e relatorio_sorvete.xlsx (15 dias).
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -434,7 +434,7 @@
         <v>35</v>
       </c>
       <c r="O4" s="36">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="P4" s="37">
         <v>39</v>
@@ -492,7 +492,7 @@
         <v>13</v>
       </c>
       <c r="O5" s="36">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="P5" s="37">
         <v>15</v>
@@ -550,12 +550,12 @@
         <v>17</v>
       </c>
       <c r="O6" s="36">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P6" s="37">
         <v>14</v>
       </c>
-      <c r="Q6" s="36">
+      <c r="Q6" s="35">
         <f>P6-O6</f>
       </c>
       <c r="R6" s="35">
@@ -608,12 +608,12 @@
         <v>13</v>
       </c>
       <c r="O7" s="36">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="P7" s="37">
         <v>13</v>
       </c>
-      <c r="Q7" s="34">
+      <c r="Q7" s="36">
         <f>P7-O7</f>
       </c>
       <c r="R7" s="34">
@@ -840,12 +840,12 @@
         <v>9</v>
       </c>
       <c r="O11" s="36">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P11" s="37">
         <v>7</v>
       </c>
-      <c r="Q11" s="36">
+      <c r="Q11" s="35">
         <f>P11-O11</f>
       </c>
       <c r="R11" s="35">
@@ -898,12 +898,12 @@
         <v>8</v>
       </c>
       <c r="O12" s="36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P12" s="37">
         <v>5</v>
       </c>
-      <c r="Q12" s="36">
+      <c r="Q12" s="35">
         <f>P12-O12</f>
       </c>
       <c r="R12" s="35">
@@ -956,12 +956,12 @@
         <v>1</v>
       </c>
       <c r="O13" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P13" s="37">
         <v>2</v>
       </c>
-      <c r="Q13" s="36">
+      <c r="Q13" s="35">
         <f>P13-O13</f>
       </c>
       <c r="R13" s="35">
@@ -1014,12 +1014,12 @@
         <v>2</v>
       </c>
       <c r="O14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P14" s="37">
         <v>0</v>
       </c>
-      <c r="Q14" s="36">
+      <c r="Q14" s="35">
         <f>P14-O14</f>
       </c>
       <c r="R14" s="35">
@@ -1077,7 +1077,7 @@
       <c r="P15" s="38">
         <f>SUM(P4:P14)</f>
       </c>
-      <c r="Q15" s="40">
+      <c r="Q15" s="41">
         <f>P15-O15</f>
       </c>
       <c r="R15" s="41">

</xml_diff>

<commit_message>
fix(sorvete): publica xlsx com historico 01-14 fixo + 15/10 corrigido (MINAS BAHIA=10)
Confirma publicacao dos valores validados:
- Historico 01-14/10 intacto conforme imagem fonte de verdade
  (12/10=135, 13/10=130, 14/10=125).
- Dia 15/10 hardcodado conforme planilha Christian (TOTAL=123,
  MINAS BAHIA=10 -- excluindo WO0037606 que nao consta na planilha).
Regenerado relatorio_sorvete.xlsx (15 dias, ultimo 15/10).
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -669,7 +669,7 @@
         <v>8</v>
       </c>
       <c r="P8" s="37">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="34">
         <f>P8-O8</f>
@@ -1287,7 +1287,7 @@
         <v>0</v>
       </c>
       <c r="P18" s="37">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="36" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
         <v>0</v>
       </c>
       <c r="P20" s="37">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(sorvete): restaura linhas Fechados/Abertos/Saldo/Lojas paradas (01-12/10 + 14-15/10) As linhas de resumo da aba Evolucao estavam zeradas apos o hardcode dos dias historicos. Valores restaurados: - 01-12/10: extraidos dos commits git historicos (80eab03, 771e81d, 08e7f27) - 14/10: Fechados=33, Abertos=28, Saldo=-5, Lojas=7 (do log foto_diaria 23:59) - 15/10: Fechados=24, Abertos=23, Saldo=-1, Lojas=5 (do log foto_diaria 23:59) - 13/10: mantido 0 (tarefa falhou nesse dia, sem log exato de movimentacao diaria) Regenerado relatorio_sorvete.xlsx com as linhas preenchidas. Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -1183,49 +1183,49 @@
         </is>
       </c>
       <c r="B17" s="36">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C17" s="36">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="D17" s="36">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E17" s="36">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F17" s="36">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G17" s="36">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H17" s="36">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I17" s="36">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J17" s="36">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="K17" s="36">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="L17" s="36">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="M17" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N17" s="36">
         <v>0</v>
       </c>
       <c r="O17" s="36">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="P17" s="37">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q17" s="36" t="inlineStr">
         <is>
@@ -1245,49 +1245,49 @@
         </is>
       </c>
       <c r="B18" s="36">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C18" s="36">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="D18" s="36">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="E18" s="36">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F18" s="36">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="G18" s="36">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H18" s="36">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="I18" s="36">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J18" s="36">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="K18" s="36">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="L18" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M18" s="36">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N18" s="36">
         <v>0</v>
       </c>
       <c r="O18" s="36">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="P18" s="37">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="Q18" s="36" t="inlineStr">
         <is>
@@ -1369,49 +1369,49 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="C20" s="36">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D20" s="36">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E20" s="36">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F20" s="36">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G20" s="36">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H20" s="36">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I20" s="36">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J20" s="36">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K20" s="36">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L20" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M20" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N20" s="36">
         <v>0</v>
       </c>
       <c r="O20" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P20" s="37">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(sorvete): preenche resumo do dia 13/10 (fechados/abertos/saldo/lojas) O dia 13/10 estava com as linhas de resumo zeradas porque a tarefa automatica falhou nesse dia e nao havia log exato. Valores calculados a partir da foto reconstruida (soma_sorvete_2026-10-13.json) usando a janela 12/10 23:40 -> 13/10 23:49: - Fechados: 0 - Abertos: 29 - Saldo: 29 - Lojas 100% paradas: 7 Regenerado relatorio_sorvete.xlsx com todas as linhas de resumo (01-15/10) preenchidas. Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -1281,7 +1281,7 @@
         <v>5</v>
       </c>
       <c r="N18" s="36">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="O18" s="36">
         <v>28</v>
@@ -1405,7 +1405,7 @@
         <v>7</v>
       </c>
       <c r="N20" s="36">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O20" s="36">
         <v>7</v>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-17 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -1183,49 +1183,49 @@
         </is>
       </c>
       <c r="B17" s="36">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C17" s="36">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="D17" s="36">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E17" s="36">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F17" s="36">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G17" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H17" s="36">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="I17" s="36">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="J17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="K17" s="36">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="L17" s="36">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="M17" s="36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N17" s="36">
         <v>0</v>
       </c>
       <c r="O17" s="36">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="P17" s="37">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="36" t="inlineStr">
         <is>
@@ -1245,49 +1245,49 @@
         </is>
       </c>
       <c r="B18" s="36">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C18" s="36">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="D18" s="36">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E18" s="36">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F18" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="G18" s="36">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H18" s="36">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="I18" s="36">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="J18" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K18" s="36">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="L18" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M18" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N18" s="36">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="O18" s="36">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="P18" s="37">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="36" t="inlineStr">
         <is>
@@ -1369,49 +1369,49 @@
         </is>
       </c>
       <c r="B20" s="36">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C20" s="36">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="D20" s="36">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E20" s="36">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F20" s="36">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G20" s="36">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H20" s="36">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I20" s="36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J20" s="36">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K20" s="36">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L20" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M20" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N20" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O20" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P20" s="37">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sorvete: relatorio xlsx regerado ate 19/10
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -288,13 +288,14 @@
     <col min="17" max="17" width="10" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="12" customWidth="1"/>
+    <col min="20" max="20" width="10" customWidth="1"/>
+    <col min="21" max="21" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 18/10 · variação 17/10 → 18/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 19/10 · variação 18/10 → 19/10</t>
         </is>
       </c>
     </row>
@@ -397,10 +398,15 @@
       </c>
       <c r="T3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">19/10</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="U3" s="1" t="inlineStr">
+      <c r="V3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -463,148 +469,157 @@
       <c r="R4" s="36">
         <v>39</v>
       </c>
-      <c r="S4" s="37">
+      <c r="S4" s="36">
         <v>44</v>
       </c>
-      <c r="T4" s="34">
-        <f>S4-R4</f>
-      </c>
-      <c r="U4" s="35">
-        <f>S4-B4</f>
+      <c r="T4" s="37">
+        <v>48</v>
+      </c>
+      <c r="U4" s="34">
+        <f>T4-S4</f>
+      </c>
+      <c r="V4" s="35">
+        <f>T4-B4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B5" s="36">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="C5" s="36">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D5" s="36">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E5" s="36">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F5" s="36">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="G5" s="36">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="H5" s="36">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="I5" s="36">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="J5" s="36">
+        <v>22</v>
+      </c>
+      <c r="K5" s="36">
+        <v>16</v>
+      </c>
+      <c r="L5" s="36">
+        <v>12</v>
+      </c>
+      <c r="M5" s="36">
+        <v>12</v>
+      </c>
+      <c r="N5" s="36">
+        <v>17</v>
+      </c>
+      <c r="O5" s="36">
+        <v>16</v>
+      </c>
+      <c r="P5" s="36">
         <v>14</v>
       </c>
-      <c r="K5" s="36">
-        <v>12</v>
-      </c>
-      <c r="L5" s="36">
-        <v>10</v>
-      </c>
-      <c r="M5" s="36">
-        <v>10</v>
-      </c>
-      <c r="N5" s="36">
-        <v>13</v>
-      </c>
-      <c r="O5" s="36">
-        <v>12</v>
-      </c>
-      <c r="P5" s="36">
+      <c r="Q5" s="36">
+        <v>16</v>
+      </c>
+      <c r="R5" s="36">
         <v>15</v>
       </c>
-      <c r="Q5" s="36">
-        <v>11</v>
-      </c>
-      <c r="R5" s="36">
-        <v>13</v>
-      </c>
-      <c r="S5" s="37">
-        <v>17</v>
-      </c>
-      <c r="T5" s="34">
-        <f>S5-R5</f>
+      <c r="S5" s="36">
+        <v>15</v>
+      </c>
+      <c r="T5" s="37">
+        <v>14</v>
       </c>
       <c r="U5" s="35">
-        <f>S5-B5</f>
+        <f>T5-S5</f>
+      </c>
+      <c r="V5" s="35">
+        <f>T5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C6" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D6" s="36">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="E6" s="36">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="F6" s="36">
+        <v>42</v>
+      </c>
+      <c r="G6" s="36">
+        <v>45</v>
+      </c>
+      <c r="H6" s="36">
+        <v>41</v>
+      </c>
+      <c r="I6" s="36">
+        <v>39</v>
+      </c>
+      <c r="J6" s="36">
+        <v>14</v>
+      </c>
+      <c r="K6" s="36">
+        <v>12</v>
+      </c>
+      <c r="L6" s="36">
+        <v>10</v>
+      </c>
+      <c r="M6" s="36">
+        <v>10</v>
+      </c>
+      <c r="N6" s="36">
+        <v>13</v>
+      </c>
+      <c r="O6" s="36">
+        <v>12</v>
+      </c>
+      <c r="P6" s="36">
+        <v>15</v>
+      </c>
+      <c r="Q6" s="36">
+        <v>11</v>
+      </c>
+      <c r="R6" s="36">
+        <v>13</v>
+      </c>
+      <c r="S6" s="36">
         <v>17</v>
       </c>
-      <c r="G6" s="36">
-        <v>17</v>
-      </c>
-      <c r="H6" s="36">
-        <v>18</v>
-      </c>
-      <c r="I6" s="36">
-        <v>18</v>
-      </c>
-      <c r="J6" s="36">
-        <v>22</v>
-      </c>
-      <c r="K6" s="36">
-        <v>16</v>
-      </c>
-      <c r="L6" s="36">
-        <v>12</v>
-      </c>
-      <c r="M6" s="36">
-        <v>12</v>
-      </c>
-      <c r="N6" s="36">
-        <v>17</v>
-      </c>
-      <c r="O6" s="36">
-        <v>16</v>
-      </c>
-      <c r="P6" s="36">
+      <c r="T6" s="37">
         <v>14</v>
       </c>
-      <c r="Q6" s="36">
-        <v>16</v>
-      </c>
-      <c r="R6" s="36">
-        <v>15</v>
-      </c>
-      <c r="S6" s="37">
-        <v>15</v>
-      </c>
-      <c r="T6" s="36">
-        <f>S6-R6</f>
-      </c>
       <c r="U6" s="35">
-        <f>S6-B6</f>
+        <f>T6-S6</f>
+      </c>
+      <c r="V6" s="35">
+        <f>T6-B6</f>
       </c>
     </row>
     <row r="7">
@@ -664,97 +679,103 @@
       <c r="R7" s="36">
         <v>13</v>
       </c>
-      <c r="S7" s="37">
+      <c r="S7" s="36">
         <v>10</v>
       </c>
-      <c r="T7" s="35">
-        <f>S7-R7</f>
-      </c>
-      <c r="U7" s="34">
-        <f>S7-B7</f>
+      <c r="T7" s="37">
+        <v>10</v>
+      </c>
+      <c r="U7" s="36">
+        <f>T7-S7</f>
+      </c>
+      <c r="V7" s="34">
+        <f>T7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C8" s="36">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D8" s="36">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E8" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F8" s="36">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="G8" s="36">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H8" s="36">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I8" s="36">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J8" s="36">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="K8" s="36">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="L8" s="36">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="M8" s="36">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="N8" s="36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O8" s="36">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P8" s="36">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q8" s="36">
         <v>6</v>
       </c>
       <c r="R8" s="36">
+        <v>6</v>
+      </c>
+      <c r="S8" s="36">
         <v>5</v>
       </c>
-      <c r="S8" s="37">
-        <v>7</v>
-      </c>
-      <c r="T8" s="34">
-        <f>S8-R8</f>
-      </c>
-      <c r="U8" s="35">
-        <f>S8-B8</f>
+      <c r="T8" s="37">
+        <v>8</v>
+      </c>
+      <c r="U8" s="34">
+        <f>T8-S8</f>
+      </c>
+      <c r="V8" s="35">
+        <f>T8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C9" s="36">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D9" s="36">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" s="36">
         <v>22</v>
@@ -763,250 +784,262 @@
         <v>23</v>
       </c>
       <c r="G9" s="36">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H9" s="36">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I9" s="36">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="J9" s="36">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="K9" s="36">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="L9" s="36">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="M9" s="36">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="N9" s="36">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O9" s="36">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P9" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q9" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R9" s="36">
         <v>5</v>
       </c>
-      <c r="S9" s="37">
-        <v>6</v>
-      </c>
-      <c r="T9" s="34">
-        <f>S9-R9</f>
-      </c>
-      <c r="U9" s="35">
-        <f>S9-B9</f>
+      <c r="S9" s="36">
+        <v>7</v>
+      </c>
+      <c r="T9" s="37">
+        <v>8</v>
+      </c>
+      <c r="U9" s="34">
+        <f>T9-S9</f>
+      </c>
+      <c r="V9" s="35">
+        <f>T9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B10" s="36">
+        <v>35</v>
+      </c>
+      <c r="C10" s="36">
+        <v>33</v>
+      </c>
+      <c r="D10" s="36">
+        <v>33</v>
+      </c>
+      <c r="E10" s="36">
+        <v>35</v>
+      </c>
+      <c r="F10" s="36">
+        <v>39</v>
+      </c>
+      <c r="G10" s="36">
+        <v>32</v>
+      </c>
+      <c r="H10" s="36">
+        <v>27</v>
+      </c>
+      <c r="I10" s="36">
+        <v>25</v>
+      </c>
+      <c r="J10" s="36">
+        <v>20</v>
+      </c>
+      <c r="K10" s="36">
+        <v>18</v>
+      </c>
+      <c r="L10" s="36">
+        <v>14</v>
+      </c>
+      <c r="M10" s="36">
+        <v>14</v>
+      </c>
+      <c r="N10" s="36">
         <v>11</v>
       </c>
-      <c r="C10" s="36">
+      <c r="O10" s="36">
         <v>10</v>
       </c>
-      <c r="D10" s="36">
-        <v>9</v>
-      </c>
-      <c r="E10" s="36">
+      <c r="P10" s="36">
+        <v>10</v>
+      </c>
+      <c r="Q10" s="36">
+        <v>8</v>
+      </c>
+      <c r="R10" s="36">
         <v>6</v>
       </c>
-      <c r="F10" s="36">
-        <v>5</v>
-      </c>
-      <c r="G10" s="36">
-        <v>5</v>
-      </c>
-      <c r="H10" s="36">
-        <v>5</v>
-      </c>
-      <c r="I10" s="36">
-        <v>6</v>
-      </c>
-      <c r="J10" s="36">
-        <v>5</v>
-      </c>
-      <c r="K10" s="36">
+      <c r="S10" s="36">
         <v>4</v>
       </c>
-      <c r="L10" s="36">
-        <v>4</v>
-      </c>
-      <c r="M10" s="36">
-        <v>5</v>
-      </c>
-      <c r="N10" s="36">
-        <v>8</v>
-      </c>
-      <c r="O10" s="36">
-        <v>6</v>
-      </c>
-      <c r="P10" s="36">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="36">
-        <v>5</v>
-      </c>
-      <c r="R10" s="36">
-        <v>5</v>
-      </c>
-      <c r="S10" s="37">
-        <v>6</v>
-      </c>
-      <c r="T10" s="34">
-        <f>S10-R10</f>
-      </c>
-      <c r="U10" s="35">
-        <f>S10-B10</f>
+      <c r="T10" s="37">
+        <v>7</v>
+      </c>
+      <c r="U10" s="34">
+        <f>T10-S10</f>
+      </c>
+      <c r="V10" s="35">
+        <f>T10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C11" s="36">
+        <v>22</v>
+      </c>
+      <c r="D11" s="36">
+        <v>22</v>
+      </c>
+      <c r="E11" s="36">
+        <v>22</v>
+      </c>
+      <c r="F11" s="36">
+        <v>23</v>
+      </c>
+      <c r="G11" s="36">
+        <v>25</v>
+      </c>
+      <c r="H11" s="36">
+        <v>24</v>
+      </c>
+      <c r="I11" s="36">
+        <v>28</v>
+      </c>
+      <c r="J11" s="36">
+        <v>30</v>
+      </c>
+      <c r="K11" s="36">
+        <v>31</v>
+      </c>
+      <c r="L11" s="36">
+        <v>26</v>
+      </c>
+      <c r="M11" s="36">
+        <v>24</v>
+      </c>
+      <c r="N11" s="36">
         <v>11</v>
       </c>
-      <c r="D11" s="36">
+      <c r="O11" s="36">
+        <v>8</v>
+      </c>
+      <c r="P11" s="36">
         <v>10</v>
       </c>
-      <c r="E11" s="36">
-        <v>10</v>
-      </c>
-      <c r="F11" s="36">
-        <v>12</v>
-      </c>
-      <c r="G11" s="36">
-        <v>11</v>
-      </c>
-      <c r="H11" s="36">
-        <v>12</v>
-      </c>
-      <c r="I11" s="36">
+      <c r="Q11" s="36">
         <v>7</v>
       </c>
-      <c r="J11" s="36">
+      <c r="R11" s="36">
+        <v>5</v>
+      </c>
+      <c r="S11" s="36">
         <v>6</v>
       </c>
-      <c r="K11" s="36">
-        <v>7</v>
-      </c>
-      <c r="L11" s="36">
-        <v>7</v>
-      </c>
-      <c r="M11" s="36">
-        <v>7</v>
-      </c>
-      <c r="N11" s="36">
-        <v>10</v>
-      </c>
-      <c r="O11" s="36">
-        <v>7</v>
-      </c>
-      <c r="P11" s="36">
-        <v>8</v>
-      </c>
-      <c r="Q11" s="36">
+      <c r="T11" s="37">
         <v>6</v>
       </c>
-      <c r="R11" s="36">
-        <v>6</v>
-      </c>
-      <c r="S11" s="37">
-        <v>5</v>
-      </c>
-      <c r="T11" s="35">
-        <f>S11-R11</f>
-      </c>
-      <c r="U11" s="35">
-        <f>S11-B11</f>
+      <c r="U11" s="36">
+        <f>T11-S11</f>
+      </c>
+      <c r="V11" s="35">
+        <f>T11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C12" s="36">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D12" s="36">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E12" s="36">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F12" s="36">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="G12" s="36">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H12" s="36">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="I12" s="36">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="J12" s="36">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="K12" s="36">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="L12" s="36">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M12" s="36">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="N12" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O12" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="P12" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="R12" s="36">
+        <v>5</v>
+      </c>
+      <c r="S12" s="36">
         <v>6</v>
       </c>
-      <c r="S12" s="37">
-        <v>4</v>
-      </c>
-      <c r="T12" s="35">
-        <f>S12-R12</f>
+      <c r="T12" s="37">
+        <v>5</v>
       </c>
       <c r="U12" s="35">
-        <f>S12-B12</f>
+        <f>T12-S12</f>
+      </c>
+      <c r="V12" s="35">
+        <f>T12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -1066,14 +1099,17 @@
       <c r="R13" s="36">
         <v>2</v>
       </c>
-      <c r="S13" s="37">
+      <c r="S13" s="36">
         <v>3</v>
       </c>
-      <c r="T13" s="34">
-        <f>S13-R13</f>
+      <c r="T13" s="37">
+        <v>2</v>
       </c>
       <c r="U13" s="35">
-        <f>S13-B13</f>
+        <f>T13-S13</f>
+      </c>
+      <c r="V13" s="35">
+        <f>T13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -1133,14 +1169,17 @@
       <c r="R14" s="36">
         <v>1</v>
       </c>
-      <c r="S14" s="37">
+      <c r="S14" s="36">
         <v>1</v>
       </c>
-      <c r="T14" s="36">
-        <f>S14-R14</f>
-      </c>
-      <c r="U14" s="35">
-        <f>S14-B14</f>
+      <c r="T14" s="37">
+        <v>1</v>
+      </c>
+      <c r="U14" s="36">
+        <f>T14-S14</f>
+      </c>
+      <c r="V14" s="35">
+        <f>T14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1203,11 +1242,14 @@
       <c r="S15" s="38">
         <f>SUM(S4:S14)</f>
       </c>
-      <c r="T15" s="40">
-        <f>S15-R15</f>
-      </c>
-      <c r="U15" s="41">
-        <f>S15-B15</f>
+      <c r="T15" s="38">
+        <f>SUM(T4:T14)</f>
+      </c>
+      <c r="U15" s="40">
+        <f>T15-S15</f>
+      </c>
+      <c r="V15" s="41">
+        <f>T15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1316,6 +1358,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="V16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1374,15 +1421,18 @@
       <c r="R17" s="36">
         <v>25</v>
       </c>
-      <c r="S17" s="37">
+      <c r="S17" s="36">
         <v>14</v>
       </c>
-      <c r="T17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="T17" s="37">
+        <v>29</v>
       </c>
       <c r="U17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="V17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1445,15 +1495,18 @@
       <c r="R18" s="36">
         <v>26</v>
       </c>
-      <c r="S18" s="37">
+      <c r="S18" s="36">
         <v>22</v>
       </c>
-      <c r="T18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="T18" s="37">
+        <v>34</v>
       </c>
       <c r="U18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="V18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1516,15 +1569,18 @@
       <c r="R19" s="36">
         <f>R18-R17</f>
       </c>
-      <c r="S19" s="37">
+      <c r="S19" s="36">
         <f>S18-S17</f>
       </c>
-      <c r="T19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="T19" s="37">
+        <f>T18-T17</f>
       </c>
       <c r="U19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="V19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1587,15 +1643,18 @@
       <c r="R20" s="36">
         <v>6</v>
       </c>
-      <c r="S20" s="37">
+      <c r="S20" s="36">
         <v>6</v>
       </c>
-      <c r="T20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="T20" s="37">
+        <v>9</v>
       </c>
       <c r="U20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="V20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-20 (foto da noite falhou, recorte reconstruido de 21/10)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -289,13 +289,14 @@
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="10" customWidth="1"/>
     <col min="20" max="20" width="10" customWidth="1"/>
-    <col min="21" max="21" width="12" customWidth="1"/>
+    <col min="21" max="21" width="10" customWidth="1"/>
+    <col min="22" max="22" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 19/10 · variação 18/10 → 19/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 20/10 · variação 19/10 → 20/10</t>
         </is>
       </c>
     </row>
@@ -403,10 +404,15 @@
       </c>
       <c r="U3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">20/10</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="V3" s="1" t="inlineStr">
+      <c r="W3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -472,504 +478,528 @@
       <c r="S4" s="36">
         <v>44</v>
       </c>
-      <c r="T4" s="37">
+      <c r="T4" s="36">
         <v>48</v>
       </c>
-      <c r="U4" s="34">
-        <f>T4-S4</f>
+      <c r="U4" s="37">
+        <v>36</v>
       </c>
       <c r="V4" s="35">
-        <f>T4-B4</f>
+        <f>U4-T4</f>
+      </c>
+      <c r="W4" s="35">
+        <f>U4-B4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B5" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C5" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D5" s="36">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="E5" s="36">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="F5" s="36">
+        <v>42</v>
+      </c>
+      <c r="G5" s="36">
+        <v>45</v>
+      </c>
+      <c r="H5" s="36">
+        <v>41</v>
+      </c>
+      <c r="I5" s="36">
+        <v>39</v>
+      </c>
+      <c r="J5" s="36">
+        <v>14</v>
+      </c>
+      <c r="K5" s="36">
+        <v>12</v>
+      </c>
+      <c r="L5" s="36">
+        <v>10</v>
+      </c>
+      <c r="M5" s="36">
+        <v>10</v>
+      </c>
+      <c r="N5" s="36">
+        <v>13</v>
+      </c>
+      <c r="O5" s="36">
+        <v>12</v>
+      </c>
+      <c r="P5" s="36">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="36">
+        <v>11</v>
+      </c>
+      <c r="R5" s="36">
+        <v>13</v>
+      </c>
+      <c r="S5" s="36">
         <v>17</v>
       </c>
-      <c r="G5" s="36">
-        <v>17</v>
-      </c>
-      <c r="H5" s="36">
-        <v>18</v>
-      </c>
-      <c r="I5" s="36">
-        <v>18</v>
-      </c>
-      <c r="J5" s="36">
-        <v>22</v>
-      </c>
-      <c r="K5" s="36">
-        <v>16</v>
-      </c>
-      <c r="L5" s="36">
-        <v>12</v>
-      </c>
-      <c r="M5" s="36">
-        <v>12</v>
-      </c>
-      <c r="N5" s="36">
-        <v>17</v>
-      </c>
-      <c r="O5" s="36">
-        <v>16</v>
-      </c>
-      <c r="P5" s="36">
+      <c r="T5" s="36">
         <v>14</v>
       </c>
-      <c r="Q5" s="36">
-        <v>16</v>
-      </c>
-      <c r="R5" s="36">
-        <v>15</v>
-      </c>
-      <c r="S5" s="36">
-        <v>15</v>
-      </c>
-      <c r="T5" s="37">
+      <c r="U5" s="37">
         <v>14</v>
       </c>
-      <c r="U5" s="35">
-        <f>T5-S5</f>
-      </c>
-      <c r="V5" s="35">
-        <f>T5-B5</f>
+      <c r="V5" s="36">
+        <f>U5-T5</f>
+      </c>
+      <c r="W5" s="35">
+        <f>U5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C6" s="36">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D6" s="36">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E6" s="36">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="F6" s="36">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="G6" s="36">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="H6" s="36">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="I6" s="36">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="J6" s="36">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K6" s="36">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="L6" s="36">
+        <v>7</v>
+      </c>
+      <c r="M6" s="36">
+        <v>7</v>
+      </c>
+      <c r="N6" s="36">
         <v>10</v>
       </c>
-      <c r="M6" s="36">
-        <v>10</v>
-      </c>
-      <c r="N6" s="36">
-        <v>13</v>
-      </c>
       <c r="O6" s="36">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="P6" s="36">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Q6" s="36">
+        <v>6</v>
+      </c>
+      <c r="R6" s="36">
+        <v>6</v>
+      </c>
+      <c r="S6" s="36">
+        <v>5</v>
+      </c>
+      <c r="T6" s="36">
+        <v>8</v>
+      </c>
+      <c r="U6" s="37">
         <v>11</v>
       </c>
-      <c r="R6" s="36">
-        <v>13</v>
-      </c>
-      <c r="S6" s="36">
-        <v>17</v>
-      </c>
-      <c r="T6" s="37">
-        <v>14</v>
-      </c>
-      <c r="U6" s="35">
-        <f>T6-S6</f>
-      </c>
-      <c r="V6" s="35">
-        <f>T6-B6</f>
+      <c r="V6" s="34">
+        <f>U6-T6</f>
+      </c>
+      <c r="W6" s="35">
+        <f>U6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C7" s="36">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="D7" s="36">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E7" s="36">
+        <v>20</v>
+      </c>
+      <c r="F7" s="36">
+        <v>17</v>
+      </c>
+      <c r="G7" s="36">
+        <v>17</v>
+      </c>
+      <c r="H7" s="36">
+        <v>18</v>
+      </c>
+      <c r="I7" s="36">
+        <v>18</v>
+      </c>
+      <c r="J7" s="36">
+        <v>22</v>
+      </c>
+      <c r="K7" s="36">
+        <v>16</v>
+      </c>
+      <c r="L7" s="36">
         <v>12</v>
       </c>
-      <c r="F7" s="36">
-        <v>13</v>
-      </c>
-      <c r="G7" s="36">
-        <v>9</v>
-      </c>
-      <c r="H7" s="36">
-        <v>11</v>
-      </c>
-      <c r="I7" s="36">
-        <v>7</v>
-      </c>
-      <c r="J7" s="36">
-        <v>6</v>
-      </c>
-      <c r="K7" s="36">
-        <v>6</v>
-      </c>
-      <c r="L7" s="36">
-        <v>7</v>
-      </c>
       <c r="M7" s="36">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="N7" s="36">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="O7" s="36">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="P7" s="36">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q7" s="36">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="R7" s="36">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="S7" s="36">
-        <v>10</v>
-      </c>
-      <c r="T7" s="37">
-        <v>10</v>
-      </c>
-      <c r="U7" s="36">
-        <f>T7-S7</f>
-      </c>
-      <c r="V7" s="34">
-        <f>T7-B7</f>
+        <v>15</v>
+      </c>
+      <c r="T7" s="36">
+        <v>14</v>
+      </c>
+      <c r="U7" s="37">
+        <v>8</v>
+      </c>
+      <c r="V7" s="35">
+        <f>U7-T7</f>
+      </c>
+      <c r="W7" s="35">
+        <f>U7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C8" s="36">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D8" s="36">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E8" s="36">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F8" s="36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G8" s="36">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H8" s="36">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="I8" s="36">
+        <v>18</v>
+      </c>
+      <c r="J8" s="36">
+        <v>19</v>
+      </c>
+      <c r="K8" s="36">
+        <v>17</v>
+      </c>
+      <c r="L8" s="36">
+        <v>13</v>
+      </c>
+      <c r="M8" s="36">
+        <v>14</v>
+      </c>
+      <c r="N8" s="36">
+        <v>9</v>
+      </c>
+      <c r="O8" s="36">
+        <v>9</v>
+      </c>
+      <c r="P8" s="36">
         <v>7</v>
-      </c>
-      <c r="J8" s="36">
-        <v>6</v>
-      </c>
-      <c r="K8" s="36">
-        <v>7</v>
-      </c>
-      <c r="L8" s="36">
-        <v>7</v>
-      </c>
-      <c r="M8" s="36">
-        <v>7</v>
-      </c>
-      <c r="N8" s="36">
-        <v>10</v>
-      </c>
-      <c r="O8" s="36">
-        <v>7</v>
-      </c>
-      <c r="P8" s="36">
-        <v>8</v>
       </c>
       <c r="Q8" s="36">
         <v>6</v>
       </c>
       <c r="R8" s="36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" s="36">
-        <v>5</v>
-      </c>
-      <c r="T8" s="37">
+        <v>7</v>
+      </c>
+      <c r="T8" s="36">
         <v>8</v>
       </c>
-      <c r="U8" s="34">
-        <f>T8-S8</f>
-      </c>
-      <c r="V8" s="35">
-        <f>T8-B8</f>
+      <c r="U8" s="37">
+        <v>8</v>
+      </c>
+      <c r="V8" s="36">
+        <f>U8-T8</f>
+      </c>
+      <c r="W8" s="35">
+        <f>U8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C9" s="36">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D9" s="36">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E9" s="36">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F9" s="36">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G9" s="36">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="H9" s="36">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="I9" s="36">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J9" s="36">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="K9" s="36">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="L9" s="36">
+        <v>7</v>
+      </c>
+      <c r="M9" s="36">
+        <v>7</v>
+      </c>
+      <c r="N9" s="36">
         <v>13</v>
       </c>
-      <c r="M9" s="36">
-        <v>14</v>
-      </c>
-      <c r="N9" s="36">
-        <v>9</v>
-      </c>
       <c r="O9" s="36">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="P9" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q9" s="36">
+        <v>10</v>
+      </c>
+      <c r="R9" s="36">
+        <v>13</v>
+      </c>
+      <c r="S9" s="36">
+        <v>10</v>
+      </c>
+      <c r="T9" s="36">
+        <v>10</v>
+      </c>
+      <c r="U9" s="37">
         <v>7</v>
       </c>
-      <c r="Q9" s="36">
-        <v>6</v>
-      </c>
-      <c r="R9" s="36">
-        <v>5</v>
-      </c>
-      <c r="S9" s="36">
-        <v>7</v>
-      </c>
-      <c r="T9" s="37">
-        <v>8</v>
-      </c>
-      <c r="U9" s="34">
-        <f>T9-S9</f>
-      </c>
       <c r="V9" s="35">
-        <f>T9-B9</f>
+        <f>U9-T9</f>
+      </c>
+      <c r="W9" s="35">
+        <f>U9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C10" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D10" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="E10" s="36">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F10" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G10" s="36">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H10" s="36">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I10" s="36">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J10" s="36">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K10" s="36">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="L10" s="36">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="M10" s="36">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N10" s="36">
         <v>11</v>
       </c>
       <c r="O10" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P10" s="36">
         <v>10</v>
       </c>
       <c r="Q10" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R10" s="36">
+        <v>5</v>
+      </c>
+      <c r="S10" s="36">
         <v>6</v>
       </c>
-      <c r="S10" s="36">
-        <v>4</v>
-      </c>
-      <c r="T10" s="37">
-        <v>7</v>
-      </c>
-      <c r="U10" s="34">
-        <f>T10-S10</f>
-      </c>
-      <c r="V10" s="35">
-        <f>T10-B10</f>
+      <c r="T10" s="36">
+        <v>6</v>
+      </c>
+      <c r="U10" s="37">
+        <v>6</v>
+      </c>
+      <c r="V10" s="36">
+        <f>U10-T10</f>
+      </c>
+      <c r="W10" s="35">
+        <f>U10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C11" s="36">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D11" s="36">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E11" s="36">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="F11" s="36">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G11" s="36">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H11" s="36">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="I11" s="36">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="J11" s="36">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="K11" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="L11" s="36">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="M11" s="36">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="N11" s="36">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="O11" s="36">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="P11" s="36">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q11" s="36">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R11" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S11" s="36">
-        <v>6</v>
-      </c>
-      <c r="T11" s="37">
-        <v>6</v>
-      </c>
-      <c r="U11" s="36">
-        <f>T11-S11</f>
-      </c>
-      <c r="V11" s="35">
-        <f>T11-B11</f>
+        <v>3</v>
+      </c>
+      <c r="T11" s="36">
+        <v>2</v>
+      </c>
+      <c r="U11" s="37">
+        <v>4</v>
+      </c>
+      <c r="V11" s="34">
+        <f>U11-T11</f>
+      </c>
+      <c r="W11" s="36">
+        <f>U11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -1032,84 +1062,90 @@
       <c r="S12" s="36">
         <v>6</v>
       </c>
-      <c r="T12" s="37">
+      <c r="T12" s="36">
         <v>5</v>
       </c>
-      <c r="U12" s="35">
-        <f>T12-S12</f>
+      <c r="U12" s="37">
+        <v>3</v>
       </c>
       <c r="V12" s="35">
-        <f>T12-B12</f>
+        <f>U12-T12</f>
+      </c>
+      <c r="W12" s="35">
+        <f>U12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B13" s="36">
+        <v>35</v>
+      </c>
+      <c r="C13" s="36">
+        <v>33</v>
+      </c>
+      <c r="D13" s="36">
+        <v>33</v>
+      </c>
+      <c r="E13" s="36">
+        <v>35</v>
+      </c>
+      <c r="F13" s="36">
+        <v>39</v>
+      </c>
+      <c r="G13" s="36">
+        <v>32</v>
+      </c>
+      <c r="H13" s="36">
+        <v>27</v>
+      </c>
+      <c r="I13" s="36">
+        <v>25</v>
+      </c>
+      <c r="J13" s="36">
+        <v>20</v>
+      </c>
+      <c r="K13" s="36">
+        <v>18</v>
+      </c>
+      <c r="L13" s="36">
+        <v>14</v>
+      </c>
+      <c r="M13" s="36">
+        <v>14</v>
+      </c>
+      <c r="N13" s="36">
+        <v>11</v>
+      </c>
+      <c r="O13" s="36">
+        <v>10</v>
+      </c>
+      <c r="P13" s="36">
+        <v>10</v>
+      </c>
+      <c r="Q13" s="36">
+        <v>8</v>
+      </c>
+      <c r="R13" s="36">
+        <v>6</v>
+      </c>
+      <c r="S13" s="36">
         <v>4</v>
       </c>
-      <c r="C13" s="36">
-        <v>4</v>
-      </c>
-      <c r="D13" s="36">
-        <v>3</v>
-      </c>
-      <c r="E13" s="36">
-        <v>3</v>
-      </c>
-      <c r="F13" s="36">
+      <c r="T13" s="36">
+        <v>7</v>
+      </c>
+      <c r="U13" s="37">
         <v>2</v>
       </c>
-      <c r="G13" s="36">
-        <v>4</v>
-      </c>
-      <c r="H13" s="36">
-        <v>2</v>
-      </c>
-      <c r="I13" s="36">
-        <v>4</v>
-      </c>
-      <c r="J13" s="36">
-        <v>3</v>
-      </c>
-      <c r="K13" s="36">
-        <v>0</v>
-      </c>
-      <c r="L13" s="36">
-        <v>0</v>
-      </c>
-      <c r="M13" s="36">
-        <v>0</v>
-      </c>
-      <c r="N13" s="36">
-        <v>1</v>
-      </c>
-      <c r="O13" s="36">
-        <v>3</v>
-      </c>
-      <c r="P13" s="36">
-        <v>2</v>
-      </c>
-      <c r="Q13" s="36">
-        <v>2</v>
-      </c>
-      <c r="R13" s="36">
-        <v>2</v>
-      </c>
-      <c r="S13" s="36">
-        <v>3</v>
-      </c>
-      <c r="T13" s="37">
-        <v>2</v>
-      </c>
-      <c r="U13" s="35">
-        <f>T13-S13</f>
-      </c>
       <c r="V13" s="35">
-        <f>T13-B13</f>
+        <f>U13-T13</f>
+      </c>
+      <c r="W13" s="35">
+        <f>U13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -1172,14 +1208,17 @@
       <c r="S14" s="36">
         <v>1</v>
       </c>
-      <c r="T14" s="37">
+      <c r="T14" s="36">
         <v>1</v>
       </c>
-      <c r="U14" s="36">
-        <f>T14-S14</f>
-      </c>
-      <c r="V14" s="35">
-        <f>T14-B14</f>
+      <c r="U14" s="37">
+        <v>1</v>
+      </c>
+      <c r="V14" s="36">
+        <f>U14-T14</f>
+      </c>
+      <c r="W14" s="35">
+        <f>U14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1245,11 +1284,14 @@
       <c r="T15" s="38">
         <f>SUM(T4:T14)</f>
       </c>
-      <c r="U15" s="40">
-        <f>T15-S15</f>
+      <c r="U15" s="38">
+        <f>SUM(U4:U14)</f>
       </c>
       <c r="V15" s="41">
-        <f>T15-B15</f>
+        <f>U15-T15</f>
+      </c>
+      <c r="W15" s="41">
+        <f>U15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1363,6 +1405,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="W16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1424,15 +1471,18 @@
       <c r="S17" s="36">
         <v>14</v>
       </c>
-      <c r="T17" s="37">
+      <c r="T17" s="36">
         <v>29</v>
       </c>
-      <c r="U17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="U17" s="37">
+        <v>51</v>
       </c>
       <c r="V17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="W17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1498,15 +1548,18 @@
       <c r="S18" s="36">
         <v>22</v>
       </c>
-      <c r="T18" s="37">
+      <c r="T18" s="36">
         <v>34</v>
       </c>
-      <c r="U18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="U18" s="37">
+        <v>28</v>
       </c>
       <c r="V18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="W18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1572,15 +1625,18 @@
       <c r="S19" s="36">
         <f>S18-S17</f>
       </c>
-      <c r="T19" s="37">
+      <c r="T19" s="36">
         <f>T18-T17</f>
       </c>
-      <c r="U19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="U19" s="37">
+        <f>U18-U17</f>
       </c>
       <c r="V19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="W19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1646,15 +1702,18 @@
       <c r="S20" s="36">
         <v>6</v>
       </c>
-      <c r="T20" s="37">
+      <c r="T20" s="36">
         <v>9</v>
       </c>
-      <c r="U20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="U20" s="37">
+        <v>8</v>
       </c>
       <c r="V20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="W20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-21 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -290,13 +290,14 @@
     <col min="19" max="19" width="10" customWidth="1"/>
     <col min="20" max="20" width="10" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
-    <col min="22" max="22" width="12" customWidth="1"/>
+    <col min="22" max="22" width="10" customWidth="1"/>
+    <col min="23" max="23" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 20/10 · variação 19/10 → 20/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 21/10 · variação 20/10 → 21/10</t>
         </is>
       </c>
     </row>
@@ -409,10 +410,15 @@
       </c>
       <c r="V3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">21/10</t>
+        </is>
+      </c>
+      <c r="W3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="W3" s="1" t="inlineStr">
+      <c r="X3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -481,14 +487,17 @@
       <c r="T4" s="36">
         <v>48</v>
       </c>
-      <c r="U4" s="37">
+      <c r="U4" s="36">
         <v>36</v>
       </c>
-      <c r="V4" s="35">
-        <f>U4-T4</f>
+      <c r="V4" s="37">
+        <v>35</v>
       </c>
       <c r="W4" s="35">
-        <f>U4-B4</f>
+        <f>V4-U4</f>
+      </c>
+      <c r="X4" s="35">
+        <f>V4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -554,176 +563,185 @@
       <c r="T5" s="36">
         <v>14</v>
       </c>
-      <c r="U5" s="37">
+      <c r="U5" s="36">
         <v>14</v>
       </c>
-      <c r="V5" s="36">
-        <f>U5-T5</f>
+      <c r="V5" s="37">
+        <v>13</v>
       </c>
       <c r="W5" s="35">
-        <f>U5-B5</f>
+        <f>V5-U5</f>
+      </c>
+      <c r="X5" s="35">
+        <f>V5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B6" s="36">
+        <v>21</v>
+      </c>
+      <c r="C6" s="36">
+        <v>21</v>
+      </c>
+      <c r="D6" s="36">
+        <v>18</v>
+      </c>
+      <c r="E6" s="36">
+        <v>20</v>
+      </c>
+      <c r="F6" s="36">
+        <v>17</v>
+      </c>
+      <c r="G6" s="36">
+        <v>17</v>
+      </c>
+      <c r="H6" s="36">
+        <v>18</v>
+      </c>
+      <c r="I6" s="36">
+        <v>18</v>
+      </c>
+      <c r="J6" s="36">
+        <v>22</v>
+      </c>
+      <c r="K6" s="36">
+        <v>16</v>
+      </c>
+      <c r="L6" s="36">
         <v>12</v>
       </c>
-      <c r="C6" s="36">
+      <c r="M6" s="36">
+        <v>12</v>
+      </c>
+      <c r="N6" s="36">
+        <v>17</v>
+      </c>
+      <c r="O6" s="36">
+        <v>16</v>
+      </c>
+      <c r="P6" s="36">
+        <v>14</v>
+      </c>
+      <c r="Q6" s="36">
+        <v>16</v>
+      </c>
+      <c r="R6" s="36">
+        <v>15</v>
+      </c>
+      <c r="S6" s="36">
+        <v>15</v>
+      </c>
+      <c r="T6" s="36">
+        <v>14</v>
+      </c>
+      <c r="U6" s="36">
+        <v>8</v>
+      </c>
+      <c r="V6" s="37">
         <v>11</v>
       </c>
-      <c r="D6" s="36">
-        <v>10</v>
-      </c>
-      <c r="E6" s="36">
-        <v>10</v>
-      </c>
-      <c r="F6" s="36">
-        <v>12</v>
-      </c>
-      <c r="G6" s="36">
-        <v>11</v>
-      </c>
-      <c r="H6" s="36">
-        <v>12</v>
-      </c>
-      <c r="I6" s="36">
-        <v>7</v>
-      </c>
-      <c r="J6" s="36">
-        <v>6</v>
-      </c>
-      <c r="K6" s="36">
-        <v>7</v>
-      </c>
-      <c r="L6" s="36">
-        <v>7</v>
-      </c>
-      <c r="M6" s="36">
-        <v>7</v>
-      </c>
-      <c r="N6" s="36">
-        <v>10</v>
-      </c>
-      <c r="O6" s="36">
-        <v>7</v>
-      </c>
-      <c r="P6" s="36">
-        <v>8</v>
-      </c>
-      <c r="Q6" s="36">
-        <v>6</v>
-      </c>
-      <c r="R6" s="36">
-        <v>6</v>
-      </c>
-      <c r="S6" s="36">
-        <v>5</v>
-      </c>
-      <c r="T6" s="36">
-        <v>8</v>
-      </c>
-      <c r="U6" s="37">
-        <v>11</v>
-      </c>
-      <c r="V6" s="34">
-        <f>U6-T6</f>
-      </c>
-      <c r="W6" s="35">
-        <f>U6-B6</f>
+      <c r="W6" s="34">
+        <f>V6-U6</f>
+      </c>
+      <c r="X6" s="35">
+        <f>V6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C7" s="36">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D7" s="36">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E7" s="36">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F7" s="36">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G7" s="36">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="H7" s="36">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I7" s="36">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J7" s="36">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="K7" s="36">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="L7" s="36">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M7" s="36">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="N7" s="36">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="O7" s="36">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="P7" s="36">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="Q7" s="36">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="R7" s="36">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="S7" s="36">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="T7" s="36">
-        <v>14</v>
-      </c>
-      <c r="U7" s="37">
         <v>8</v>
       </c>
-      <c r="V7" s="35">
-        <f>U7-T7</f>
+      <c r="U7" s="36">
+        <v>11</v>
+      </c>
+      <c r="V7" s="37">
+        <v>8</v>
       </c>
       <c r="W7" s="35">
-        <f>U7-B7</f>
+        <f>V7-U7</f>
+      </c>
+      <c r="X7" s="35">
+        <f>V7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C8" s="36">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D8" s="36">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E8" s="36">
         <v>22</v>
@@ -732,55 +750,58 @@
         <v>23</v>
       </c>
       <c r="G8" s="36">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H8" s="36">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="I8" s="36">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="J8" s="36">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K8" s="36">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="L8" s="36">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="M8" s="36">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N8" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O8" s="36">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P8" s="36">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R8" s="36">
         <v>5</v>
       </c>
       <c r="S8" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T8" s="36">
-        <v>8</v>
-      </c>
-      <c r="U8" s="37">
-        <v>8</v>
-      </c>
-      <c r="V8" s="36">
-        <f>U8-T8</f>
-      </c>
-      <c r="W8" s="35">
-        <f>U8-B8</f>
+        <v>6</v>
+      </c>
+      <c r="U8" s="36">
+        <v>6</v>
+      </c>
+      <c r="V8" s="37">
+        <v>7</v>
+      </c>
+      <c r="W8" s="34">
+        <f>V8-U8</f>
+      </c>
+      <c r="X8" s="35">
+        <f>V8-B8</f>
       </c>
     </row>
     <row r="9">
@@ -846,160 +867,169 @@
       <c r="T9" s="36">
         <v>10</v>
       </c>
-      <c r="U9" s="37">
-        <v>7</v>
-      </c>
-      <c r="V9" s="35">
-        <f>U9-T9</f>
+      <c r="U9" s="36">
+        <v>7</v>
+      </c>
+      <c r="V9" s="37">
+        <v>6</v>
       </c>
       <c r="W9" s="35">
-        <f>U9-B9</f>
+        <f>V9-U9</f>
+      </c>
+      <c r="X9" s="35">
+        <f>V9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="C10" s="36">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E10" s="36">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="F10" s="36">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G10" s="36">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H10" s="36">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="I10" s="36">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="J10" s="36">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="K10" s="36">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="L10" s="36">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="M10" s="36">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="N10" s="36">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="O10" s="36">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="P10" s="36">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="36">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R10" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S10" s="36">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T10" s="36">
-        <v>6</v>
-      </c>
-      <c r="U10" s="37">
-        <v>6</v>
-      </c>
-      <c r="V10" s="36">
-        <f>U10-T10</f>
-      </c>
-      <c r="W10" s="35">
-        <f>U10-B10</f>
+        <v>2</v>
+      </c>
+      <c r="U10" s="36">
+        <v>4</v>
+      </c>
+      <c r="V10" s="37">
+        <v>4</v>
+      </c>
+      <c r="W10" s="36">
+        <f>V10-U10</f>
+      </c>
+      <c r="X10" s="36">
+        <f>V10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B11" s="36">
+        <v>8</v>
+      </c>
+      <c r="C11" s="36">
+        <v>7</v>
+      </c>
+      <c r="D11" s="36">
+        <v>9</v>
+      </c>
+      <c r="E11" s="36">
+        <v>14</v>
+      </c>
+      <c r="F11" s="36">
+        <v>7</v>
+      </c>
+      <c r="G11" s="36">
+        <v>6</v>
+      </c>
+      <c r="H11" s="36">
+        <v>8</v>
+      </c>
+      <c r="I11" s="36">
+        <v>11</v>
+      </c>
+      <c r="J11" s="36">
+        <v>11</v>
+      </c>
+      <c r="K11" s="36">
+        <v>12</v>
+      </c>
+      <c r="L11" s="36">
         <v>4</v>
       </c>
-      <c r="C11" s="36">
+      <c r="M11" s="36">
         <v>4</v>
       </c>
-      <c r="D11" s="36">
-        <v>3</v>
-      </c>
-      <c r="E11" s="36">
-        <v>3</v>
-      </c>
-      <c r="F11" s="36">
+      <c r="N11" s="36">
         <v>2</v>
-      </c>
-      <c r="G11" s="36">
-        <v>4</v>
-      </c>
-      <c r="H11" s="36">
-        <v>2</v>
-      </c>
-      <c r="I11" s="36">
-        <v>4</v>
-      </c>
-      <c r="J11" s="36">
-        <v>3</v>
-      </c>
-      <c r="K11" s="36">
-        <v>0</v>
-      </c>
-      <c r="L11" s="36">
-        <v>0</v>
-      </c>
-      <c r="M11" s="36">
-        <v>0</v>
-      </c>
-      <c r="N11" s="36">
-        <v>1</v>
       </c>
       <c r="O11" s="36">
         <v>3</v>
       </c>
       <c r="P11" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="36">
         <v>2</v>
       </c>
       <c r="R11" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S11" s="36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T11" s="36">
-        <v>2</v>
-      </c>
-      <c r="U11" s="37">
+        <v>1</v>
+      </c>
+      <c r="U11" s="36">
+        <v>1</v>
+      </c>
+      <c r="V11" s="37">
         <v>4</v>
       </c>
-      <c r="V11" s="34">
-        <f>U11-T11</f>
-      </c>
-      <c r="W11" s="36">
-        <f>U11-B11</f>
+      <c r="W11" s="34">
+        <f>V11-U11</f>
+      </c>
+      <c r="X11" s="35">
+        <f>V11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -1065,160 +1095,169 @@
       <c r="T12" s="36">
         <v>5</v>
       </c>
-      <c r="U12" s="37">
+      <c r="U12" s="36">
         <v>3</v>
       </c>
-      <c r="V12" s="35">
-        <f>U12-T12</f>
-      </c>
-      <c r="W12" s="35">
-        <f>U12-B12</f>
+      <c r="V12" s="37">
+        <v>3</v>
+      </c>
+      <c r="W12" s="36">
+        <f>V12-U12</f>
+      </c>
+      <c r="X12" s="35">
+        <f>V12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="C13" s="36">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D13" s="36">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E13" s="36">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F13" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G13" s="36">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="H13" s="36">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="I13" s="36">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J13" s="36">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K13" s="36">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L13" s="36">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M13" s="36">
         <v>14</v>
       </c>
       <c r="N13" s="36">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O13" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P13" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q13" s="36">
+        <v>6</v>
+      </c>
+      <c r="R13" s="36">
+        <v>5</v>
+      </c>
+      <c r="S13" s="36">
+        <v>7</v>
+      </c>
+      <c r="T13" s="36">
         <v>8</v>
       </c>
-      <c r="R13" s="36">
-        <v>6</v>
-      </c>
-      <c r="S13" s="36">
-        <v>4</v>
-      </c>
-      <c r="T13" s="36">
-        <v>7</v>
-      </c>
-      <c r="U13" s="37">
-        <v>2</v>
-      </c>
-      <c r="V13" s="35">
-        <f>U13-T13</f>
+      <c r="U13" s="36">
+        <v>8</v>
+      </c>
+      <c r="V13" s="37">
+        <v>3</v>
       </c>
       <c r="W13" s="35">
-        <f>U13-B13</f>
+        <f>V13-U13</f>
+      </c>
+      <c r="X13" s="35">
+        <f>V13-B13</f>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B14" s="36">
+        <v>35</v>
+      </c>
+      <c r="C14" s="36">
+        <v>33</v>
+      </c>
+      <c r="D14" s="36">
+        <v>33</v>
+      </c>
+      <c r="E14" s="36">
+        <v>35</v>
+      </c>
+      <c r="F14" s="36">
+        <v>39</v>
+      </c>
+      <c r="G14" s="36">
+        <v>32</v>
+      </c>
+      <c r="H14" s="36">
+        <v>27</v>
+      </c>
+      <c r="I14" s="36">
+        <v>25</v>
+      </c>
+      <c r="J14" s="36">
+        <v>20</v>
+      </c>
+      <c r="K14" s="36">
+        <v>18</v>
+      </c>
+      <c r="L14" s="36">
+        <v>14</v>
+      </c>
+      <c r="M14" s="36">
+        <v>14</v>
+      </c>
+      <c r="N14" s="36">
+        <v>11</v>
+      </c>
+      <c r="O14" s="36">
+        <v>10</v>
+      </c>
+      <c r="P14" s="36">
+        <v>10</v>
+      </c>
+      <c r="Q14" s="36">
         <v>8</v>
       </c>
-      <c r="C14" s="36">
-        <v>7</v>
-      </c>
-      <c r="D14" s="36">
-        <v>9</v>
-      </c>
-      <c r="E14" s="36">
-        <v>14</v>
-      </c>
-      <c r="F14" s="36">
-        <v>7</v>
-      </c>
-      <c r="G14" s="36">
+      <c r="R14" s="36">
         <v>6</v>
       </c>
-      <c r="H14" s="36">
-        <v>8</v>
-      </c>
-      <c r="I14" s="36">
-        <v>11</v>
-      </c>
-      <c r="J14" s="36">
-        <v>11</v>
-      </c>
-      <c r="K14" s="36">
-        <v>12</v>
-      </c>
-      <c r="L14" s="36">
+      <c r="S14" s="36">
         <v>4</v>
       </c>
-      <c r="M14" s="36">
-        <v>4</v>
-      </c>
-      <c r="N14" s="36">
+      <c r="T14" s="36">
+        <v>7</v>
+      </c>
+      <c r="U14" s="36">
         <v>2</v>
       </c>
-      <c r="O14" s="36">
+      <c r="V14" s="37">
         <v>3</v>
       </c>
-      <c r="P14" s="36">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="36">
-        <v>2</v>
-      </c>
-      <c r="R14" s="36">
-        <v>1</v>
-      </c>
-      <c r="S14" s="36">
-        <v>1</v>
-      </c>
-      <c r="T14" s="36">
-        <v>1</v>
-      </c>
-      <c r="U14" s="37">
-        <v>1</v>
-      </c>
-      <c r="V14" s="36">
-        <f>U14-T14</f>
-      </c>
-      <c r="W14" s="35">
-        <f>U14-B14</f>
+      <c r="W14" s="34">
+        <f>V14-U14</f>
+      </c>
+      <c r="X14" s="35">
+        <f>V14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1287,11 +1326,14 @@
       <c r="U15" s="38">
         <f>SUM(U4:U14)</f>
       </c>
-      <c r="V15" s="41">
-        <f>U15-T15</f>
+      <c r="V15" s="38">
+        <f>SUM(V4:V14)</f>
       </c>
       <c r="W15" s="41">
-        <f>U15-B15</f>
+        <f>V15-U15</f>
+      </c>
+      <c r="X15" s="41">
+        <f>V15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1410,6 +1452,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="X16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1474,15 +1521,18 @@
       <c r="T17" s="36">
         <v>29</v>
       </c>
-      <c r="U17" s="37">
+      <c r="U17" s="36">
         <v>51</v>
       </c>
-      <c r="V17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="V17" s="37">
+        <v>27</v>
       </c>
       <c r="W17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="X17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1551,15 +1601,18 @@
       <c r="T18" s="36">
         <v>34</v>
       </c>
-      <c r="U18" s="37">
+      <c r="U18" s="36">
         <v>28</v>
       </c>
-      <c r="V18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="V18" s="37">
+        <v>24</v>
       </c>
       <c r="W18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="X18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1628,15 +1681,18 @@
       <c r="T19" s="36">
         <f>T18-T17</f>
       </c>
-      <c r="U19" s="37">
+      <c r="U19" s="36">
         <f>U18-U17</f>
       </c>
-      <c r="V19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="V19" s="37">
+        <f>V18-V17</f>
       </c>
       <c r="W19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="X19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1705,15 +1761,18 @@
       <c r="T20" s="36">
         <v>9</v>
       </c>
-      <c r="U20" s="37">
+      <c r="U20" s="36">
         <v>8</v>
       </c>
-      <c r="V20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="V20" s="37">
+        <v>7</v>
       </c>
       <c r="W20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="X20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-22 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -291,13 +291,14 @@
     <col min="20" max="20" width="10" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="10" customWidth="1"/>
-    <col min="23" max="23" width="12" customWidth="1"/>
+    <col min="23" max="23" width="10" customWidth="1"/>
+    <col min="24" max="24" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 21/10 · variação 20/10 → 21/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 22/10 · variação 21/10 → 22/10</t>
         </is>
       </c>
     </row>
@@ -415,10 +416,15 @@
       </c>
       <c r="W3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">22/10</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="X3" s="1" t="inlineStr">
+      <c r="Y3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -490,346 +496,361 @@
       <c r="U4" s="36">
         <v>36</v>
       </c>
-      <c r="V4" s="37">
+      <c r="V4" s="36">
         <v>35</v>
       </c>
-      <c r="W4" s="35">
-        <f>V4-U4</f>
+      <c r="W4" s="37">
+        <v>31</v>
       </c>
       <c r="X4" s="35">
-        <f>V4-B4</f>
+        <f>W4-V4</f>
+      </c>
+      <c r="Y4" s="35">
+        <f>W4-B4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B5" s="36">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="C5" s="36">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D5" s="36">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E5" s="36">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F5" s="36">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="G5" s="36">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="H5" s="36">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="I5" s="36">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="J5" s="36">
+        <v>22</v>
+      </c>
+      <c r="K5" s="36">
+        <v>16</v>
+      </c>
+      <c r="L5" s="36">
+        <v>12</v>
+      </c>
+      <c r="M5" s="36">
+        <v>12</v>
+      </c>
+      <c r="N5" s="36">
+        <v>17</v>
+      </c>
+      <c r="O5" s="36">
+        <v>16</v>
+      </c>
+      <c r="P5" s="36">
         <v>14</v>
       </c>
-      <c r="K5" s="36">
-        <v>12</v>
-      </c>
-      <c r="L5" s="36">
-        <v>10</v>
-      </c>
-      <c r="M5" s="36">
-        <v>10</v>
-      </c>
-      <c r="N5" s="36">
-        <v>13</v>
-      </c>
-      <c r="O5" s="36">
-        <v>12</v>
-      </c>
-      <c r="P5" s="36">
+      <c r="Q5" s="36">
+        <v>16</v>
+      </c>
+      <c r="R5" s="36">
         <v>15</v>
       </c>
-      <c r="Q5" s="36">
-        <v>11</v>
-      </c>
-      <c r="R5" s="36">
-        <v>13</v>
-      </c>
       <c r="S5" s="36">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="T5" s="36">
         <v>14</v>
       </c>
       <c r="U5" s="36">
+        <v>8</v>
+      </c>
+      <c r="V5" s="36">
+        <v>11</v>
+      </c>
+      <c r="W5" s="37">
         <v>14</v>
       </c>
-      <c r="V5" s="37">
-        <v>13</v>
-      </c>
-      <c r="W5" s="35">
-        <f>V5-U5</f>
-      </c>
-      <c r="X5" s="35">
-        <f>V5-B5</f>
+      <c r="X5" s="34">
+        <f>W5-V5</f>
+      </c>
+      <c r="Y5" s="35">
+        <f>W5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C6" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D6" s="36">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="E6" s="36">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="F6" s="36">
+        <v>42</v>
+      </c>
+      <c r="G6" s="36">
+        <v>45</v>
+      </c>
+      <c r="H6" s="36">
+        <v>41</v>
+      </c>
+      <c r="I6" s="36">
+        <v>39</v>
+      </c>
+      <c r="J6" s="36">
+        <v>14</v>
+      </c>
+      <c r="K6" s="36">
+        <v>12</v>
+      </c>
+      <c r="L6" s="36">
+        <v>10</v>
+      </c>
+      <c r="M6" s="36">
+        <v>10</v>
+      </c>
+      <c r="N6" s="36">
+        <v>13</v>
+      </c>
+      <c r="O6" s="36">
+        <v>12</v>
+      </c>
+      <c r="P6" s="36">
+        <v>15</v>
+      </c>
+      <c r="Q6" s="36">
+        <v>11</v>
+      </c>
+      <c r="R6" s="36">
+        <v>13</v>
+      </c>
+      <c r="S6" s="36">
         <v>17</v>
-      </c>
-      <c r="G6" s="36">
-        <v>17</v>
-      </c>
-      <c r="H6" s="36">
-        <v>18</v>
-      </c>
-      <c r="I6" s="36">
-        <v>18</v>
-      </c>
-      <c r="J6" s="36">
-        <v>22</v>
-      </c>
-      <c r="K6" s="36">
-        <v>16</v>
-      </c>
-      <c r="L6" s="36">
-        <v>12</v>
-      </c>
-      <c r="M6" s="36">
-        <v>12</v>
-      </c>
-      <c r="N6" s="36">
-        <v>17</v>
-      </c>
-      <c r="O6" s="36">
-        <v>16</v>
-      </c>
-      <c r="P6" s="36">
-        <v>14</v>
-      </c>
-      <c r="Q6" s="36">
-        <v>16</v>
-      </c>
-      <c r="R6" s="36">
-        <v>15</v>
-      </c>
-      <c r="S6" s="36">
-        <v>15</v>
       </c>
       <c r="T6" s="36">
         <v>14</v>
       </c>
       <c r="U6" s="36">
-        <v>8</v>
-      </c>
-      <c r="V6" s="37">
-        <v>11</v>
-      </c>
-      <c r="W6" s="34">
-        <f>V6-U6</f>
-      </c>
-      <c r="X6" s="35">
-        <f>V6-B6</f>
+        <v>14</v>
+      </c>
+      <c r="V6" s="36">
+        <v>13</v>
+      </c>
+      <c r="W6" s="37">
+        <v>14</v>
+      </c>
+      <c r="X6" s="34">
+        <f>W6-V6</f>
+      </c>
+      <c r="Y6" s="35">
+        <f>W6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C7" s="36">
+        <v>33</v>
+      </c>
+      <c r="D7" s="36">
+        <v>33</v>
+      </c>
+      <c r="E7" s="36">
+        <v>35</v>
+      </c>
+      <c r="F7" s="36">
+        <v>39</v>
+      </c>
+      <c r="G7" s="36">
+        <v>32</v>
+      </c>
+      <c r="H7" s="36">
+        <v>27</v>
+      </c>
+      <c r="I7" s="36">
+        <v>25</v>
+      </c>
+      <c r="J7" s="36">
+        <v>20</v>
+      </c>
+      <c r="K7" s="36">
+        <v>18</v>
+      </c>
+      <c r="L7" s="36">
+        <v>14</v>
+      </c>
+      <c r="M7" s="36">
+        <v>14</v>
+      </c>
+      <c r="N7" s="36">
         <v>11</v>
       </c>
-      <c r="D7" s="36">
+      <c r="O7" s="36">
         <v>10</v>
       </c>
-      <c r="E7" s="36">
+      <c r="P7" s="36">
         <v>10</v>
       </c>
-      <c r="F7" s="36">
-        <v>12</v>
-      </c>
-      <c r="G7" s="36">
-        <v>11</v>
-      </c>
-      <c r="H7" s="36">
-        <v>12</v>
-      </c>
-      <c r="I7" s="36">
-        <v>7</v>
-      </c>
-      <c r="J7" s="36">
-        <v>6</v>
-      </c>
-      <c r="K7" s="36">
-        <v>7</v>
-      </c>
-      <c r="L7" s="36">
-        <v>7</v>
-      </c>
-      <c r="M7" s="36">
-        <v>7</v>
-      </c>
-      <c r="N7" s="36">
-        <v>10</v>
-      </c>
-      <c r="O7" s="36">
-        <v>7</v>
-      </c>
-      <c r="P7" s="36">
+      <c r="Q7" s="36">
         <v>8</v>
-      </c>
-      <c r="Q7" s="36">
-        <v>6</v>
       </c>
       <c r="R7" s="36">
         <v>6</v>
       </c>
       <c r="S7" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T7" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U7" s="36">
-        <v>11</v>
-      </c>
-      <c r="V7" s="37">
-        <v>8</v>
-      </c>
-      <c r="W7" s="35">
-        <f>V7-U7</f>
-      </c>
-      <c r="X7" s="35">
-        <f>V7-B7</f>
+        <v>2</v>
+      </c>
+      <c r="V7" s="36">
+        <v>3</v>
+      </c>
+      <c r="W7" s="37">
+        <v>6</v>
+      </c>
+      <c r="X7" s="34">
+        <f>W7-V7</f>
+      </c>
+      <c r="Y7" s="35">
+        <f>W7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C8" s="36">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="E8" s="36">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F8" s="36">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G8" s="36">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="H8" s="36">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="I8" s="36">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J8" s="36">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="K8" s="36">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="L8" s="36">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="M8" s="36">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="N8" s="36">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O8" s="36">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="P8" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="36">
         <v>10</v>
       </c>
-      <c r="Q8" s="36">
+      <c r="R8" s="36">
+        <v>13</v>
+      </c>
+      <c r="S8" s="36">
+        <v>10</v>
+      </c>
+      <c r="T8" s="36">
+        <v>10</v>
+      </c>
+      <c r="U8" s="36">
         <v>7</v>
       </c>
-      <c r="R8" s="36">
+      <c r="V8" s="36">
+        <v>6</v>
+      </c>
+      <c r="W8" s="37">
         <v>5</v>
       </c>
-      <c r="S8" s="36">
-        <v>6</v>
-      </c>
-      <c r="T8" s="36">
-        <v>6</v>
-      </c>
-      <c r="U8" s="36">
-        <v>6</v>
-      </c>
-      <c r="V8" s="37">
-        <v>7</v>
-      </c>
-      <c r="W8" s="34">
-        <f>V8-U8</f>
-      </c>
       <c r="X8" s="35">
-        <f>V8-B8</f>
+        <f>W8-V8</f>
+      </c>
+      <c r="Y8" s="35">
+        <f>W8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C9" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D9" s="36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="36">
+        <v>10</v>
+      </c>
+      <c r="F9" s="36">
         <v>12</v>
       </c>
-      <c r="F9" s="36">
-        <v>13</v>
-      </c>
       <c r="G9" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H9" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I9" s="36">
         <v>7</v>
@@ -838,7 +859,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L9" s="36">
         <v>7</v>
@@ -847,189 +868,198 @@
         <v>7</v>
       </c>
       <c r="N9" s="36">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O9" s="36">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="P9" s="36">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="Q9" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="R9" s="36">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="S9" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T9" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U9" s="36">
-        <v>7</v>
-      </c>
-      <c r="V9" s="37">
-        <v>6</v>
-      </c>
-      <c r="W9" s="35">
-        <f>V9-U9</f>
+        <v>11</v>
+      </c>
+      <c r="V9" s="36">
+        <v>8</v>
+      </c>
+      <c r="W9" s="37">
+        <v>4</v>
       </c>
       <c r="X9" s="35">
-        <f>V9-B9</f>
+        <f>W9-V9</f>
+      </c>
+      <c r="Y9" s="35">
+        <f>W9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B10" s="36">
+        <v>18</v>
+      </c>
+      <c r="C10" s="36">
+        <v>16</v>
+      </c>
+      <c r="D10" s="36">
+        <v>20</v>
+      </c>
+      <c r="E10" s="36">
+        <v>22</v>
+      </c>
+      <c r="F10" s="36">
+        <v>23</v>
+      </c>
+      <c r="G10" s="36">
+        <v>20</v>
+      </c>
+      <c r="H10" s="36">
+        <v>18</v>
+      </c>
+      <c r="I10" s="36">
+        <v>18</v>
+      </c>
+      <c r="J10" s="36">
+        <v>19</v>
+      </c>
+      <c r="K10" s="36">
+        <v>17</v>
+      </c>
+      <c r="L10" s="36">
+        <v>13</v>
+      </c>
+      <c r="M10" s="36">
+        <v>14</v>
+      </c>
+      <c r="N10" s="36">
+        <v>9</v>
+      </c>
+      <c r="O10" s="36">
+        <v>9</v>
+      </c>
+      <c r="P10" s="36">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="36">
+        <v>6</v>
+      </c>
+      <c r="R10" s="36">
+        <v>5</v>
+      </c>
+      <c r="S10" s="36">
+        <v>7</v>
+      </c>
+      <c r="T10" s="36">
+        <v>8</v>
+      </c>
+      <c r="U10" s="36">
+        <v>8</v>
+      </c>
+      <c r="V10" s="36">
+        <v>3</v>
+      </c>
+      <c r="W10" s="37">
         <v>4</v>
       </c>
-      <c r="C10" s="36">
-        <v>4</v>
-      </c>
-      <c r="D10" s="36">
-        <v>3</v>
-      </c>
-      <c r="E10" s="36">
-        <v>3</v>
-      </c>
-      <c r="F10" s="36">
-        <v>2</v>
-      </c>
-      <c r="G10" s="36">
-        <v>4</v>
-      </c>
-      <c r="H10" s="36">
-        <v>2</v>
-      </c>
-      <c r="I10" s="36">
-        <v>4</v>
-      </c>
-      <c r="J10" s="36">
-        <v>3</v>
-      </c>
-      <c r="K10" s="36">
-        <v>0</v>
-      </c>
-      <c r="L10" s="36">
-        <v>0</v>
-      </c>
-      <c r="M10" s="36">
-        <v>0</v>
-      </c>
-      <c r="N10" s="36">
-        <v>1</v>
-      </c>
-      <c r="O10" s="36">
-        <v>3</v>
-      </c>
-      <c r="P10" s="36">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="36">
-        <v>2</v>
-      </c>
-      <c r="R10" s="36">
-        <v>2</v>
-      </c>
-      <c r="S10" s="36">
-        <v>3</v>
-      </c>
-      <c r="T10" s="36">
-        <v>2</v>
-      </c>
-      <c r="U10" s="36">
-        <v>4</v>
-      </c>
-      <c r="V10" s="37">
-        <v>4</v>
-      </c>
-      <c r="W10" s="36">
-        <f>V10-U10</f>
-      </c>
-      <c r="X10" s="36">
-        <f>V10-B10</f>
+      <c r="X10" s="34">
+        <f>W10-V10</f>
+      </c>
+      <c r="Y10" s="35">
+        <f>W10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C11" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D11" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E11" s="36">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F11" s="36">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G11" s="36">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H11" s="36">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I11" s="36">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J11" s="36">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K11" s="36">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L11" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M11" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N11" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O11" s="36">
         <v>3</v>
       </c>
       <c r="P11" s="36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q11" s="36">
         <v>2</v>
       </c>
       <c r="R11" s="36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" s="36">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T11" s="36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U11" s="36">
-        <v>1</v>
-      </c>
-      <c r="V11" s="37">
         <v>4</v>
       </c>
-      <c r="W11" s="34">
-        <f>V11-U11</f>
+      <c r="V11" s="36">
+        <v>4</v>
+      </c>
+      <c r="W11" s="37">
+        <v>3</v>
       </c>
       <c r="X11" s="35">
-        <f>V11-B11</f>
+        <f>W11-V11</f>
+      </c>
+      <c r="Y11" s="35">
+        <f>W11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -1098,166 +1128,175 @@
       <c r="U12" s="36">
         <v>3</v>
       </c>
-      <c r="V12" s="37">
+      <c r="V12" s="36">
         <v>3</v>
       </c>
-      <c r="W12" s="36">
-        <f>V12-U12</f>
-      </c>
-      <c r="X12" s="35">
-        <f>V12-B12</f>
+      <c r="W12" s="37">
+        <v>3</v>
+      </c>
+      <c r="X12" s="36">
+        <f>W12-V12</f>
+      </c>
+      <c r="Y12" s="35">
+        <f>W12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C13" s="36">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D13" s="36">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E13" s="36">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F13" s="36">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="G13" s="36">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H13" s="36">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="I13" s="36">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="J13" s="36">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="K13" s="36">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="L13" s="36">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M13" s="36">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="N13" s="36">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O13" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="P13" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R13" s="36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S13" s="36">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="T13" s="36">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="U13" s="36">
-        <v>8</v>
-      </c>
-      <c r="V13" s="37">
-        <v>3</v>
-      </c>
-      <c r="W13" s="35">
-        <f>V13-U13</f>
+        <v>1</v>
+      </c>
+      <c r="V13" s="36">
+        <v>4</v>
+      </c>
+      <c r="W13" s="37">
+        <v>2</v>
       </c>
       <c r="X13" s="35">
-        <f>V13-B13</f>
+        <f>W13-V13</f>
+      </c>
+      <c r="Y13" s="35">
+        <f>W13-B13</f>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B14" s="36">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C14" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D14" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="E14" s="36">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F14" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G14" s="36">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H14" s="36">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I14" s="36">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J14" s="36">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K14" s="36">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="L14" s="36">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="M14" s="36">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N14" s="36">
         <v>11</v>
       </c>
       <c r="O14" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P14" s="36">
         <v>10</v>
       </c>
       <c r="Q14" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R14" s="36">
+        <v>5</v>
+      </c>
+      <c r="S14" s="36">
         <v>6</v>
       </c>
-      <c r="S14" s="36">
-        <v>4</v>
-      </c>
       <c r="T14" s="36">
+        <v>6</v>
+      </c>
+      <c r="U14" s="36">
+        <v>6</v>
+      </c>
+      <c r="V14" s="36">
         <v>7</v>
       </c>
-      <c r="U14" s="36">
+      <c r="W14" s="37">
         <v>2</v>
       </c>
-      <c r="V14" s="37">
-        <v>3</v>
-      </c>
-      <c r="W14" s="34">
-        <f>V14-U14</f>
-      </c>
       <c r="X14" s="35">
-        <f>V14-B14</f>
+        <f>W14-V14</f>
+      </c>
+      <c r="Y14" s="35">
+        <f>W14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1329,11 +1368,14 @@
       <c r="V15" s="38">
         <f>SUM(V4:V14)</f>
       </c>
-      <c r="W15" s="41">
-        <f>V15-U15</f>
+      <c r="W15" s="38">
+        <f>SUM(W4:W14)</f>
       </c>
       <c r="X15" s="41">
-        <f>V15-B15</f>
+        <f>W15-V15</f>
+      </c>
+      <c r="Y15" s="41">
+        <f>W15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1457,6 +1499,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Y16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1524,15 +1571,18 @@
       <c r="U17" s="36">
         <v>51</v>
       </c>
-      <c r="V17" s="37">
+      <c r="V17" s="36">
         <v>27</v>
       </c>
-      <c r="W17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="W17" s="37">
+        <v>36</v>
       </c>
       <c r="X17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Y17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1604,15 +1654,18 @@
       <c r="U18" s="36">
         <v>28</v>
       </c>
-      <c r="V18" s="37">
+      <c r="V18" s="36">
         <v>24</v>
       </c>
-      <c r="W18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="W18" s="37">
+        <v>27</v>
       </c>
       <c r="X18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Y18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1684,15 +1737,18 @@
       <c r="U19" s="36">
         <f>U18-U17</f>
       </c>
-      <c r="V19" s="37">
+      <c r="V19" s="36">
         <f>V18-V17</f>
       </c>
-      <c r="W19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="W19" s="37">
+        <f>W18-W17</f>
       </c>
       <c r="X19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Y19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1764,15 +1820,18 @@
       <c r="U20" s="36">
         <v>8</v>
       </c>
-      <c r="V20" s="37">
+      <c r="V20" s="36">
         <v>7</v>
       </c>
-      <c r="W20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="W20" s="37">
+        <v>5</v>
       </c>
       <c r="X20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Y20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-25 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -292,13 +292,16 @@
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="10" customWidth="1"/>
     <col min="23" max="23" width="10" customWidth="1"/>
-    <col min="24" max="24" width="12" customWidth="1"/>
+    <col min="24" max="24" width="10" customWidth="1"/>
+    <col min="25" max="25" width="10" customWidth="1"/>
+    <col min="26" max="26" width="10" customWidth="1"/>
+    <col min="27" max="27" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 22/10 · variação 21/10 → 22/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 25/10 · variação 24/10 → 25/10</t>
         </is>
       </c>
     </row>
@@ -421,10 +424,25 @@
       </c>
       <c r="X3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">23/10</t>
+        </is>
+      </c>
+      <c r="Y3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24/10</t>
+        </is>
+      </c>
+      <c r="Z3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25/10</t>
+        </is>
+      </c>
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="Y3" s="1" t="inlineStr">
+      <c r="AB3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -499,279 +517,315 @@
       <c r="V4" s="36">
         <v>35</v>
       </c>
-      <c r="W4" s="37">
+      <c r="W4" s="36">
         <v>31</v>
       </c>
-      <c r="X4" s="35">
-        <f>W4-V4</f>
-      </c>
-      <c r="Y4" s="35">
-        <f>W4-B4</f>
+      <c r="X4" s="36">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="36">
+        <v>36</v>
+      </c>
+      <c r="Z4" s="37">
+        <v>36</v>
+      </c>
+      <c r="AA4" s="36">
+        <f>Z4-Y4</f>
+      </c>
+      <c r="AB4" s="35">
+        <f>Z4-B4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">NE</t>
         </is>
       </c>
       <c r="B5" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C5" s="36">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D5" s="36">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="E5" s="36">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="F5" s="36">
+        <v>42</v>
+      </c>
+      <c r="G5" s="36">
+        <v>45</v>
+      </c>
+      <c r="H5" s="36">
+        <v>41</v>
+      </c>
+      <c r="I5" s="36">
+        <v>39</v>
+      </c>
+      <c r="J5" s="36">
+        <v>14</v>
+      </c>
+      <c r="K5" s="36">
+        <v>12</v>
+      </c>
+      <c r="L5" s="36">
+        <v>10</v>
+      </c>
+      <c r="M5" s="36">
+        <v>10</v>
+      </c>
+      <c r="N5" s="36">
+        <v>13</v>
+      </c>
+      <c r="O5" s="36">
+        <v>12</v>
+      </c>
+      <c r="P5" s="36">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="36">
+        <v>11</v>
+      </c>
+      <c r="R5" s="36">
+        <v>13</v>
+      </c>
+      <c r="S5" s="36">
         <v>17</v>
-      </c>
-      <c r="G5" s="36">
-        <v>17</v>
-      </c>
-      <c r="H5" s="36">
-        <v>18</v>
-      </c>
-      <c r="I5" s="36">
-        <v>18</v>
-      </c>
-      <c r="J5" s="36">
-        <v>22</v>
-      </c>
-      <c r="K5" s="36">
-        <v>16</v>
-      </c>
-      <c r="L5" s="36">
-        <v>12</v>
-      </c>
-      <c r="M5" s="36">
-        <v>12</v>
-      </c>
-      <c r="N5" s="36">
-        <v>17</v>
-      </c>
-      <c r="O5" s="36">
-        <v>16</v>
-      </c>
-      <c r="P5" s="36">
-        <v>14</v>
-      </c>
-      <c r="Q5" s="36">
-        <v>16</v>
-      </c>
-      <c r="R5" s="36">
-        <v>15</v>
-      </c>
-      <c r="S5" s="36">
-        <v>15</v>
       </c>
       <c r="T5" s="36">
         <v>14</v>
       </c>
       <c r="U5" s="36">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="V5" s="36">
-        <v>11</v>
-      </c>
-      <c r="W5" s="37">
+        <v>13</v>
+      </c>
+      <c r="W5" s="36">
         <v>14</v>
       </c>
-      <c r="X5" s="34">
-        <f>W5-V5</f>
-      </c>
-      <c r="Y5" s="35">
-        <f>W5-B5</f>
+      <c r="X5" s="36">
+        <v>17</v>
+      </c>
+      <c r="Y5" s="36">
+        <v>15</v>
+      </c>
+      <c r="Z5" s="37">
+        <v>15</v>
+      </c>
+      <c r="AA5" s="36">
+        <f>Z5-Y5</f>
+      </c>
+      <c r="AB5" s="35">
+        <f>Z5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">NE</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="C6" s="36">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D6" s="36">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E6" s="36">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F6" s="36">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="G6" s="36">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="H6" s="36">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="I6" s="36">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="J6" s="36">
+        <v>22</v>
+      </c>
+      <c r="K6" s="36">
+        <v>16</v>
+      </c>
+      <c r="L6" s="36">
+        <v>12</v>
+      </c>
+      <c r="M6" s="36">
+        <v>12</v>
+      </c>
+      <c r="N6" s="36">
+        <v>17</v>
+      </c>
+      <c r="O6" s="36">
+        <v>16</v>
+      </c>
+      <c r="P6" s="36">
         <v>14</v>
       </c>
-      <c r="K6" s="36">
-        <v>12</v>
-      </c>
-      <c r="L6" s="36">
-        <v>10</v>
-      </c>
-      <c r="M6" s="36">
-        <v>10</v>
-      </c>
-      <c r="N6" s="36">
-        <v>13</v>
-      </c>
-      <c r="O6" s="36">
-        <v>12</v>
-      </c>
-      <c r="P6" s="36">
+      <c r="Q6" s="36">
+        <v>16</v>
+      </c>
+      <c r="R6" s="36">
         <v>15</v>
       </c>
-      <c r="Q6" s="36">
-        <v>11</v>
-      </c>
-      <c r="R6" s="36">
-        <v>13</v>
-      </c>
       <c r="S6" s="36">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="T6" s="36">
         <v>14</v>
       </c>
       <c r="U6" s="36">
+        <v>8</v>
+      </c>
+      <c r="V6" s="36">
+        <v>11</v>
+      </c>
+      <c r="W6" s="36">
         <v>14</v>
       </c>
-      <c r="V6" s="36">
-        <v>13</v>
-      </c>
-      <c r="W6" s="37">
-        <v>14</v>
-      </c>
-      <c r="X6" s="34">
-        <f>W6-V6</f>
-      </c>
-      <c r="Y6" s="35">
-        <f>W6-B6</f>
+      <c r="X6" s="36">
+        <v>12</v>
+      </c>
+      <c r="Y6" s="36">
+        <v>11</v>
+      </c>
+      <c r="Z6" s="37">
+        <v>9</v>
+      </c>
+      <c r="AA6" s="35">
+        <f>Z6-Y6</f>
+      </c>
+      <c r="AB6" s="35">
+        <f>Z6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C7" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D7" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="E7" s="36">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F7" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G7" s="36">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H7" s="36">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I7" s="36">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J7" s="36">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K7" s="36">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="L7" s="36">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="M7" s="36">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N7" s="36">
         <v>11</v>
       </c>
       <c r="O7" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P7" s="36">
         <v>10</v>
       </c>
       <c r="Q7" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R7" s="36">
+        <v>5</v>
+      </c>
+      <c r="S7" s="36">
         <v>6</v>
       </c>
-      <c r="S7" s="36">
+      <c r="T7" s="36">
+        <v>6</v>
+      </c>
+      <c r="U7" s="36">
+        <v>6</v>
+      </c>
+      <c r="V7" s="36">
+        <v>7</v>
+      </c>
+      <c r="W7" s="36">
+        <v>2</v>
+      </c>
+      <c r="X7" s="36">
         <v>4</v>
       </c>
-      <c r="T7" s="36">
-        <v>7</v>
-      </c>
-      <c r="U7" s="36">
+      <c r="Y7" s="36">
         <v>2</v>
       </c>
-      <c r="V7" s="36">
-        <v>3</v>
-      </c>
-      <c r="W7" s="37">
-        <v>6</v>
-      </c>
-      <c r="X7" s="34">
-        <f>W7-V7</f>
-      </c>
-      <c r="Y7" s="35">
-        <f>W7-B7</f>
+      <c r="Z7" s="37">
+        <v>5</v>
+      </c>
+      <c r="AA7" s="34">
+        <f>Z7-Y7</f>
+      </c>
+      <c r="AB7" s="35">
+        <f>Z7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C8" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D8" s="36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E8" s="36">
+        <v>10</v>
+      </c>
+      <c r="F8" s="36">
         <v>12</v>
       </c>
-      <c r="F8" s="36">
-        <v>13</v>
-      </c>
       <c r="G8" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H8" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I8" s="36">
         <v>7</v>
@@ -780,207 +834,234 @@
         <v>6</v>
       </c>
       <c r="K8" s="36">
+        <v>7</v>
+      </c>
+      <c r="L8" s="36">
+        <v>7</v>
+      </c>
+      <c r="M8" s="36">
+        <v>7</v>
+      </c>
+      <c r="N8" s="36">
+        <v>10</v>
+      </c>
+      <c r="O8" s="36">
+        <v>7</v>
+      </c>
+      <c r="P8" s="36">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="36">
         <v>6</v>
       </c>
-      <c r="L8" s="36">
-        <v>7</v>
-      </c>
-      <c r="M8" s="36">
-        <v>7</v>
-      </c>
-      <c r="N8" s="36">
-        <v>13</v>
-      </c>
-      <c r="O8" s="36">
-        <v>13</v>
-      </c>
-      <c r="P8" s="36">
-        <v>13</v>
-      </c>
-      <c r="Q8" s="36">
-        <v>10</v>
-      </c>
       <c r="R8" s="36">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="S8" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T8" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U8" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="V8" s="36">
+        <v>8</v>
+      </c>
+      <c r="W8" s="36">
+        <v>4</v>
+      </c>
+      <c r="X8" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y8" s="36">
         <v>6</v>
       </c>
-      <c r="W8" s="37">
+      <c r="Z8" s="37">
         <v>5</v>
       </c>
-      <c r="X8" s="35">
-        <f>W8-V8</f>
-      </c>
-      <c r="Y8" s="35">
-        <f>W8-B8</f>
+      <c r="AA8" s="35">
+        <f>Z8-Y8</f>
+      </c>
+      <c r="AB8" s="35">
+        <f>Z8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="36">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F9" s="36">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G9" s="36">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H9" s="36">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I9" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J9" s="36">
+        <v>5</v>
+      </c>
+      <c r="K9" s="36">
+        <v>4</v>
+      </c>
+      <c r="L9" s="36">
+        <v>4</v>
+      </c>
+      <c r="M9" s="36">
+        <v>5</v>
+      </c>
+      <c r="N9" s="36">
+        <v>8</v>
+      </c>
+      <c r="O9" s="36">
         <v>6</v>
       </c>
-      <c r="K9" s="36">
-        <v>7</v>
-      </c>
-      <c r="L9" s="36">
-        <v>7</v>
-      </c>
-      <c r="M9" s="36">
-        <v>7</v>
-      </c>
-      <c r="N9" s="36">
-        <v>10</v>
-      </c>
-      <c r="O9" s="36">
-        <v>7</v>
-      </c>
       <c r="P9" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="36">
+        <v>5</v>
+      </c>
+      <c r="R9" s="36">
+        <v>5</v>
+      </c>
+      <c r="S9" s="36">
         <v>6</v>
       </c>
-      <c r="R9" s="36">
-        <v>6</v>
-      </c>
-      <c r="S9" s="36">
+      <c r="T9" s="36">
         <v>5</v>
       </c>
-      <c r="T9" s="36">
-        <v>8</v>
-      </c>
       <c r="U9" s="36">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="V9" s="36">
-        <v>8</v>
-      </c>
-      <c r="W9" s="37">
+        <v>3</v>
+      </c>
+      <c r="W9" s="36">
+        <v>3</v>
+      </c>
+      <c r="X9" s="36">
         <v>4</v>
       </c>
-      <c r="X9" s="35">
-        <f>W9-V9</f>
-      </c>
-      <c r="Y9" s="35">
-        <f>W9-B9</f>
+      <c r="Y9" s="36">
+        <v>4</v>
+      </c>
+      <c r="Z9" s="37">
+        <v>4</v>
+      </c>
+      <c r="AA9" s="36">
+        <f>Z9-Y9</f>
+      </c>
+      <c r="AB9" s="35">
+        <f>Z9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B10" s="36">
+        <v>35</v>
+      </c>
+      <c r="C10" s="36">
+        <v>33</v>
+      </c>
+      <c r="D10" s="36">
+        <v>33</v>
+      </c>
+      <c r="E10" s="36">
+        <v>35</v>
+      </c>
+      <c r="F10" s="36">
+        <v>39</v>
+      </c>
+      <c r="G10" s="36">
+        <v>32</v>
+      </c>
+      <c r="H10" s="36">
+        <v>27</v>
+      </c>
+      <c r="I10" s="36">
+        <v>25</v>
+      </c>
+      <c r="J10" s="36">
+        <v>20</v>
+      </c>
+      <c r="K10" s="36">
         <v>18</v>
       </c>
-      <c r="C10" s="36">
-        <v>16</v>
-      </c>
-      <c r="D10" s="36">
-        <v>20</v>
-      </c>
-      <c r="E10" s="36">
-        <v>22</v>
-      </c>
-      <c r="F10" s="36">
-        <v>23</v>
-      </c>
-      <c r="G10" s="36">
-        <v>20</v>
-      </c>
-      <c r="H10" s="36">
-        <v>18</v>
-      </c>
-      <c r="I10" s="36">
-        <v>18</v>
-      </c>
-      <c r="J10" s="36">
-        <v>19</v>
-      </c>
-      <c r="K10" s="36">
-        <v>17</v>
-      </c>
       <c r="L10" s="36">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M10" s="36">
         <v>14</v>
       </c>
       <c r="N10" s="36">
+        <v>11</v>
+      </c>
+      <c r="O10" s="36">
+        <v>10</v>
+      </c>
+      <c r="P10" s="36">
+        <v>10</v>
+      </c>
+      <c r="Q10" s="36">
         <v>9</v>
       </c>
-      <c r="O10" s="36">
-        <v>9</v>
-      </c>
-      <c r="P10" s="36">
-        <v>7</v>
-      </c>
-      <c r="Q10" s="36">
-        <v>6</v>
-      </c>
       <c r="R10" s="36">
+        <v>7</v>
+      </c>
+      <c r="S10" s="36">
         <v>5</v>
-      </c>
-      <c r="S10" s="36">
-        <v>7</v>
       </c>
       <c r="T10" s="36">
         <v>8</v>
       </c>
       <c r="U10" s="36">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="V10" s="36">
-        <v>3</v>
-      </c>
-      <c r="W10" s="37">
         <v>4</v>
       </c>
-      <c r="X10" s="34">
-        <f>W10-V10</f>
-      </c>
-      <c r="Y10" s="35">
-        <f>W10-B10</f>
+      <c r="W10" s="36">
+        <v>7</v>
+      </c>
+      <c r="X10" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y10" s="36">
+        <v>7</v>
+      </c>
+      <c r="Z10" s="37">
+        <v>4</v>
+      </c>
+      <c r="AA10" s="35">
+        <f>Z10-Y10</f>
+      </c>
+      <c r="AB10" s="35">
+        <f>Z10-B10</f>
       </c>
     </row>
     <row r="11">
@@ -1052,103 +1133,121 @@
       <c r="V11" s="36">
         <v>4</v>
       </c>
-      <c r="W11" s="37">
+      <c r="W11" s="36">
         <v>3</v>
       </c>
-      <c r="X11" s="35">
-        <f>W11-V11</f>
-      </c>
-      <c r="Y11" s="35">
-        <f>W11-B11</f>
+      <c r="X11" s="36">
+        <v>4</v>
+      </c>
+      <c r="Y11" s="36">
+        <v>4</v>
+      </c>
+      <c r="Z11" s="37">
+        <v>3</v>
+      </c>
+      <c r="AA11" s="35">
+        <f>Z11-Y11</f>
+      </c>
+      <c r="AB11" s="35">
+        <f>Z11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C12" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D12" s="36">
         <v>9</v>
       </c>
       <c r="E12" s="36">
+        <v>14</v>
+      </c>
+      <c r="F12" s="36">
+        <v>7</v>
+      </c>
+      <c r="G12" s="36">
         <v>6</v>
       </c>
-      <c r="F12" s="36">
-        <v>5</v>
-      </c>
-      <c r="G12" s="36">
-        <v>5</v>
-      </c>
       <c r="H12" s="36">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I12" s="36">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J12" s="36">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="K12" s="36">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="L12" s="36">
         <v>4</v>
       </c>
       <c r="M12" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12" s="36">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O12" s="36">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P12" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R12" s="36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S12" s="36">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T12" s="36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U12" s="36">
+        <v>1</v>
+      </c>
+      <c r="V12" s="36">
+        <v>4</v>
+      </c>
+      <c r="W12" s="36">
+        <v>2</v>
+      </c>
+      <c r="X12" s="36">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="36">
         <v>3</v>
       </c>
-      <c r="V12" s="36">
+      <c r="Z12" s="37">
         <v>3</v>
       </c>
-      <c r="W12" s="37">
-        <v>3</v>
-      </c>
-      <c r="X12" s="36">
-        <f>W12-V12</f>
-      </c>
-      <c r="Y12" s="35">
-        <f>W12-B12</f>
+      <c r="AA12" s="36">
+        <f>Z12-Y12</f>
+      </c>
+      <c r="AB12" s="35">
+        <f>Z12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="36">
         <v>7</v>
@@ -1157,83 +1256,92 @@
         <v>9</v>
       </c>
       <c r="E13" s="36">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F13" s="36">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G13" s="36">
+        <v>9</v>
+      </c>
+      <c r="H13" s="36">
+        <v>11</v>
+      </c>
+      <c r="I13" s="36">
+        <v>7</v>
+      </c>
+      <c r="J13" s="36">
         <v>6</v>
       </c>
-      <c r="H13" s="36">
-        <v>8</v>
-      </c>
-      <c r="I13" s="36">
-        <v>11</v>
-      </c>
-      <c r="J13" s="36">
-        <v>11</v>
-      </c>
       <c r="K13" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L13" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M13" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N13" s="36">
+        <v>13</v>
+      </c>
+      <c r="O13" s="36">
+        <v>13</v>
+      </c>
+      <c r="P13" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q13" s="36">
+        <v>10</v>
+      </c>
+      <c r="R13" s="36">
+        <v>13</v>
+      </c>
+      <c r="S13" s="36">
+        <v>10</v>
+      </c>
+      <c r="T13" s="36">
+        <v>10</v>
+      </c>
+      <c r="U13" s="36">
+        <v>7</v>
+      </c>
+      <c r="V13" s="36">
+        <v>6</v>
+      </c>
+      <c r="W13" s="36">
+        <v>5</v>
+      </c>
+      <c r="X13" s="36">
+        <v>3</v>
+      </c>
+      <c r="Y13" s="36">
+        <v>3</v>
+      </c>
+      <c r="Z13" s="37">
         <v>2</v>
       </c>
-      <c r="O13" s="36">
-        <v>3</v>
-      </c>
-      <c r="P13" s="36">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="36">
-        <v>2</v>
-      </c>
-      <c r="R13" s="36">
-        <v>1</v>
-      </c>
-      <c r="S13" s="36">
-        <v>1</v>
-      </c>
-      <c r="T13" s="36">
-        <v>1</v>
-      </c>
-      <c r="U13" s="36">
-        <v>1</v>
-      </c>
-      <c r="V13" s="36">
-        <v>4</v>
-      </c>
-      <c r="W13" s="37">
-        <v>2</v>
-      </c>
-      <c r="X13" s="35">
-        <f>W13-V13</f>
-      </c>
-      <c r="Y13" s="35">
-        <f>W13-B13</f>
+      <c r="AA13" s="35">
+        <f>Z13-Y13</f>
+      </c>
+      <c r="AB13" s="35">
+        <f>Z13-B13</f>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B14" s="36">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C14" s="36">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D14" s="36">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E14" s="36">
         <v>22</v>
@@ -1242,61 +1350,70 @@
         <v>23</v>
       </c>
       <c r="G14" s="36">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H14" s="36">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I14" s="36">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="J14" s="36">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="K14" s="36">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="L14" s="36">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="M14" s="36">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="N14" s="36">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O14" s="36">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P14" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q14" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R14" s="36">
         <v>5</v>
       </c>
       <c r="S14" s="36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T14" s="36">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U14" s="36">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V14" s="36">
-        <v>7</v>
-      </c>
-      <c r="W14" s="37">
+        <v>3</v>
+      </c>
+      <c r="W14" s="36">
+        <v>4</v>
+      </c>
+      <c r="X14" s="36">
         <v>2</v>
       </c>
-      <c r="X14" s="35">
-        <f>W14-V14</f>
-      </c>
-      <c r="Y14" s="35">
-        <f>W14-B14</f>
+      <c r="Y14" s="36">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="37">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="36">
+        <f>Z14-Y14</f>
+      </c>
+      <c r="AB14" s="35">
+        <f>Z14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1371,11 +1488,20 @@
       <c r="W15" s="38">
         <f>SUM(W4:W14)</f>
       </c>
-      <c r="X15" s="41">
-        <f>W15-V15</f>
-      </c>
-      <c r="Y15" s="41">
-        <f>W15-B15</f>
+      <c r="X15" s="38">
+        <f>SUM(X4:X14)</f>
+      </c>
+      <c r="Y15" s="38">
+        <f>SUM(Y4:Y14)</f>
+      </c>
+      <c r="Z15" s="38">
+        <f>SUM(Z4:Z14)</f>
+      </c>
+      <c r="AA15" s="41">
+        <f>Z15-Y15</f>
+      </c>
+      <c r="AB15" s="41">
+        <f>Z15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1504,6 +1630,21 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="Z16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1574,15 +1715,24 @@
       <c r="V17" s="36">
         <v>27</v>
       </c>
-      <c r="W17" s="37">
+      <c r="W17" s="36">
         <v>36</v>
       </c>
-      <c r="X17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Y17" s="36" t="inlineStr">
+      <c r="X17" s="36">
+        <v>22</v>
+      </c>
+      <c r="Y17" s="36">
+        <v>21</v>
+      </c>
+      <c r="Z17" s="37">
+        <v>28</v>
+      </c>
+      <c r="AA17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1657,15 +1807,24 @@
       <c r="V18" s="36">
         <v>24</v>
       </c>
-      <c r="W18" s="37">
+      <c r="W18" s="36">
         <v>27</v>
       </c>
-      <c r="X18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Y18" s="36" t="inlineStr">
+      <c r="X18" s="36">
+        <v>22</v>
+      </c>
+      <c r="Y18" s="36">
+        <v>23</v>
+      </c>
+      <c r="Z18" s="37">
+        <v>23</v>
+      </c>
+      <c r="AA18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1740,15 +1899,24 @@
       <c r="V19" s="36">
         <f>V18-V17</f>
       </c>
-      <c r="W19" s="37">
+      <c r="W19" s="36">
         <f>W18-W17</f>
       </c>
-      <c r="X19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Y19" s="36" t="inlineStr">
+      <c r="X19" s="36">
+        <f>X18-X17</f>
+      </c>
+      <c r="Y19" s="36">
+        <f>Y18-Y17</f>
+      </c>
+      <c r="Z19" s="37">
+        <f>Z18-Z17</f>
+      </c>
+      <c r="AA19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1823,15 +1991,24 @@
       <c r="V20" s="36">
         <v>7</v>
       </c>
-      <c r="W20" s="37">
+      <c r="W20" s="36">
         <v>5</v>
       </c>
-      <c r="X20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Y20" s="36" t="inlineStr">
+      <c r="X20" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y20" s="36">
+        <v>6</v>
+      </c>
+      <c r="Z20" s="37">
+        <v>7</v>
+      </c>
+      <c r="AA20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-26 (foto da noite falhou, recorte reconstruido de 27/10)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -295,13 +295,14 @@
     <col min="24" max="24" width="10" customWidth="1"/>
     <col min="25" max="25" width="10" customWidth="1"/>
     <col min="26" max="26" width="10" customWidth="1"/>
-    <col min="27" max="27" width="12" customWidth="1"/>
+    <col min="27" max="27" width="10" customWidth="1"/>
+    <col min="28" max="28" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 25/10 · variação 24/10 → 25/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 26/10 · variação 25/10 → 26/10</t>
         </is>
       </c>
     </row>
@@ -439,10 +440,15 @@
       </c>
       <c r="AA3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">26/10</t>
+        </is>
+      </c>
+      <c r="AB3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="AB3" s="1" t="inlineStr">
+      <c r="AC3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -526,14 +532,17 @@
       <c r="Y4" s="36">
         <v>36</v>
       </c>
-      <c r="Z4" s="37">
+      <c r="Z4" s="36">
         <v>36</v>
       </c>
-      <c r="AA4" s="36">
-        <f>Z4-Y4</f>
+      <c r="AA4" s="37">
+        <v>32</v>
       </c>
       <c r="AB4" s="35">
-        <f>Z4-B4</f>
+        <f>AA4-Z4</f>
+      </c>
+      <c r="AC4" s="35">
+        <f>AA4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -614,14 +623,17 @@
       <c r="Y5" s="36">
         <v>15</v>
       </c>
-      <c r="Z5" s="37">
+      <c r="Z5" s="36">
         <v>15</v>
       </c>
-      <c r="AA5" s="36">
-        <f>Z5-Y5</f>
+      <c r="AA5" s="37">
+        <v>13</v>
       </c>
       <c r="AB5" s="35">
-        <f>Z5-B5</f>
+        <f>AA5-Z5</f>
+      </c>
+      <c r="AC5" s="35">
+        <f>AA5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -702,14 +714,17 @@
       <c r="Y6" s="36">
         <v>11</v>
       </c>
-      <c r="Z6" s="37">
+      <c r="Z6" s="36">
         <v>9</v>
       </c>
-      <c r="AA6" s="35">
-        <f>Z6-Y6</f>
-      </c>
-      <c r="AB6" s="35">
-        <f>Z6-B6</f>
+      <c r="AA6" s="37">
+        <v>9</v>
+      </c>
+      <c r="AB6" s="36">
+        <f>AA6-Z6</f>
+      </c>
+      <c r="AC6" s="35">
+        <f>AA6-B6</f>
       </c>
     </row>
     <row r="7">
@@ -790,72 +805,75 @@
       <c r="Y7" s="36">
         <v>2</v>
       </c>
-      <c r="Z7" s="37">
+      <c r="Z7" s="36">
         <v>5</v>
       </c>
-      <c r="AA7" s="34">
-        <f>Z7-Y7</f>
-      </c>
-      <c r="AB7" s="35">
-        <f>Z7-B7</f>
+      <c r="AA7" s="37">
+        <v>7</v>
+      </c>
+      <c r="AB7" s="34">
+        <f>AA7-Z7</f>
+      </c>
+      <c r="AC7" s="35">
+        <f>AA7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C8" s="36">
+        <v>33</v>
+      </c>
+      <c r="D8" s="36">
+        <v>33</v>
+      </c>
+      <c r="E8" s="36">
+        <v>35</v>
+      </c>
+      <c r="F8" s="36">
+        <v>39</v>
+      </c>
+      <c r="G8" s="36">
+        <v>32</v>
+      </c>
+      <c r="H8" s="36">
+        <v>27</v>
+      </c>
+      <c r="I8" s="36">
+        <v>25</v>
+      </c>
+      <c r="J8" s="36">
+        <v>20</v>
+      </c>
+      <c r="K8" s="36">
+        <v>18</v>
+      </c>
+      <c r="L8" s="36">
+        <v>14</v>
+      </c>
+      <c r="M8" s="36">
+        <v>14</v>
+      </c>
+      <c r="N8" s="36">
         <v>11</v>
       </c>
-      <c r="D8" s="36">
+      <c r="O8" s="36">
         <v>10</v>
       </c>
-      <c r="E8" s="36">
+      <c r="P8" s="36">
         <v>10</v>
       </c>
-      <c r="F8" s="36">
-        <v>12</v>
-      </c>
-      <c r="G8" s="36">
-        <v>11</v>
-      </c>
-      <c r="H8" s="36">
-        <v>12</v>
-      </c>
-      <c r="I8" s="36">
-        <v>7</v>
-      </c>
-      <c r="J8" s="36">
-        <v>6</v>
-      </c>
-      <c r="K8" s="36">
-        <v>7</v>
-      </c>
-      <c r="L8" s="36">
-        <v>7</v>
-      </c>
-      <c r="M8" s="36">
-        <v>7</v>
-      </c>
-      <c r="N8" s="36">
-        <v>10</v>
-      </c>
-      <c r="O8" s="36">
-        <v>7</v>
-      </c>
-      <c r="P8" s="36">
-        <v>8</v>
-      </c>
       <c r="Q8" s="36">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="R8" s="36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" s="36">
         <v>5</v>
@@ -864,204 +882,213 @@
         <v>8</v>
       </c>
       <c r="U8" s="36">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="V8" s="36">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W8" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="X8" s="36">
         <v>5</v>
       </c>
       <c r="Y8" s="36">
-        <v>6</v>
-      </c>
-      <c r="Z8" s="37">
+        <v>7</v>
+      </c>
+      <c r="Z8" s="36">
+        <v>4</v>
+      </c>
+      <c r="AA8" s="37">
         <v>5</v>
       </c>
-      <c r="AA8" s="35">
-        <f>Z8-Y8</f>
-      </c>
-      <c r="AB8" s="35">
-        <f>Z8-B8</f>
+      <c r="AB8" s="34">
+        <f>AA8-Z8</f>
+      </c>
+      <c r="AC8" s="35">
+        <f>AA8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B9" s="36">
+        <v>12</v>
+      </c>
+      <c r="C9" s="36">
         <v>11</v>
       </c>
-      <c r="C9" s="36">
+      <c r="D9" s="36">
         <v>10</v>
       </c>
-      <c r="D9" s="36">
-        <v>9</v>
-      </c>
       <c r="E9" s="36">
+        <v>10</v>
+      </c>
+      <c r="F9" s="36">
+        <v>12</v>
+      </c>
+      <c r="G9" s="36">
+        <v>11</v>
+      </c>
+      <c r="H9" s="36">
+        <v>12</v>
+      </c>
+      <c r="I9" s="36">
+        <v>7</v>
+      </c>
+      <c r="J9" s="36">
         <v>6</v>
       </c>
-      <c r="F9" s="36">
+      <c r="K9" s="36">
+        <v>7</v>
+      </c>
+      <c r="L9" s="36">
+        <v>7</v>
+      </c>
+      <c r="M9" s="36">
+        <v>7</v>
+      </c>
+      <c r="N9" s="36">
+        <v>10</v>
+      </c>
+      <c r="O9" s="36">
+        <v>7</v>
+      </c>
+      <c r="P9" s="36">
+        <v>8</v>
+      </c>
+      <c r="Q9" s="36">
+        <v>6</v>
+      </c>
+      <c r="R9" s="36">
+        <v>6</v>
+      </c>
+      <c r="S9" s="36">
         <v>5</v>
       </c>
-      <c r="G9" s="36">
+      <c r="T9" s="36">
+        <v>8</v>
+      </c>
+      <c r="U9" s="36">
+        <v>11</v>
+      </c>
+      <c r="V9" s="36">
+        <v>8</v>
+      </c>
+      <c r="W9" s="36">
+        <v>4</v>
+      </c>
+      <c r="X9" s="36">
         <v>5</v>
       </c>
-      <c r="H9" s="36">
+      <c r="Y9" s="36">
+        <v>6</v>
+      </c>
+      <c r="Z9" s="36">
         <v>5</v>
       </c>
-      <c r="I9" s="36">
-        <v>6</v>
-      </c>
-      <c r="J9" s="36">
-        <v>5</v>
-      </c>
-      <c r="K9" s="36">
-        <v>4</v>
-      </c>
-      <c r="L9" s="36">
-        <v>4</v>
-      </c>
-      <c r="M9" s="36">
-        <v>5</v>
-      </c>
-      <c r="N9" s="36">
-        <v>8</v>
-      </c>
-      <c r="O9" s="36">
-        <v>6</v>
-      </c>
-      <c r="P9" s="36">
-        <v>5</v>
-      </c>
-      <c r="Q9" s="36">
-        <v>5</v>
-      </c>
-      <c r="R9" s="36">
-        <v>5</v>
-      </c>
-      <c r="S9" s="36">
-        <v>6</v>
-      </c>
-      <c r="T9" s="36">
-        <v>5</v>
-      </c>
-      <c r="U9" s="36">
-        <v>3</v>
-      </c>
-      <c r="V9" s="36">
-        <v>3</v>
-      </c>
-      <c r="W9" s="36">
-        <v>3</v>
-      </c>
-      <c r="X9" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y9" s="36">
-        <v>4</v>
-      </c>
-      <c r="Z9" s="37">
-        <v>4</v>
-      </c>
-      <c r="AA9" s="36">
-        <f>Z9-Y9</f>
+      <c r="AA9" s="37">
+        <v>4</v>
       </c>
       <c r="AB9" s="35">
-        <f>Z9-B9</f>
+        <f>AA9-Z9</f>
+      </c>
+      <c r="AC9" s="35">
+        <f>AA9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C10" s="36">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D10" s="36">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E10" s="36">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F10" s="36">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="G10" s="36">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H10" s="36">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="I10" s="36">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="J10" s="36">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="K10" s="36">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="L10" s="36">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M10" s="36">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="N10" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O10" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="P10" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="36">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="R10" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S10" s="36">
+        <v>6</v>
+      </c>
+      <c r="T10" s="36">
         <v>5</v>
-      </c>
-      <c r="T10" s="36">
-        <v>8</v>
       </c>
       <c r="U10" s="36">
         <v>3</v>
       </c>
       <c r="V10" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W10" s="36">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="X10" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Y10" s="36">
-        <v>7</v>
-      </c>
-      <c r="Z10" s="37">
-        <v>4</v>
-      </c>
-      <c r="AA10" s="35">
-        <f>Z10-Y10</f>
+        <v>4</v>
+      </c>
+      <c r="Z10" s="36">
+        <v>4</v>
+      </c>
+      <c r="AA10" s="37">
+        <v>3</v>
       </c>
       <c r="AB10" s="35">
-        <f>Z10-B10</f>
+        <f>AA10-Z10</f>
+      </c>
+      <c r="AC10" s="35">
+        <f>AA10-B10</f>
       </c>
     </row>
     <row r="11">
@@ -1142,24 +1169,27 @@
       <c r="Y11" s="36">
         <v>4</v>
       </c>
-      <c r="Z11" s="37">
+      <c r="Z11" s="36">
         <v>3</v>
       </c>
-      <c r="AA11" s="35">
-        <f>Z11-Y11</f>
+      <c r="AA11" s="37">
+        <v>2</v>
       </c>
       <c r="AB11" s="35">
-        <f>Z11-B11</f>
+        <f>AA11-Z11</f>
+      </c>
+      <c r="AC11" s="35">
+        <f>AA11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="36">
         <v>7</v>
@@ -1168,86 +1198,89 @@
         <v>9</v>
       </c>
       <c r="E12" s="36">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F12" s="36">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G12" s="36">
+        <v>9</v>
+      </c>
+      <c r="H12" s="36">
+        <v>11</v>
+      </c>
+      <c r="I12" s="36">
+        <v>7</v>
+      </c>
+      <c r="J12" s="36">
         <v>6</v>
       </c>
-      <c r="H12" s="36">
-        <v>8</v>
-      </c>
-      <c r="I12" s="36">
-        <v>11</v>
-      </c>
-      <c r="J12" s="36">
-        <v>11</v>
-      </c>
       <c r="K12" s="36">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L12" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M12" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N12" s="36">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="O12" s="36">
+        <v>13</v>
+      </c>
+      <c r="P12" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q12" s="36">
+        <v>10</v>
+      </c>
+      <c r="R12" s="36">
+        <v>13</v>
+      </c>
+      <c r="S12" s="36">
+        <v>10</v>
+      </c>
+      <c r="T12" s="36">
+        <v>10</v>
+      </c>
+      <c r="U12" s="36">
+        <v>7</v>
+      </c>
+      <c r="V12" s="36">
+        <v>6</v>
+      </c>
+      <c r="W12" s="36">
+        <v>5</v>
+      </c>
+      <c r="X12" s="36">
         <v>3</v>
-      </c>
-      <c r="P12" s="36">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="36">
-        <v>2</v>
-      </c>
-      <c r="R12" s="36">
-        <v>1</v>
-      </c>
-      <c r="S12" s="36">
-        <v>1</v>
-      </c>
-      <c r="T12" s="36">
-        <v>1</v>
-      </c>
-      <c r="U12" s="36">
-        <v>1</v>
-      </c>
-      <c r="V12" s="36">
-        <v>4</v>
-      </c>
-      <c r="W12" s="36">
-        <v>2</v>
-      </c>
-      <c r="X12" s="36">
-        <v>0</v>
       </c>
       <c r="Y12" s="36">
         <v>3</v>
       </c>
-      <c r="Z12" s="37">
-        <v>3</v>
-      </c>
-      <c r="AA12" s="36">
-        <f>Z12-Y12</f>
-      </c>
-      <c r="AB12" s="35">
-        <f>Z12-B12</f>
+      <c r="Z12" s="36">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="37">
+        <v>2</v>
+      </c>
+      <c r="AB12" s="36">
+        <f>AA12-Z12</f>
+      </c>
+      <c r="AC12" s="35">
+        <f>AA12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C13" s="36">
         <v>7</v>
@@ -1256,76 +1289,79 @@
         <v>9</v>
       </c>
       <c r="E13" s="36">
+        <v>14</v>
+      </c>
+      <c r="F13" s="36">
+        <v>7</v>
+      </c>
+      <c r="G13" s="36">
+        <v>6</v>
+      </c>
+      <c r="H13" s="36">
+        <v>8</v>
+      </c>
+      <c r="I13" s="36">
+        <v>11</v>
+      </c>
+      <c r="J13" s="36">
+        <v>11</v>
+      </c>
+      <c r="K13" s="36">
         <v>12</v>
       </c>
-      <c r="F13" s="36">
-        <v>13</v>
-      </c>
-      <c r="G13" s="36">
-        <v>9</v>
-      </c>
-      <c r="H13" s="36">
-        <v>11</v>
-      </c>
-      <c r="I13" s="36">
-        <v>7</v>
-      </c>
-      <c r="J13" s="36">
-        <v>6</v>
-      </c>
-      <c r="K13" s="36">
-        <v>6</v>
-      </c>
       <c r="L13" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M13" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N13" s="36">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="O13" s="36">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P13" s="36">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="36">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="R13" s="36">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="S13" s="36">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="T13" s="36">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="U13" s="36">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="V13" s="36">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W13" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="X13" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="36">
         <v>3</v>
       </c>
-      <c r="Z13" s="37">
+      <c r="Z13" s="36">
+        <v>3</v>
+      </c>
+      <c r="AA13" s="37">
         <v>2</v>
       </c>
-      <c r="AA13" s="35">
-        <f>Z13-Y13</f>
-      </c>
       <c r="AB13" s="35">
-        <f>Z13-B13</f>
+        <f>AA13-Z13</f>
+      </c>
+      <c r="AC13" s="35">
+        <f>AA13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -1406,14 +1442,17 @@
       <c r="Y14" s="36">
         <v>0</v>
       </c>
-      <c r="Z14" s="37">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="36">
-        <f>Z14-Y14</f>
-      </c>
-      <c r="AB14" s="35">
-        <f>Z14-B14</f>
+      <c r="Z14" s="36">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="37">
+        <v>2</v>
+      </c>
+      <c r="AB14" s="34">
+        <f>AA14-Z14</f>
+      </c>
+      <c r="AC14" s="35">
+        <f>AA14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1497,11 +1536,14 @@
       <c r="Z15" s="38">
         <f>SUM(Z4:Z14)</f>
       </c>
-      <c r="AA15" s="41">
-        <f>Z15-Y15</f>
+      <c r="AA15" s="38">
+        <f>SUM(AA4:AA14)</f>
       </c>
       <c r="AB15" s="41">
-        <f>Z15-B15</f>
+        <f>AA15-Z15</f>
+      </c>
+      <c r="AC15" s="41">
+        <f>AA15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1645,6 +1687,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="AC16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1724,15 +1771,18 @@
       <c r="Y17" s="36">
         <v>21</v>
       </c>
-      <c r="Z17" s="37">
+      <c r="Z17" s="36">
         <v>28</v>
       </c>
-      <c r="AA17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AA17" s="37">
+        <v>35</v>
       </c>
       <c r="AB17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AC17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1816,15 +1866,18 @@
       <c r="Y18" s="36">
         <v>23</v>
       </c>
-      <c r="Z18" s="37">
+      <c r="Z18" s="36">
         <v>23</v>
       </c>
-      <c r="AA18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AA18" s="37">
+        <v>30</v>
       </c>
       <c r="AB18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AC18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1908,15 +1961,18 @@
       <c r="Y19" s="36">
         <f>Y18-Y17</f>
       </c>
-      <c r="Z19" s="37">
+      <c r="Z19" s="36">
         <f>Z18-Z17</f>
       </c>
-      <c r="AA19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AA19" s="37">
+        <f>AA18-AA17</f>
       </c>
       <c r="AB19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AC19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2000,15 +2056,18 @@
       <c r="Y20" s="36">
         <v>6</v>
       </c>
-      <c r="Z20" s="37">
-        <v>7</v>
-      </c>
-      <c r="AA20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="Z20" s="36">
+        <v>7</v>
+      </c>
+      <c r="AA20" s="37">
+        <v>4</v>
       </c>
       <c r="AB20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AC20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-27 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -296,13 +296,14 @@
     <col min="25" max="25" width="10" customWidth="1"/>
     <col min="26" max="26" width="10" customWidth="1"/>
     <col min="27" max="27" width="10" customWidth="1"/>
-    <col min="28" max="28" width="12" customWidth="1"/>
+    <col min="28" max="28" width="10" customWidth="1"/>
+    <col min="29" max="29" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 26/10 · variação 25/10 → 26/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 27/10 · variação 26/10 → 27/10</t>
         </is>
       </c>
     </row>
@@ -445,10 +446,15 @@
       </c>
       <c r="AB3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">27/10</t>
+        </is>
+      </c>
+      <c r="AC3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="AC3" s="1" t="inlineStr">
+      <c r="AD3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -535,14 +541,17 @@
       <c r="Z4" s="36">
         <v>36</v>
       </c>
-      <c r="AA4" s="37">
+      <c r="AA4" s="36">
         <v>32</v>
       </c>
-      <c r="AB4" s="35">
-        <f>AA4-Z4</f>
-      </c>
-      <c r="AC4" s="35">
-        <f>AA4-B4</f>
+      <c r="AB4" s="37">
+        <v>32</v>
+      </c>
+      <c r="AC4" s="36">
+        <f>AB4-AA4</f>
+      </c>
+      <c r="AD4" s="35">
+        <f>AB4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -626,469 +635,487 @@
       <c r="Z5" s="36">
         <v>15</v>
       </c>
-      <c r="AA5" s="37">
+      <c r="AA5" s="36">
         <v>13</v>
       </c>
-      <c r="AB5" s="35">
-        <f>AA5-Z5</f>
-      </c>
-      <c r="AC5" s="35">
-        <f>AA5-B5</f>
+      <c r="AB5" s="37">
+        <v>14</v>
+      </c>
+      <c r="AC5" s="34">
+        <f>AB5-AA5</f>
+      </c>
+      <c r="AD5" s="35">
+        <f>AB5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C6" s="36">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="D6" s="36">
+        <v>33</v>
+      </c>
+      <c r="E6" s="36">
+        <v>35</v>
+      </c>
+      <c r="F6" s="36">
+        <v>39</v>
+      </c>
+      <c r="G6" s="36">
+        <v>32</v>
+      </c>
+      <c r="H6" s="36">
+        <v>27</v>
+      </c>
+      <c r="I6" s="36">
+        <v>25</v>
+      </c>
+      <c r="J6" s="36">
+        <v>20</v>
+      </c>
+      <c r="K6" s="36">
         <v>18</v>
       </c>
-      <c r="E6" s="36">
-        <v>20</v>
-      </c>
-      <c r="F6" s="36">
-        <v>17</v>
-      </c>
-      <c r="G6" s="36">
-        <v>17</v>
-      </c>
-      <c r="H6" s="36">
-        <v>18</v>
-      </c>
-      <c r="I6" s="36">
-        <v>18</v>
-      </c>
-      <c r="J6" s="36">
-        <v>22</v>
-      </c>
-      <c r="K6" s="36">
-        <v>16</v>
-      </c>
       <c r="L6" s="36">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M6" s="36">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N6" s="36">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="O6" s="36">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="P6" s="36">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="Q6" s="36">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="R6" s="36">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="S6" s="36">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="T6" s="36">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="U6" s="36">
+        <v>3</v>
+      </c>
+      <c r="V6" s="36">
+        <v>4</v>
+      </c>
+      <c r="W6" s="36">
+        <v>7</v>
+      </c>
+      <c r="X6" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y6" s="36">
+        <v>7</v>
+      </c>
+      <c r="Z6" s="36">
+        <v>4</v>
+      </c>
+      <c r="AA6" s="36">
+        <v>5</v>
+      </c>
+      <c r="AB6" s="37">
         <v>8</v>
       </c>
-      <c r="V6" s="36">
-        <v>11</v>
-      </c>
-      <c r="W6" s="36">
-        <v>14</v>
-      </c>
-      <c r="X6" s="36">
-        <v>12</v>
-      </c>
-      <c r="Y6" s="36">
-        <v>11</v>
-      </c>
-      <c r="Z6" s="36">
-        <v>9</v>
-      </c>
-      <c r="AA6" s="37">
-        <v>9</v>
-      </c>
-      <c r="AB6" s="36">
-        <f>AA6-Z6</f>
-      </c>
-      <c r="AC6" s="35">
-        <f>AA6-B6</f>
+      <c r="AC6" s="34">
+        <f>AB6-AA6</f>
+      </c>
+      <c r="AD6" s="35">
+        <f>AB6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C7" s="36">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D7" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E7" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F7" s="36">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="G7" s="36">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H7" s="36">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="I7" s="36">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J7" s="36">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="K7" s="36">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="L7" s="36">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="M7" s="36">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="N7" s="36">
+        <v>10</v>
+      </c>
+      <c r="O7" s="36">
+        <v>7</v>
+      </c>
+      <c r="P7" s="36">
+        <v>8</v>
+      </c>
+      <c r="Q7" s="36">
+        <v>6</v>
+      </c>
+      <c r="R7" s="36">
+        <v>6</v>
+      </c>
+      <c r="S7" s="36">
+        <v>5</v>
+      </c>
+      <c r="T7" s="36">
+        <v>8</v>
+      </c>
+      <c r="U7" s="36">
         <v>11</v>
       </c>
-      <c r="O7" s="36">
+      <c r="V7" s="36">
         <v>8</v>
       </c>
-      <c r="P7" s="36">
-        <v>10</v>
-      </c>
-      <c r="Q7" s="36">
-        <v>7</v>
-      </c>
-      <c r="R7" s="36">
-        <v>5</v>
-      </c>
-      <c r="S7" s="36">
+      <c r="W7" s="36">
+        <v>4</v>
+      </c>
+      <c r="X7" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y7" s="36">
         <v>6</v>
       </c>
-      <c r="T7" s="36">
+      <c r="Z7" s="36">
+        <v>5</v>
+      </c>
+      <c r="AA7" s="36">
+        <v>4</v>
+      </c>
+      <c r="AB7" s="37">
         <v>6</v>
       </c>
-      <c r="U7" s="36">
-        <v>6</v>
-      </c>
-      <c r="V7" s="36">
-        <v>7</v>
-      </c>
-      <c r="W7" s="36">
-        <v>2</v>
-      </c>
-      <c r="X7" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y7" s="36">
-        <v>2</v>
-      </c>
-      <c r="Z7" s="36">
-        <v>5</v>
-      </c>
-      <c r="AA7" s="37">
-        <v>7</v>
-      </c>
-      <c r="AB7" s="34">
-        <f>AA7-Z7</f>
-      </c>
-      <c r="AC7" s="35">
-        <f>AA7-B7</f>
+      <c r="AC7" s="34">
+        <f>AB7-AA7</f>
+      </c>
+      <c r="AD7" s="35">
+        <f>AB7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C8" s="36">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D8" s="36">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E8" s="36">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F8" s="36">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="G8" s="36">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H8" s="36">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="I8" s="36">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="J8" s="36">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="K8" s="36">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="L8" s="36">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M8" s="36">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="N8" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O8" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="P8" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="36">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="R8" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S8" s="36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T8" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U8" s="36">
         <v>3</v>
       </c>
       <c r="V8" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W8" s="36">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="X8" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Y8" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Z8" s="36">
         <v>4</v>
       </c>
-      <c r="AA8" s="37">
-        <v>5</v>
-      </c>
-      <c r="AB8" s="34">
-        <f>AA8-Z8</f>
-      </c>
-      <c r="AC8" s="35">
-        <f>AA8-B8</f>
+      <c r="AA8" s="36">
+        <v>3</v>
+      </c>
+      <c r="AB8" s="37">
+        <v>5</v>
+      </c>
+      <c r="AC8" s="34">
+        <f>AB8-AA8</f>
+      </c>
+      <c r="AD8" s="35">
+        <f>AB8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C9" s="36">
+        <v>22</v>
+      </c>
+      <c r="D9" s="36">
+        <v>22</v>
+      </c>
+      <c r="E9" s="36">
+        <v>22</v>
+      </c>
+      <c r="F9" s="36">
+        <v>23</v>
+      </c>
+      <c r="G9" s="36">
+        <v>25</v>
+      </c>
+      <c r="H9" s="36">
+        <v>24</v>
+      </c>
+      <c r="I9" s="36">
+        <v>28</v>
+      </c>
+      <c r="J9" s="36">
+        <v>30</v>
+      </c>
+      <c r="K9" s="36">
+        <v>31</v>
+      </c>
+      <c r="L9" s="36">
+        <v>26</v>
+      </c>
+      <c r="M9" s="36">
+        <v>24</v>
+      </c>
+      <c r="N9" s="36">
         <v>11</v>
       </c>
-      <c r="D9" s="36">
+      <c r="O9" s="36">
+        <v>8</v>
+      </c>
+      <c r="P9" s="36">
         <v>10</v>
       </c>
-      <c r="E9" s="36">
-        <v>10</v>
-      </c>
-      <c r="F9" s="36">
-        <v>12</v>
-      </c>
-      <c r="G9" s="36">
-        <v>11</v>
-      </c>
-      <c r="H9" s="36">
-        <v>12</v>
-      </c>
-      <c r="I9" s="36">
-        <v>7</v>
-      </c>
-      <c r="J9" s="36">
+      <c r="Q9" s="36">
+        <v>7</v>
+      </c>
+      <c r="R9" s="36">
+        <v>5</v>
+      </c>
+      <c r="S9" s="36">
         <v>6</v>
       </c>
-      <c r="K9" s="36">
-        <v>7</v>
-      </c>
-      <c r="L9" s="36">
-        <v>7</v>
-      </c>
-      <c r="M9" s="36">
-        <v>7</v>
-      </c>
-      <c r="N9" s="36">
-        <v>10</v>
-      </c>
-      <c r="O9" s="36">
-        <v>7</v>
-      </c>
-      <c r="P9" s="36">
-        <v>8</v>
-      </c>
-      <c r="Q9" s="36">
+      <c r="T9" s="36">
         <v>6</v>
       </c>
-      <c r="R9" s="36">
+      <c r="U9" s="36">
         <v>6</v>
       </c>
-      <c r="S9" s="36">
-        <v>5</v>
-      </c>
-      <c r="T9" s="36">
-        <v>8</v>
-      </c>
-      <c r="U9" s="36">
-        <v>11</v>
-      </c>
       <c r="V9" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W9" s="36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X9" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Y9" s="36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z9" s="36">
         <v>5</v>
       </c>
-      <c r="AA9" s="37">
-        <v>4</v>
-      </c>
-      <c r="AB9" s="35">
-        <f>AA9-Z9</f>
+      <c r="AA9" s="36">
+        <v>7</v>
+      </c>
+      <c r="AB9" s="37">
+        <v>4</v>
       </c>
       <c r="AC9" s="35">
-        <f>AA9-B9</f>
+        <f>AB9-AA9</f>
+      </c>
+      <c r="AD9" s="35">
+        <f>AB9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B10" s="36">
+        <v>21</v>
+      </c>
+      <c r="C10" s="36">
+        <v>21</v>
+      </c>
+      <c r="D10" s="36">
+        <v>18</v>
+      </c>
+      <c r="E10" s="36">
+        <v>20</v>
+      </c>
+      <c r="F10" s="36">
+        <v>17</v>
+      </c>
+      <c r="G10" s="36">
+        <v>17</v>
+      </c>
+      <c r="H10" s="36">
+        <v>18</v>
+      </c>
+      <c r="I10" s="36">
+        <v>18</v>
+      </c>
+      <c r="J10" s="36">
+        <v>22</v>
+      </c>
+      <c r="K10" s="36">
+        <v>16</v>
+      </c>
+      <c r="L10" s="36">
+        <v>12</v>
+      </c>
+      <c r="M10" s="36">
+        <v>12</v>
+      </c>
+      <c r="N10" s="36">
+        <v>17</v>
+      </c>
+      <c r="O10" s="36">
+        <v>16</v>
+      </c>
+      <c r="P10" s="36">
+        <v>14</v>
+      </c>
+      <c r="Q10" s="36">
+        <v>16</v>
+      </c>
+      <c r="R10" s="36">
+        <v>15</v>
+      </c>
+      <c r="S10" s="36">
+        <v>15</v>
+      </c>
+      <c r="T10" s="36">
+        <v>14</v>
+      </c>
+      <c r="U10" s="36">
+        <v>8</v>
+      </c>
+      <c r="V10" s="36">
         <v>11</v>
       </c>
-      <c r="C10" s="36">
-        <v>10</v>
-      </c>
-      <c r="D10" s="36">
+      <c r="W10" s="36">
+        <v>14</v>
+      </c>
+      <c r="X10" s="36">
+        <v>12</v>
+      </c>
+      <c r="Y10" s="36">
+        <v>11</v>
+      </c>
+      <c r="Z10" s="36">
         <v>9</v>
       </c>
-      <c r="E10" s="36">
-        <v>6</v>
-      </c>
-      <c r="F10" s="36">
-        <v>5</v>
-      </c>
-      <c r="G10" s="36">
-        <v>5</v>
-      </c>
-      <c r="H10" s="36">
-        <v>5</v>
-      </c>
-      <c r="I10" s="36">
-        <v>6</v>
-      </c>
-      <c r="J10" s="36">
-        <v>5</v>
-      </c>
-      <c r="K10" s="36">
-        <v>4</v>
-      </c>
-      <c r="L10" s="36">
-        <v>4</v>
-      </c>
-      <c r="M10" s="36">
-        <v>5</v>
-      </c>
-      <c r="N10" s="36">
-        <v>8</v>
-      </c>
-      <c r="O10" s="36">
-        <v>6</v>
-      </c>
-      <c r="P10" s="36">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="36">
-        <v>5</v>
-      </c>
-      <c r="R10" s="36">
-        <v>5</v>
-      </c>
-      <c r="S10" s="36">
-        <v>6</v>
-      </c>
-      <c r="T10" s="36">
-        <v>5</v>
-      </c>
-      <c r="U10" s="36">
+      <c r="AA10" s="36">
+        <v>9</v>
+      </c>
+      <c r="AB10" s="37">
         <v>3</v>
       </c>
-      <c r="V10" s="36">
-        <v>3</v>
-      </c>
-      <c r="W10" s="36">
-        <v>3</v>
-      </c>
-      <c r="X10" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y10" s="36">
-        <v>4</v>
-      </c>
-      <c r="Z10" s="36">
-        <v>4</v>
-      </c>
-      <c r="AA10" s="37">
-        <v>3</v>
-      </c>
-      <c r="AB10" s="35">
-        <f>AA10-Z10</f>
-      </c>
       <c r="AC10" s="35">
-        <f>AA10-B10</f>
+        <f>AB10-AA10</f>
+      </c>
+      <c r="AD10" s="35">
+        <f>AB10-B10</f>
       </c>
     </row>
     <row r="11">
@@ -1172,14 +1199,17 @@
       <c r="Z11" s="36">
         <v>3</v>
       </c>
-      <c r="AA11" s="37">
+      <c r="AA11" s="36">
         <v>2</v>
       </c>
-      <c r="AB11" s="35">
-        <f>AA11-Z11</f>
-      </c>
-      <c r="AC11" s="35">
-        <f>AA11-B11</f>
+      <c r="AB11" s="37">
+        <v>2</v>
+      </c>
+      <c r="AC11" s="36">
+        <f>AB11-AA11</f>
+      </c>
+      <c r="AD11" s="35">
+        <f>AB11-B11</f>
       </c>
     </row>
     <row r="12">
@@ -1263,14 +1293,17 @@
       <c r="Z12" s="36">
         <v>2</v>
       </c>
-      <c r="AA12" s="37">
+      <c r="AA12" s="36">
         <v>2</v>
       </c>
-      <c r="AB12" s="36">
-        <f>AA12-Z12</f>
-      </c>
-      <c r="AC12" s="35">
-        <f>AA12-B12</f>
+      <c r="AB12" s="37">
+        <v>2</v>
+      </c>
+      <c r="AC12" s="36">
+        <f>AB12-AA12</f>
+      </c>
+      <c r="AD12" s="35">
+        <f>AB12-B12</f>
       </c>
     </row>
     <row r="13">
@@ -1354,14 +1387,17 @@
       <c r="Z13" s="36">
         <v>3</v>
       </c>
-      <c r="AA13" s="37">
+      <c r="AA13" s="36">
         <v>2</v>
       </c>
-      <c r="AB13" s="35">
-        <f>AA13-Z13</f>
+      <c r="AB13" s="37">
+        <v>1</v>
       </c>
       <c r="AC13" s="35">
-        <f>AA13-B13</f>
+        <f>AB13-AA13</f>
+      </c>
+      <c r="AD13" s="35">
+        <f>AB13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -1445,14 +1481,17 @@
       <c r="Z14" s="36">
         <v>0</v>
       </c>
-      <c r="AA14" s="37">
+      <c r="AA14" s="36">
         <v>2</v>
       </c>
-      <c r="AB14" s="34">
-        <f>AA14-Z14</f>
+      <c r="AB14" s="37">
+        <v>1</v>
       </c>
       <c r="AC14" s="35">
-        <f>AA14-B14</f>
+        <f>AB14-AA14</f>
+      </c>
+      <c r="AD14" s="35">
+        <f>AB14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1539,11 +1578,14 @@
       <c r="AA15" s="38">
         <f>SUM(AA4:AA14)</f>
       </c>
-      <c r="AB15" s="41">
-        <f>AA15-Z15</f>
+      <c r="AB15" s="38">
+        <f>SUM(AB4:AB14)</f>
       </c>
       <c r="AC15" s="41">
-        <f>AA15-B15</f>
+        <f>AB15-AA15</f>
+      </c>
+      <c r="AD15" s="41">
+        <f>AB15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1692,6 +1734,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="AD16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1774,15 +1821,18 @@
       <c r="Z17" s="36">
         <v>28</v>
       </c>
-      <c r="AA17" s="37">
+      <c r="AA17" s="36">
         <v>35</v>
       </c>
-      <c r="AB17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AB17" s="37">
+        <v>33</v>
       </c>
       <c r="AC17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AD17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1869,15 +1919,18 @@
       <c r="Z18" s="36">
         <v>23</v>
       </c>
-      <c r="AA18" s="37">
+      <c r="AA18" s="36">
         <v>30</v>
       </c>
-      <c r="AB18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AB18" s="37">
+        <v>30</v>
       </c>
       <c r="AC18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AD18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1964,15 +2017,18 @@
       <c r="Z19" s="36">
         <f>Z18-Z17</f>
       </c>
-      <c r="AA19" s="37">
+      <c r="AA19" s="36">
         <f>AA18-AA17</f>
       </c>
-      <c r="AB19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AB19" s="37">
+        <f>AB18-AB17</f>
       </c>
       <c r="AC19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AD19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2059,15 +2115,18 @@
       <c r="Z20" s="36">
         <v>7</v>
       </c>
-      <c r="AA20" s="37">
-        <v>4</v>
-      </c>
-      <c r="AB20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AA20" s="36">
+        <v>4</v>
+      </c>
+      <c r="AB20" s="37">
+        <v>5</v>
       </c>
       <c r="AC20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AD20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-28 (foto de 29/10 07:26 reconstruindo o dia 28)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -297,13 +297,14 @@
     <col min="26" max="26" width="10" customWidth="1"/>
     <col min="27" max="27" width="10" customWidth="1"/>
     <col min="28" max="28" width="10" customWidth="1"/>
-    <col min="29" max="29" width="12" customWidth="1"/>
+    <col min="29" max="29" width="10" customWidth="1"/>
+    <col min="30" max="30" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 27/10 · variação 26/10 → 27/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 28/10 · variação 27/10 → 28/10</t>
         </is>
       </c>
     </row>
@@ -451,10 +452,15 @@
       </c>
       <c r="AC3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">28/10</t>
+        </is>
+      </c>
+      <c r="AD3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="AD3" s="1" t="inlineStr">
+      <c r="AE3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -544,14 +550,17 @@
       <c r="AA4" s="36">
         <v>32</v>
       </c>
-      <c r="AB4" s="37">
+      <c r="AB4" s="36">
         <v>32</v>
       </c>
-      <c r="AC4" s="36">
-        <f>AB4-AA4</f>
+      <c r="AC4" s="37">
+        <v>28</v>
       </c>
       <c r="AD4" s="35">
-        <f>AB4-B4</f>
+        <f>AC4-AB4</f>
+      </c>
+      <c r="AE4" s="35">
+        <f>AC4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -638,14 +647,17 @@
       <c r="AA5" s="36">
         <v>13</v>
       </c>
-      <c r="AB5" s="37">
+      <c r="AB5" s="36">
         <v>14</v>
       </c>
-      <c r="AC5" s="34">
-        <f>AB5-AA5</f>
-      </c>
-      <c r="AD5" s="35">
-        <f>AB5-B5</f>
+      <c r="AC5" s="37">
+        <v>17</v>
+      </c>
+      <c r="AD5" s="34">
+        <f>AC5-AB5</f>
+      </c>
+      <c r="AE5" s="35">
+        <f>AC5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -732,257 +744,266 @@
       <c r="AA6" s="36">
         <v>5</v>
       </c>
-      <c r="AB6" s="37">
+      <c r="AB6" s="36">
         <v>8</v>
       </c>
-      <c r="AC6" s="34">
-        <f>AB6-AA6</f>
-      </c>
-      <c r="AD6" s="35">
-        <f>AB6-B6</f>
+      <c r="AC6" s="37">
+        <v>10</v>
+      </c>
+      <c r="AD6" s="34">
+        <f>AC6-AB6</f>
+      </c>
+      <c r="AE6" s="35">
+        <f>AC6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C7" s="36">
+        <v>22</v>
+      </c>
+      <c r="D7" s="36">
+        <v>22</v>
+      </c>
+      <c r="E7" s="36">
+        <v>22</v>
+      </c>
+      <c r="F7" s="36">
+        <v>23</v>
+      </c>
+      <c r="G7" s="36">
+        <v>25</v>
+      </c>
+      <c r="H7" s="36">
+        <v>24</v>
+      </c>
+      <c r="I7" s="36">
+        <v>28</v>
+      </c>
+      <c r="J7" s="36">
+        <v>30</v>
+      </c>
+      <c r="K7" s="36">
+        <v>31</v>
+      </c>
+      <c r="L7" s="36">
+        <v>26</v>
+      </c>
+      <c r="M7" s="36">
+        <v>24</v>
+      </c>
+      <c r="N7" s="36">
         <v>11</v>
       </c>
-      <c r="D7" s="36">
+      <c r="O7" s="36">
+        <v>8</v>
+      </c>
+      <c r="P7" s="36">
         <v>10</v>
       </c>
-      <c r="E7" s="36">
-        <v>10</v>
-      </c>
-      <c r="F7" s="36">
-        <v>12</v>
-      </c>
-      <c r="G7" s="36">
-        <v>11</v>
-      </c>
-      <c r="H7" s="36">
-        <v>12</v>
-      </c>
-      <c r="I7" s="36">
-        <v>7</v>
-      </c>
-      <c r="J7" s="36">
+      <c r="Q7" s="36">
+        <v>7</v>
+      </c>
+      <c r="R7" s="36">
+        <v>5</v>
+      </c>
+      <c r="S7" s="36">
         <v>6</v>
       </c>
-      <c r="K7" s="36">
-        <v>7</v>
-      </c>
-      <c r="L7" s="36">
-        <v>7</v>
-      </c>
-      <c r="M7" s="36">
-        <v>7</v>
-      </c>
-      <c r="N7" s="36">
-        <v>10</v>
-      </c>
-      <c r="O7" s="36">
-        <v>7</v>
-      </c>
-      <c r="P7" s="36">
+      <c r="T7" s="36">
+        <v>6</v>
+      </c>
+      <c r="U7" s="36">
+        <v>6</v>
+      </c>
+      <c r="V7" s="36">
+        <v>7</v>
+      </c>
+      <c r="W7" s="36">
+        <v>2</v>
+      </c>
+      <c r="X7" s="36">
+        <v>4</v>
+      </c>
+      <c r="Y7" s="36">
+        <v>2</v>
+      </c>
+      <c r="Z7" s="36">
+        <v>5</v>
+      </c>
+      <c r="AA7" s="36">
+        <v>7</v>
+      </c>
+      <c r="AB7" s="36">
+        <v>4</v>
+      </c>
+      <c r="AC7" s="37">
         <v>8</v>
       </c>
-      <c r="Q7" s="36">
-        <v>6</v>
-      </c>
-      <c r="R7" s="36">
-        <v>6</v>
-      </c>
-      <c r="S7" s="36">
-        <v>5</v>
-      </c>
-      <c r="T7" s="36">
-        <v>8</v>
-      </c>
-      <c r="U7" s="36">
-        <v>11</v>
-      </c>
-      <c r="V7" s="36">
-        <v>8</v>
-      </c>
-      <c r="W7" s="36">
-        <v>4</v>
-      </c>
-      <c r="X7" s="36">
-        <v>5</v>
-      </c>
-      <c r="Y7" s="36">
-        <v>6</v>
-      </c>
-      <c r="Z7" s="36">
-        <v>5</v>
-      </c>
-      <c r="AA7" s="36">
-        <v>4</v>
-      </c>
-      <c r="AB7" s="37">
-        <v>6</v>
-      </c>
-      <c r="AC7" s="34">
-        <f>AB7-AA7</f>
-      </c>
-      <c r="AD7" s="35">
-        <f>AB7-B7</f>
+      <c r="AD7" s="34">
+        <f>AC7-AB7</f>
+      </c>
+      <c r="AE7" s="35">
+        <f>AC7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B8" s="36">
+        <v>12</v>
+      </c>
+      <c r="C8" s="36">
         <v>11</v>
       </c>
-      <c r="C8" s="36">
+      <c r="D8" s="36">
         <v>10</v>
       </c>
-      <c r="D8" s="36">
-        <v>9</v>
-      </c>
       <c r="E8" s="36">
+        <v>10</v>
+      </c>
+      <c r="F8" s="36">
+        <v>12</v>
+      </c>
+      <c r="G8" s="36">
+        <v>11</v>
+      </c>
+      <c r="H8" s="36">
+        <v>12</v>
+      </c>
+      <c r="I8" s="36">
+        <v>7</v>
+      </c>
+      <c r="J8" s="36">
         <v>6</v>
       </c>
-      <c r="F8" s="36">
-        <v>5</v>
-      </c>
-      <c r="G8" s="36">
-        <v>5</v>
-      </c>
-      <c r="H8" s="36">
-        <v>5</v>
-      </c>
-      <c r="I8" s="36">
+      <c r="K8" s="36">
+        <v>7</v>
+      </c>
+      <c r="L8" s="36">
+        <v>7</v>
+      </c>
+      <c r="M8" s="36">
+        <v>7</v>
+      </c>
+      <c r="N8" s="36">
+        <v>10</v>
+      </c>
+      <c r="O8" s="36">
+        <v>7</v>
+      </c>
+      <c r="P8" s="36">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="36">
         <v>6</v>
       </c>
-      <c r="J8" s="36">
-        <v>5</v>
-      </c>
-      <c r="K8" s="36">
-        <v>4</v>
-      </c>
-      <c r="L8" s="36">
-        <v>4</v>
-      </c>
-      <c r="M8" s="36">
-        <v>5</v>
-      </c>
-      <c r="N8" s="36">
+      <c r="R8" s="36">
+        <v>6</v>
+      </c>
+      <c r="S8" s="36">
+        <v>5</v>
+      </c>
+      <c r="T8" s="36">
         <v>8</v>
       </c>
-      <c r="O8" s="36">
+      <c r="U8" s="36">
+        <v>11</v>
+      </c>
+      <c r="V8" s="36">
+        <v>8</v>
+      </c>
+      <c r="W8" s="36">
+        <v>4</v>
+      </c>
+      <c r="X8" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y8" s="36">
         <v>6</v>
       </c>
-      <c r="P8" s="36">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="36">
-        <v>5</v>
-      </c>
-      <c r="R8" s="36">
-        <v>5</v>
-      </c>
-      <c r="S8" s="36">
+      <c r="Z8" s="36">
+        <v>5</v>
+      </c>
+      <c r="AA8" s="36">
+        <v>4</v>
+      </c>
+      <c r="AB8" s="36">
         <v>6</v>
       </c>
-      <c r="T8" s="36">
-        <v>5</v>
-      </c>
-      <c r="U8" s="36">
-        <v>3</v>
-      </c>
-      <c r="V8" s="36">
-        <v>3</v>
-      </c>
-      <c r="W8" s="36">
-        <v>3</v>
-      </c>
-      <c r="X8" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y8" s="36">
-        <v>4</v>
-      </c>
-      <c r="Z8" s="36">
-        <v>4</v>
-      </c>
-      <c r="AA8" s="36">
-        <v>3</v>
-      </c>
-      <c r="AB8" s="37">
-        <v>5</v>
-      </c>
-      <c r="AC8" s="34">
-        <f>AB8-AA8</f>
-      </c>
-      <c r="AD8" s="35">
-        <f>AB8-B8</f>
+      <c r="AC8" s="37">
+        <v>6</v>
+      </c>
+      <c r="AD8" s="36">
+        <f>AC8-AB8</f>
+      </c>
+      <c r="AE8" s="35">
+        <f>AC8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="C9" s="36">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="D9" s="36">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="E9" s="36">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="F9" s="36">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="G9" s="36">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="H9" s="36">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="I9" s="36">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="J9" s="36">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K9" s="36">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="L9" s="36">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="M9" s="36">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="N9" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O9" s="36">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P9" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R9" s="36">
         <v>5</v>
@@ -991,37 +1012,40 @@
         <v>6</v>
       </c>
       <c r="T9" s="36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U9" s="36">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V9" s="36">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="W9" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X9" s="36">
         <v>4</v>
       </c>
       <c r="Y9" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Z9" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA9" s="36">
-        <v>7</v>
-      </c>
-      <c r="AB9" s="37">
-        <v>4</v>
-      </c>
-      <c r="AC9" s="35">
-        <f>AB9-AA9</f>
-      </c>
-      <c r="AD9" s="35">
-        <f>AB9-B9</f>
+        <v>3</v>
+      </c>
+      <c r="AB9" s="36">
+        <v>5</v>
+      </c>
+      <c r="AC9" s="37">
+        <v>5</v>
+      </c>
+      <c r="AD9" s="36">
+        <f>AC9-AB9</f>
+      </c>
+      <c r="AE9" s="35">
+        <f>AC9-B9</f>
       </c>
     </row>
     <row r="10">
@@ -1108,390 +1132,405 @@
       <c r="AA10" s="36">
         <v>9</v>
       </c>
-      <c r="AB10" s="37">
+      <c r="AB10" s="36">
         <v>3</v>
       </c>
-      <c r="AC10" s="35">
-        <f>AB10-AA10</f>
-      </c>
-      <c r="AD10" s="35">
-        <f>AB10-B10</f>
+      <c r="AC10" s="37">
+        <v>4</v>
+      </c>
+      <c r="AD10" s="34">
+        <f>AC10-AB10</f>
+      </c>
+      <c r="AE10" s="35">
+        <f>AC10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C11" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D11" s="36">
+        <v>9</v>
+      </c>
+      <c r="E11" s="36">
+        <v>12</v>
+      </c>
+      <c r="F11" s="36">
+        <v>13</v>
+      </c>
+      <c r="G11" s="36">
+        <v>9</v>
+      </c>
+      <c r="H11" s="36">
+        <v>11</v>
+      </c>
+      <c r="I11" s="36">
+        <v>7</v>
+      </c>
+      <c r="J11" s="36">
+        <v>6</v>
+      </c>
+      <c r="K11" s="36">
+        <v>6</v>
+      </c>
+      <c r="L11" s="36">
+        <v>7</v>
+      </c>
+      <c r="M11" s="36">
+        <v>7</v>
+      </c>
+      <c r="N11" s="36">
+        <v>13</v>
+      </c>
+      <c r="O11" s="36">
+        <v>13</v>
+      </c>
+      <c r="P11" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q11" s="36">
+        <v>10</v>
+      </c>
+      <c r="R11" s="36">
+        <v>13</v>
+      </c>
+      <c r="S11" s="36">
+        <v>10</v>
+      </c>
+      <c r="T11" s="36">
+        <v>10</v>
+      </c>
+      <c r="U11" s="36">
+        <v>7</v>
+      </c>
+      <c r="V11" s="36">
+        <v>6</v>
+      </c>
+      <c r="W11" s="36">
+        <v>5</v>
+      </c>
+      <c r="X11" s="36">
         <v>3</v>
       </c>
-      <c r="E11" s="36">
+      <c r="Y11" s="36">
         <v>3</v>
       </c>
-      <c r="F11" s="36">
+      <c r="Z11" s="36">
         <v>2</v>
-      </c>
-      <c r="G11" s="36">
-        <v>4</v>
-      </c>
-      <c r="H11" s="36">
-        <v>2</v>
-      </c>
-      <c r="I11" s="36">
-        <v>4</v>
-      </c>
-      <c r="J11" s="36">
-        <v>3</v>
-      </c>
-      <c r="K11" s="36">
-        <v>0</v>
-      </c>
-      <c r="L11" s="36">
-        <v>0</v>
-      </c>
-      <c r="M11" s="36">
-        <v>0</v>
-      </c>
-      <c r="N11" s="36">
-        <v>1</v>
-      </c>
-      <c r="O11" s="36">
-        <v>3</v>
-      </c>
-      <c r="P11" s="36">
-        <v>2</v>
-      </c>
-      <c r="Q11" s="36">
-        <v>2</v>
-      </c>
-      <c r="R11" s="36">
-        <v>2</v>
-      </c>
-      <c r="S11" s="36">
-        <v>3</v>
-      </c>
-      <c r="T11" s="36">
-        <v>2</v>
-      </c>
-      <c r="U11" s="36">
-        <v>4</v>
-      </c>
-      <c r="V11" s="36">
-        <v>4</v>
-      </c>
-      <c r="W11" s="36">
-        <v>3</v>
-      </c>
-      <c r="X11" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y11" s="36">
-        <v>4</v>
-      </c>
-      <c r="Z11" s="36">
-        <v>3</v>
       </c>
       <c r="AA11" s="36">
         <v>2</v>
       </c>
-      <c r="AB11" s="37">
+      <c r="AB11" s="36">
         <v>2</v>
       </c>
-      <c r="AC11" s="36">
-        <f>AB11-AA11</f>
-      </c>
-      <c r="AD11" s="35">
-        <f>AB11-B11</f>
+      <c r="AC11" s="37">
+        <v>3</v>
+      </c>
+      <c r="AD11" s="34">
+        <f>AC11-AB11</f>
+      </c>
+      <c r="AE11" s="35">
+        <f>AC11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C12" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D12" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E12" s="36">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F12" s="36">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="G12" s="36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H12" s="36">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="I12" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J12" s="36">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K12" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L12" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M12" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N12" s="36">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="O12" s="36">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P12" s="36">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="36">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="R12" s="36">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="S12" s="36">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="T12" s="36">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="U12" s="36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V12" s="36">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W12" s="36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="X12" s="36">
+        <v>4</v>
+      </c>
+      <c r="Y12" s="36">
+        <v>4</v>
+      </c>
+      <c r="Z12" s="36">
         <v>3</v>
-      </c>
-      <c r="Y12" s="36">
-        <v>3</v>
-      </c>
-      <c r="Z12" s="36">
-        <v>2</v>
       </c>
       <c r="AA12" s="36">
         <v>2</v>
       </c>
-      <c r="AB12" s="37">
+      <c r="AB12" s="36">
         <v>2</v>
       </c>
-      <c r="AC12" s="36">
-        <f>AB12-AA12</f>
+      <c r="AC12" s="37">
+        <v>1</v>
       </c>
       <c r="AD12" s="35">
-        <f>AB12-B12</f>
+        <f>AC12-AB12</f>
+      </c>
+      <c r="AE12" s="35">
+        <f>AC12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B13" s="36">
+        <v>18</v>
+      </c>
+      <c r="C13" s="36">
+        <v>16</v>
+      </c>
+      <c r="D13" s="36">
+        <v>20</v>
+      </c>
+      <c r="E13" s="36">
+        <v>22</v>
+      </c>
+      <c r="F13" s="36">
+        <v>23</v>
+      </c>
+      <c r="G13" s="36">
+        <v>20</v>
+      </c>
+      <c r="H13" s="36">
+        <v>18</v>
+      </c>
+      <c r="I13" s="36">
+        <v>18</v>
+      </c>
+      <c r="J13" s="36">
+        <v>19</v>
+      </c>
+      <c r="K13" s="36">
+        <v>17</v>
+      </c>
+      <c r="L13" s="36">
+        <v>13</v>
+      </c>
+      <c r="M13" s="36">
+        <v>14</v>
+      </c>
+      <c r="N13" s="36">
+        <v>9</v>
+      </c>
+      <c r="O13" s="36">
+        <v>9</v>
+      </c>
+      <c r="P13" s="36">
+        <v>7</v>
+      </c>
+      <c r="Q13" s="36">
+        <v>6</v>
+      </c>
+      <c r="R13" s="36">
+        <v>5</v>
+      </c>
+      <c r="S13" s="36">
+        <v>7</v>
+      </c>
+      <c r="T13" s="36">
         <v>8</v>
       </c>
-      <c r="C13" s="36">
-        <v>7</v>
-      </c>
-      <c r="D13" s="36">
-        <v>9</v>
-      </c>
-      <c r="E13" s="36">
-        <v>14</v>
-      </c>
-      <c r="F13" s="36">
-        <v>7</v>
-      </c>
-      <c r="G13" s="36">
-        <v>6</v>
-      </c>
-      <c r="H13" s="36">
+      <c r="U13" s="36">
         <v>8</v>
       </c>
-      <c r="I13" s="36">
-        <v>11</v>
-      </c>
-      <c r="J13" s="36">
-        <v>11</v>
-      </c>
-      <c r="K13" s="36">
-        <v>12</v>
-      </c>
-      <c r="L13" s="36">
-        <v>4</v>
-      </c>
-      <c r="M13" s="36">
-        <v>4</v>
-      </c>
-      <c r="N13" s="36">
+      <c r="V13" s="36">
+        <v>3</v>
+      </c>
+      <c r="W13" s="36">
+        <v>4</v>
+      </c>
+      <c r="X13" s="36">
         <v>2</v>
       </c>
-      <c r="O13" s="36">
-        <v>3</v>
-      </c>
-      <c r="P13" s="36">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="36">
-        <v>2</v>
-      </c>
-      <c r="R13" s="36">
-        <v>1</v>
-      </c>
-      <c r="S13" s="36">
-        <v>1</v>
-      </c>
-      <c r="T13" s="36">
-        <v>1</v>
-      </c>
-      <c r="U13" s="36">
-        <v>1</v>
-      </c>
-      <c r="V13" s="36">
-        <v>4</v>
-      </c>
-      <c r="W13" s="36">
-        <v>2</v>
-      </c>
-      <c r="X13" s="36">
-        <v>0</v>
-      </c>
       <c r="Y13" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="36">
         <v>2</v>
       </c>
-      <c r="AB13" s="37">
+      <c r="AB13" s="36">
         <v>1</v>
       </c>
-      <c r="AC13" s="35">
-        <f>AB13-AA13</f>
-      </c>
-      <c r="AD13" s="35">
-        <f>AB13-B13</f>
+      <c r="AC13" s="37">
+        <v>1</v>
+      </c>
+      <c r="AD13" s="36">
+        <f>AC13-AB13</f>
+      </c>
+      <c r="AE13" s="35">
+        <f>AC13-B13</f>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B14" s="36">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C14" s="36">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D14" s="36">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E14" s="36">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F14" s="36">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="G14" s="36">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H14" s="36">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="I14" s="36">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="J14" s="36">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="K14" s="36">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="L14" s="36">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M14" s="36">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="N14" s="36">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O14" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="P14" s="36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R14" s="36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S14" s="36">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="T14" s="36">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="U14" s="36">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="V14" s="36">
+        <v>4</v>
+      </c>
+      <c r="W14" s="36">
+        <v>2</v>
+      </c>
+      <c r="X14" s="36">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="36">
         <v>3</v>
       </c>
-      <c r="W14" s="36">
-        <v>4</v>
-      </c>
-      <c r="X14" s="36">
-        <v>2</v>
-      </c>
-      <c r="Y14" s="36">
-        <v>0</v>
-      </c>
       <c r="Z14" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA14" s="36">
         <v>2</v>
       </c>
-      <c r="AB14" s="37">
+      <c r="AB14" s="36">
         <v>1</v>
       </c>
-      <c r="AC14" s="35">
-        <f>AB14-AA14</f>
+      <c r="AC14" s="37">
+        <v>0</v>
       </c>
       <c r="AD14" s="35">
-        <f>AB14-B14</f>
+        <f>AC14-AB14</f>
+      </c>
+      <c r="AE14" s="35">
+        <f>AC14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1581,11 +1620,14 @@
       <c r="AB15" s="38">
         <f>SUM(AB4:AB14)</f>
       </c>
-      <c r="AC15" s="41">
-        <f>AB15-AA15</f>
-      </c>
-      <c r="AD15" s="41">
-        <f>AB15-B15</f>
+      <c r="AC15" s="38">
+        <f>SUM(AC4:AC14)</f>
+      </c>
+      <c r="AD15" s="40">
+        <f>AC15-AB15</f>
+      </c>
+      <c r="AE15" s="41">
+        <f>AC15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1739,6 +1781,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="AE16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1824,15 +1871,18 @@
       <c r="AA17" s="36">
         <v>35</v>
       </c>
-      <c r="AB17" s="37">
+      <c r="AB17" s="36">
         <v>33</v>
       </c>
-      <c r="AC17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AC17" s="37">
+        <v>14</v>
       </c>
       <c r="AD17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AE17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1922,15 +1972,18 @@
       <c r="AA18" s="36">
         <v>30</v>
       </c>
-      <c r="AB18" s="37">
+      <c r="AB18" s="36">
         <v>30</v>
       </c>
-      <c r="AC18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AC18" s="37">
+        <v>19</v>
       </c>
       <c r="AD18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AE18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2020,15 +2073,18 @@
       <c r="AA19" s="36">
         <f>AA18-AA17</f>
       </c>
-      <c r="AB19" s="37">
+      <c r="AB19" s="36">
         <f>AB18-AB17</f>
       </c>
-      <c r="AC19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AC19" s="37">
+        <f>AC18-AC17</f>
       </c>
       <c r="AD19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AE19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2118,15 +2174,18 @@
       <c r="AA20" s="36">
         <v>4</v>
       </c>
-      <c r="AB20" s="37">
-        <v>5</v>
-      </c>
-      <c r="AC20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AB20" s="36">
+        <v>5</v>
+      </c>
+      <c r="AC20" s="37">
+        <v>7</v>
       </c>
       <c r="AD20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AE20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-29 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -298,13 +298,14 @@
     <col min="27" max="27" width="10" customWidth="1"/>
     <col min="28" max="28" width="10" customWidth="1"/>
     <col min="29" max="29" width="10" customWidth="1"/>
-    <col min="30" max="30" width="12" customWidth="1"/>
+    <col min="30" max="30" width="10" customWidth="1"/>
+    <col min="31" max="31" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 28/10 · variação 27/10 → 28/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 29/10 · variação 28/10 → 29/10</t>
         </is>
       </c>
     </row>
@@ -457,10 +458,15 @@
       </c>
       <c r="AD3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">29/10</t>
+        </is>
+      </c>
+      <c r="AE3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="AE3" s="1" t="inlineStr">
+      <c r="AF3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -553,14 +559,17 @@
       <c r="AB4" s="36">
         <v>32</v>
       </c>
-      <c r="AC4" s="37">
+      <c r="AC4" s="36">
         <v>28</v>
       </c>
-      <c r="AD4" s="35">
-        <f>AC4-AB4</f>
+      <c r="AD4" s="37">
+        <v>23</v>
       </c>
       <c r="AE4" s="35">
-        <f>AC4-B4</f>
+        <f>AD4-AC4</f>
+      </c>
+      <c r="AF4" s="35">
+        <f>AD4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -650,14 +659,17 @@
       <c r="AB5" s="36">
         <v>14</v>
       </c>
-      <c r="AC5" s="37">
+      <c r="AC5" s="36">
         <v>17</v>
       </c>
-      <c r="AD5" s="34">
-        <f>AC5-AB5</f>
+      <c r="AD5" s="37">
+        <v>14</v>
       </c>
       <c r="AE5" s="35">
-        <f>AC5-B5</f>
+        <f>AD5-AC5</f>
+      </c>
+      <c r="AF5" s="35">
+        <f>AD5-B5</f>
       </c>
     </row>
     <row r="6">
@@ -747,14 +759,17 @@
       <c r="AB6" s="36">
         <v>8</v>
       </c>
-      <c r="AC6" s="37">
+      <c r="AC6" s="36">
         <v>10</v>
       </c>
-      <c r="AD6" s="34">
-        <f>AC6-AB6</f>
+      <c r="AD6" s="37">
+        <v>9</v>
       </c>
       <c r="AE6" s="35">
-        <f>AC6-B6</f>
+        <f>AD6-AC6</f>
+      </c>
+      <c r="AF6" s="35">
+        <f>AD6-B6</f>
       </c>
     </row>
     <row r="7">
@@ -844,208 +859,217 @@
       <c r="AB7" s="36">
         <v>4</v>
       </c>
-      <c r="AC7" s="37">
+      <c r="AC7" s="36">
         <v>8</v>
       </c>
-      <c r="AD7" s="34">
-        <f>AC7-AB7</f>
+      <c r="AD7" s="37">
+        <v>7</v>
       </c>
       <c r="AE7" s="35">
-        <f>AC7-B7</f>
+        <f>AD7-AC7</f>
+      </c>
+      <c r="AF7" s="35">
+        <f>AD7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="36">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="36">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F8" s="36">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G8" s="36">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H8" s="36">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I8" s="36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J8" s="36">
+        <v>5</v>
+      </c>
+      <c r="K8" s="36">
+        <v>4</v>
+      </c>
+      <c r="L8" s="36">
+        <v>4</v>
+      </c>
+      <c r="M8" s="36">
+        <v>5</v>
+      </c>
+      <c r="N8" s="36">
+        <v>8</v>
+      </c>
+      <c r="O8" s="36">
         <v>6</v>
       </c>
-      <c r="K8" s="36">
-        <v>7</v>
-      </c>
-      <c r="L8" s="36">
-        <v>7</v>
-      </c>
-      <c r="M8" s="36">
-        <v>7</v>
-      </c>
-      <c r="N8" s="36">
-        <v>10</v>
-      </c>
-      <c r="O8" s="36">
-        <v>7</v>
-      </c>
       <c r="P8" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="36">
+        <v>5</v>
+      </c>
+      <c r="R8" s="36">
+        <v>5</v>
+      </c>
+      <c r="S8" s="36">
         <v>6</v>
       </c>
-      <c r="R8" s="36">
-        <v>6</v>
-      </c>
-      <c r="S8" s="36">
-        <v>5</v>
-      </c>
       <c r="T8" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U8" s="36">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="V8" s="36">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="W8" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X8" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Y8" s="36">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Z8" s="36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA8" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AB8" s="36">
-        <v>6</v>
-      </c>
-      <c r="AC8" s="37">
-        <v>6</v>
-      </c>
-      <c r="AD8" s="36">
-        <f>AC8-AB8</f>
-      </c>
-      <c r="AE8" s="35">
-        <f>AC8-B8</f>
+        <v>5</v>
+      </c>
+      <c r="AC8" s="36">
+        <v>5</v>
+      </c>
+      <c r="AD8" s="37">
+        <v>5</v>
+      </c>
+      <c r="AE8" s="36">
+        <f>AD8-AC8</f>
+      </c>
+      <c r="AF8" s="35">
+        <f>AD8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B9" s="36">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C9" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D9" s="36">
         <v>9</v>
       </c>
       <c r="E9" s="36">
+        <v>12</v>
+      </c>
+      <c r="F9" s="36">
+        <v>13</v>
+      </c>
+      <c r="G9" s="36">
+        <v>9</v>
+      </c>
+      <c r="H9" s="36">
+        <v>11</v>
+      </c>
+      <c r="I9" s="36">
+        <v>7</v>
+      </c>
+      <c r="J9" s="36">
         <v>6</v>
       </c>
-      <c r="F9" s="36">
-        <v>5</v>
-      </c>
-      <c r="G9" s="36">
-        <v>5</v>
-      </c>
-      <c r="H9" s="36">
-        <v>5</v>
-      </c>
-      <c r="I9" s="36">
+      <c r="K9" s="36">
         <v>6</v>
       </c>
-      <c r="J9" s="36">
-        <v>5</v>
-      </c>
-      <c r="K9" s="36">
-        <v>4</v>
-      </c>
       <c r="L9" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M9" s="36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N9" s="36">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="O9" s="36">
+        <v>13</v>
+      </c>
+      <c r="P9" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q9" s="36">
+        <v>10</v>
+      </c>
+      <c r="R9" s="36">
+        <v>13</v>
+      </c>
+      <c r="S9" s="36">
+        <v>10</v>
+      </c>
+      <c r="T9" s="36">
+        <v>10</v>
+      </c>
+      <c r="U9" s="36">
+        <v>7</v>
+      </c>
+      <c r="V9" s="36">
         <v>6</v>
       </c>
-      <c r="P9" s="36">
-        <v>5</v>
-      </c>
-      <c r="Q9" s="36">
-        <v>5</v>
-      </c>
-      <c r="R9" s="36">
-        <v>5</v>
-      </c>
-      <c r="S9" s="36">
-        <v>6</v>
-      </c>
-      <c r="T9" s="36">
-        <v>5</v>
-      </c>
-      <c r="U9" s="36">
+      <c r="W9" s="36">
+        <v>5</v>
+      </c>
+      <c r="X9" s="36">
         <v>3</v>
       </c>
-      <c r="V9" s="36">
+      <c r="Y9" s="36">
         <v>3</v>
       </c>
-      <c r="W9" s="36">
+      <c r="Z9" s="36">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="36">
+        <v>2</v>
+      </c>
+      <c r="AB9" s="36">
+        <v>2</v>
+      </c>
+      <c r="AC9" s="36">
         <v>3</v>
       </c>
-      <c r="X9" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y9" s="36">
-        <v>4</v>
-      </c>
-      <c r="Z9" s="36">
-        <v>4</v>
-      </c>
-      <c r="AA9" s="36">
-        <v>3</v>
-      </c>
-      <c r="AB9" s="36">
-        <v>5</v>
-      </c>
-      <c r="AC9" s="37">
-        <v>5</v>
-      </c>
-      <c r="AD9" s="36">
-        <f>AC9-AB9</f>
-      </c>
-      <c r="AE9" s="35">
-        <f>AC9-B9</f>
+      <c r="AD9" s="37">
+        <v>4</v>
+      </c>
+      <c r="AE9" s="34">
+        <f>AD9-AC9</f>
+      </c>
+      <c r="AF9" s="35">
+        <f>AD9-B9</f>
       </c>
     </row>
     <row r="10">
@@ -1135,42 +1159,45 @@
       <c r="AB10" s="36">
         <v>3</v>
       </c>
-      <c r="AC10" s="37">
-        <v>4</v>
-      </c>
-      <c r="AD10" s="34">
-        <f>AC10-AB10</f>
+      <c r="AC10" s="36">
+        <v>4</v>
+      </c>
+      <c r="AD10" s="37">
+        <v>3</v>
       </c>
       <c r="AE10" s="35">
-        <f>AC10-B10</f>
+        <f>AD10-AC10</f>
+      </c>
+      <c r="AF10" s="35">
+        <f>AD10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C11" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D11" s="36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11" s="36">
+        <v>10</v>
+      </c>
+      <c r="F11" s="36">
         <v>12</v>
       </c>
-      <c r="F11" s="36">
-        <v>13</v>
-      </c>
       <c r="G11" s="36">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H11" s="36">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I11" s="36">
         <v>7</v>
@@ -1179,261 +1206,270 @@
         <v>6</v>
       </c>
       <c r="K11" s="36">
+        <v>7</v>
+      </c>
+      <c r="L11" s="36">
+        <v>7</v>
+      </c>
+      <c r="M11" s="36">
+        <v>7</v>
+      </c>
+      <c r="N11" s="36">
+        <v>10</v>
+      </c>
+      <c r="O11" s="36">
+        <v>7</v>
+      </c>
+      <c r="P11" s="36">
+        <v>8</v>
+      </c>
+      <c r="Q11" s="36">
         <v>6</v>
       </c>
-      <c r="L11" s="36">
-        <v>7</v>
-      </c>
-      <c r="M11" s="36">
-        <v>7</v>
-      </c>
-      <c r="N11" s="36">
-        <v>13</v>
-      </c>
-      <c r="O11" s="36">
-        <v>13</v>
-      </c>
-      <c r="P11" s="36">
-        <v>13</v>
-      </c>
-      <c r="Q11" s="36">
-        <v>10</v>
-      </c>
       <c r="R11" s="36">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="S11" s="36">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T11" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U11" s="36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="V11" s="36">
+        <v>8</v>
+      </c>
+      <c r="W11" s="36">
+        <v>4</v>
+      </c>
+      <c r="X11" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y11" s="36">
         <v>6</v>
       </c>
-      <c r="W11" s="36">
-        <v>5</v>
-      </c>
-      <c r="X11" s="36">
-        <v>3</v>
-      </c>
-      <c r="Y11" s="36">
-        <v>3</v>
-      </c>
       <c r="Z11" s="36">
+        <v>5</v>
+      </c>
+      <c r="AA11" s="36">
+        <v>4</v>
+      </c>
+      <c r="AB11" s="36">
+        <v>6</v>
+      </c>
+      <c r="AC11" s="36">
+        <v>6</v>
+      </c>
+      <c r="AD11" s="37">
         <v>2</v>
       </c>
-      <c r="AA11" s="36">
-        <v>2</v>
-      </c>
-      <c r="AB11" s="36">
-        <v>2</v>
-      </c>
-      <c r="AC11" s="37">
-        <v>3</v>
-      </c>
-      <c r="AD11" s="34">
-        <f>AC11-AB11</f>
-      </c>
       <c r="AE11" s="35">
-        <f>AC11-B11</f>
+        <f>AD11-AC11</f>
+      </c>
+      <c r="AF11" s="35">
+        <f>AD11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C12" s="36">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D12" s="36">
+        <v>20</v>
+      </c>
+      <c r="E12" s="36">
+        <v>22</v>
+      </c>
+      <c r="F12" s="36">
+        <v>23</v>
+      </c>
+      <c r="G12" s="36">
+        <v>20</v>
+      </c>
+      <c r="H12" s="36">
+        <v>18</v>
+      </c>
+      <c r="I12" s="36">
+        <v>18</v>
+      </c>
+      <c r="J12" s="36">
+        <v>19</v>
+      </c>
+      <c r="K12" s="36">
+        <v>17</v>
+      </c>
+      <c r="L12" s="36">
+        <v>13</v>
+      </c>
+      <c r="M12" s="36">
+        <v>14</v>
+      </c>
+      <c r="N12" s="36">
+        <v>9</v>
+      </c>
+      <c r="O12" s="36">
+        <v>9</v>
+      </c>
+      <c r="P12" s="36">
+        <v>7</v>
+      </c>
+      <c r="Q12" s="36">
+        <v>6</v>
+      </c>
+      <c r="R12" s="36">
+        <v>5</v>
+      </c>
+      <c r="S12" s="36">
+        <v>7</v>
+      </c>
+      <c r="T12" s="36">
+        <v>8</v>
+      </c>
+      <c r="U12" s="36">
+        <v>8</v>
+      </c>
+      <c r="V12" s="36">
         <v>3</v>
       </c>
-      <c r="E12" s="36">
-        <v>3</v>
-      </c>
-      <c r="F12" s="36">
+      <c r="W12" s="36">
+        <v>4</v>
+      </c>
+      <c r="X12" s="36">
         <v>2</v>
       </c>
-      <c r="G12" s="36">
-        <v>4</v>
-      </c>
-      <c r="H12" s="36">
-        <v>2</v>
-      </c>
-      <c r="I12" s="36">
-        <v>4</v>
-      </c>
-      <c r="J12" s="36">
-        <v>3</v>
-      </c>
-      <c r="K12" s="36">
-        <v>0</v>
-      </c>
-      <c r="L12" s="36">
-        <v>0</v>
-      </c>
-      <c r="M12" s="36">
-        <v>0</v>
-      </c>
-      <c r="N12" s="36">
-        <v>1</v>
-      </c>
-      <c r="O12" s="36">
-        <v>3</v>
-      </c>
-      <c r="P12" s="36">
-        <v>2</v>
-      </c>
-      <c r="Q12" s="36">
-        <v>2</v>
-      </c>
-      <c r="R12" s="36">
-        <v>2</v>
-      </c>
-      <c r="S12" s="36">
-        <v>3</v>
-      </c>
-      <c r="T12" s="36">
-        <v>2</v>
-      </c>
-      <c r="U12" s="36">
-        <v>4</v>
-      </c>
-      <c r="V12" s="36">
-        <v>4</v>
-      </c>
-      <c r="W12" s="36">
-        <v>3</v>
-      </c>
-      <c r="X12" s="36">
-        <v>4</v>
-      </c>
       <c r="Y12" s="36">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="36">
         <v>2</v>
       </c>
       <c r="AB12" s="36">
+        <v>1</v>
+      </c>
+      <c r="AC12" s="36">
+        <v>1</v>
+      </c>
+      <c r="AD12" s="37">
         <v>2</v>
       </c>
-      <c r="AC12" s="37">
-        <v>1</v>
-      </c>
-      <c r="AD12" s="35">
-        <f>AC12-AB12</f>
-      </c>
-      <c r="AE12" s="35">
-        <f>AC12-B12</f>
+      <c r="AE12" s="34">
+        <f>AD12-AC12</f>
+      </c>
+      <c r="AF12" s="35">
+        <f>AD12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C13" s="36">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D13" s="36">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E13" s="36">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="F13" s="36">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G13" s="36">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="H13" s="36">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I13" s="36">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="J13" s="36">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="K13" s="36">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="L13" s="36">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="M13" s="36">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="N13" s="36">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O13" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="P13" s="36">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R13" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S13" s="36">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="T13" s="36">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="U13" s="36">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V13" s="36">
+        <v>4</v>
+      </c>
+      <c r="W13" s="36">
         <v>3</v>
       </c>
-      <c r="W13" s="36">
-        <v>4</v>
-      </c>
       <c r="X13" s="36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y13" s="36">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Z13" s="36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA13" s="36">
         <v>2</v>
       </c>
       <c r="AB13" s="36">
+        <v>2</v>
+      </c>
+      <c r="AC13" s="36">
         <v>1</v>
       </c>
-      <c r="AC13" s="37">
+      <c r="AD13" s="37">
         <v>1</v>
       </c>
-      <c r="AD13" s="36">
-        <f>AC13-AB13</f>
-      </c>
-      <c r="AE13" s="35">
-        <f>AC13-B13</f>
+      <c r="AE13" s="36">
+        <f>AD13-AC13</f>
+      </c>
+      <c r="AF13" s="35">
+        <f>AD13-B13</f>
       </c>
     </row>
     <row r="14">
@@ -1523,14 +1559,17 @@
       <c r="AB14" s="36">
         <v>1</v>
       </c>
-      <c r="AC14" s="37">
-        <v>0</v>
-      </c>
-      <c r="AD14" s="35">
-        <f>AC14-AB14</f>
-      </c>
-      <c r="AE14" s="35">
-        <f>AC14-B14</f>
+      <c r="AC14" s="36">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="37">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="36">
+        <f>AD14-AC14</f>
+      </c>
+      <c r="AF14" s="35">
+        <f>AD14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1623,11 +1662,14 @@
       <c r="AC15" s="38">
         <f>SUM(AC4:AC14)</f>
       </c>
-      <c r="AD15" s="40">
-        <f>AC15-AB15</f>
+      <c r="AD15" s="38">
+        <f>SUM(AD4:AD14)</f>
       </c>
       <c r="AE15" s="41">
-        <f>AC15-B15</f>
+        <f>AD15-AC15</f>
+      </c>
+      <c r="AF15" s="41">
+        <f>AD15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1786,6 +1828,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="AF16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1874,15 +1921,18 @@
       <c r="AB17" s="36">
         <v>33</v>
       </c>
-      <c r="AC17" s="37">
+      <c r="AC17" s="36">
         <v>14</v>
       </c>
-      <c r="AD17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AD17" s="37">
+        <v>39</v>
       </c>
       <c r="AE17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AF17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -1975,15 +2025,18 @@
       <c r="AB18" s="36">
         <v>30</v>
       </c>
-      <c r="AC18" s="37">
+      <c r="AC18" s="36">
         <v>19</v>
       </c>
-      <c r="AD18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AD18" s="37">
+        <v>26</v>
       </c>
       <c r="AE18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AF18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2076,15 +2129,18 @@
       <c r="AB19" s="36">
         <f>AB18-AB17</f>
       </c>
-      <c r="AC19" s="37">
+      <c r="AC19" s="36">
         <f>AC18-AC17</f>
       </c>
-      <c r="AD19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AD19" s="37">
+        <f>AD18-AD17</f>
       </c>
       <c r="AE19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AF19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2177,15 +2233,18 @@
       <c r="AB20" s="36">
         <v>5</v>
       </c>
-      <c r="AC20" s="37">
-        <v>7</v>
-      </c>
-      <c r="AD20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AC20" s="36">
+        <v>7</v>
+      </c>
+      <c r="AD20" s="37">
+        <v>6</v>
       </c>
       <c r="AE20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AF20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>

<commit_message>
Sorvete: evolucao ate 2026-10-30 (automatico)
</commit_message>
<xml_diff>
--- a/data/relatorio_sorvete.xlsx
+++ b/data/relatorio_sorvete.xlsx
@@ -299,13 +299,14 @@
     <col min="28" max="28" width="10" customWidth="1"/>
     <col min="29" max="29" width="10" customWidth="1"/>
     <col min="30" max="30" width="10" customWidth="1"/>
-    <col min="31" max="31" width="12" customWidth="1"/>
+    <col min="31" max="31" width="10" customWidth="1"/>
+    <col min="32" max="32" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 29/10 · variação 28/10 → 29/10</t>
+          <t xml:space="preserve">Evolução — chamados SOS e ALTO abertos, situação às 23:59 de cada dia · último dia fechado: 30/10 · variação 29/10 → 30/10</t>
         </is>
       </c>
     </row>
@@ -463,10 +464,15 @@
       </c>
       <c r="AE3" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">30/10</t>
+        </is>
+      </c>
+      <c r="AF3" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Variação DIA</t>
         </is>
       </c>
-      <c r="AF3" s="1" t="inlineStr">
+      <c r="AG3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Variação MÊS</t>
         </is>
@@ -562,14 +568,17 @@
       <c r="AC4" s="36">
         <v>28</v>
       </c>
-      <c r="AD4" s="37">
+      <c r="AD4" s="36">
         <v>23</v>
       </c>
-      <c r="AE4" s="35">
-        <f>AD4-AC4</f>
+      <c r="AE4" s="37">
+        <v>20</v>
       </c>
       <c r="AF4" s="35">
-        <f>AD4-B4</f>
+        <f>AE4-AD4</f>
+      </c>
+      <c r="AG4" s="35">
+        <f>AE4-B4</f>
       </c>
     </row>
     <row r="5">
@@ -662,793 +671,817 @@
       <c r="AC5" s="36">
         <v>17</v>
       </c>
-      <c r="AD5" s="37">
+      <c r="AD5" s="36">
         <v>14</v>
       </c>
-      <c r="AE5" s="35">
-        <f>AD5-AC5</f>
-      </c>
-      <c r="AF5" s="35">
-        <f>AD5-B5</f>
+      <c r="AE5" s="37">
+        <v>15</v>
+      </c>
+      <c r="AF5" s="34">
+        <f>AE5-AD5</f>
+      </c>
+      <c r="AG5" s="35">
+        <f>AE5-B5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUL</t>
+          <t xml:space="preserve">MINAS BAHIA</t>
         </is>
       </c>
       <c r="B6" s="36">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C6" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D6" s="36">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="E6" s="36">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F6" s="36">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G6" s="36">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H6" s="36">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I6" s="36">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J6" s="36">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K6" s="36">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="L6" s="36">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="M6" s="36">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N6" s="36">
         <v>11</v>
       </c>
       <c r="O6" s="36">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P6" s="36">
         <v>10</v>
       </c>
       <c r="Q6" s="36">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R6" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S6" s="36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T6" s="36">
+        <v>6</v>
+      </c>
+      <c r="U6" s="36">
+        <v>6</v>
+      </c>
+      <c r="V6" s="36">
+        <v>7</v>
+      </c>
+      <c r="W6" s="36">
+        <v>2</v>
+      </c>
+      <c r="X6" s="36">
+        <v>4</v>
+      </c>
+      <c r="Y6" s="36">
+        <v>2</v>
+      </c>
+      <c r="Z6" s="36">
+        <v>5</v>
+      </c>
+      <c r="AA6" s="36">
+        <v>7</v>
+      </c>
+      <c r="AB6" s="36">
+        <v>4</v>
+      </c>
+      <c r="AC6" s="36">
         <v>8</v>
       </c>
-      <c r="U6" s="36">
-        <v>3</v>
-      </c>
-      <c r="V6" s="36">
-        <v>4</v>
-      </c>
-      <c r="W6" s="36">
-        <v>7</v>
-      </c>
-      <c r="X6" s="36">
-        <v>5</v>
-      </c>
-      <c r="Y6" s="36">
-        <v>7</v>
-      </c>
-      <c r="Z6" s="36">
-        <v>4</v>
-      </c>
-      <c r="AA6" s="36">
-        <v>5</v>
-      </c>
-      <c r="AB6" s="36">
+      <c r="AD6" s="36">
+        <v>7</v>
+      </c>
+      <c r="AE6" s="37">
         <v>8</v>
       </c>
-      <c r="AC6" s="36">
-        <v>10</v>
-      </c>
-      <c r="AD6" s="37">
-        <v>9</v>
-      </c>
-      <c r="AE6" s="35">
-        <f>AD6-AC6</f>
-      </c>
-      <c r="AF6" s="35">
-        <f>AD6-B6</f>
+      <c r="AF6" s="34">
+        <f>AE6-AD6</f>
+      </c>
+      <c r="AG6" s="35">
+        <f>AE6-B6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINAS BAHIA</t>
+          <t xml:space="preserve">CENTRO OESTE</t>
         </is>
       </c>
       <c r="B7" s="36">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C7" s="36">
+        <v>21</v>
+      </c>
+      <c r="D7" s="36">
+        <v>18</v>
+      </c>
+      <c r="E7" s="36">
+        <v>20</v>
+      </c>
+      <c r="F7" s="36">
+        <v>17</v>
+      </c>
+      <c r="G7" s="36">
+        <v>17</v>
+      </c>
+      <c r="H7" s="36">
+        <v>18</v>
+      </c>
+      <c r="I7" s="36">
+        <v>18</v>
+      </c>
+      <c r="J7" s="36">
         <v>22</v>
       </c>
-      <c r="D7" s="36">
-        <v>22</v>
-      </c>
-      <c r="E7" s="36">
-        <v>22</v>
-      </c>
-      <c r="F7" s="36">
-        <v>23</v>
-      </c>
-      <c r="G7" s="36">
-        <v>25</v>
-      </c>
-      <c r="H7" s="36">
-        <v>24</v>
-      </c>
-      <c r="I7" s="36">
-        <v>28</v>
-      </c>
-      <c r="J7" s="36">
-        <v>30</v>
-      </c>
       <c r="K7" s="36">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="L7" s="36">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="M7" s="36">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N7" s="36">
+        <v>17</v>
+      </c>
+      <c r="O7" s="36">
+        <v>16</v>
+      </c>
+      <c r="P7" s="36">
+        <v>14</v>
+      </c>
+      <c r="Q7" s="36">
+        <v>16</v>
+      </c>
+      <c r="R7" s="36">
+        <v>15</v>
+      </c>
+      <c r="S7" s="36">
+        <v>15</v>
+      </c>
+      <c r="T7" s="36">
+        <v>14</v>
+      </c>
+      <c r="U7" s="36">
+        <v>8</v>
+      </c>
+      <c r="V7" s="36">
         <v>11</v>
       </c>
-      <c r="O7" s="36">
-        <v>8</v>
-      </c>
-      <c r="P7" s="36">
-        <v>10</v>
-      </c>
-      <c r="Q7" s="36">
-        <v>7</v>
-      </c>
-      <c r="R7" s="36">
-        <v>5</v>
-      </c>
-      <c r="S7" s="36">
-        <v>6</v>
-      </c>
-      <c r="T7" s="36">
-        <v>6</v>
-      </c>
-      <c r="U7" s="36">
-        <v>6</v>
-      </c>
-      <c r="V7" s="36">
-        <v>7</v>
-      </c>
       <c r="W7" s="36">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="X7" s="36">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="Y7" s="36">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="Z7" s="36">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AA7" s="36">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AB7" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC7" s="36">
-        <v>8</v>
-      </c>
-      <c r="AD7" s="37">
-        <v>7</v>
-      </c>
-      <c r="AE7" s="35">
-        <f>AD7-AC7</f>
-      </c>
-      <c r="AF7" s="35">
-        <f>AD7-B7</f>
+        <v>4</v>
+      </c>
+      <c r="AD7" s="36">
+        <v>3</v>
+      </c>
+      <c r="AE7" s="37">
+        <v>5</v>
+      </c>
+      <c r="AF7" s="34">
+        <f>AE7-AD7</f>
+      </c>
+      <c r="AG7" s="35">
+        <f>AE7-B7</f>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR NORTE</t>
+          <t xml:space="preserve">BK É FOGO LESTE</t>
         </is>
       </c>
       <c r="B8" s="36">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" s="36">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D8" s="36">
         <v>9</v>
       </c>
       <c r="E8" s="36">
+        <v>12</v>
+      </c>
+      <c r="F8" s="36">
+        <v>13</v>
+      </c>
+      <c r="G8" s="36">
+        <v>9</v>
+      </c>
+      <c r="H8" s="36">
+        <v>11</v>
+      </c>
+      <c r="I8" s="36">
+        <v>7</v>
+      </c>
+      <c r="J8" s="36">
         <v>6</v>
       </c>
-      <c r="F8" s="36">
-        <v>5</v>
-      </c>
-      <c r="G8" s="36">
-        <v>5</v>
-      </c>
-      <c r="H8" s="36">
-        <v>5</v>
-      </c>
-      <c r="I8" s="36">
+      <c r="K8" s="36">
         <v>6</v>
       </c>
-      <c r="J8" s="36">
-        <v>5</v>
-      </c>
-      <c r="K8" s="36">
-        <v>4</v>
-      </c>
       <c r="L8" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M8" s="36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N8" s="36">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="O8" s="36">
+        <v>13</v>
+      </c>
+      <c r="P8" s="36">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="36">
+        <v>10</v>
+      </c>
+      <c r="R8" s="36">
+        <v>13</v>
+      </c>
+      <c r="S8" s="36">
+        <v>10</v>
+      </c>
+      <c r="T8" s="36">
+        <v>10</v>
+      </c>
+      <c r="U8" s="36">
+        <v>7</v>
+      </c>
+      <c r="V8" s="36">
         <v>6</v>
       </c>
-      <c r="P8" s="36">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="36">
-        <v>5</v>
-      </c>
-      <c r="R8" s="36">
-        <v>5</v>
-      </c>
-      <c r="S8" s="36">
-        <v>6</v>
-      </c>
-      <c r="T8" s="36">
-        <v>5</v>
-      </c>
-      <c r="U8" s="36">
+      <c r="W8" s="36">
+        <v>5</v>
+      </c>
+      <c r="X8" s="36">
         <v>3</v>
       </c>
-      <c r="V8" s="36">
+      <c r="Y8" s="36">
         <v>3</v>
       </c>
-      <c r="W8" s="36">
+      <c r="Z8" s="36">
+        <v>2</v>
+      </c>
+      <c r="AA8" s="36">
+        <v>2</v>
+      </c>
+      <c r="AB8" s="36">
+        <v>2</v>
+      </c>
+      <c r="AC8" s="36">
         <v>3</v>
       </c>
-      <c r="X8" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y8" s="36">
-        <v>4</v>
-      </c>
-      <c r="Z8" s="36">
-        <v>4</v>
-      </c>
-      <c r="AA8" s="36">
-        <v>3</v>
-      </c>
-      <c r="AB8" s="36">
-        <v>5</v>
-      </c>
-      <c r="AC8" s="36">
-        <v>5</v>
-      </c>
-      <c r="AD8" s="37">
-        <v>5</v>
-      </c>
-      <c r="AE8" s="36">
-        <f>AD8-AC8</f>
-      </c>
-      <c r="AF8" s="35">
-        <f>AD8-B8</f>
+      <c r="AD8" s="36">
+        <v>4</v>
+      </c>
+      <c r="AE8" s="37">
+        <v>4</v>
+      </c>
+      <c r="AF8" s="36">
+        <f>AE8-AD8</f>
+      </c>
+      <c r="AG8" s="35">
+        <f>AE8-B8</f>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO LESTE</t>
+          <t xml:space="preserve">SUL</t>
         </is>
       </c>
       <c r="B9" s="36">
+        <v>35</v>
+      </c>
+      <c r="C9" s="36">
+        <v>33</v>
+      </c>
+      <c r="D9" s="36">
+        <v>33</v>
+      </c>
+      <c r="E9" s="36">
+        <v>35</v>
+      </c>
+      <c r="F9" s="36">
+        <v>39</v>
+      </c>
+      <c r="G9" s="36">
+        <v>32</v>
+      </c>
+      <c r="H9" s="36">
+        <v>27</v>
+      </c>
+      <c r="I9" s="36">
+        <v>25</v>
+      </c>
+      <c r="J9" s="36">
+        <v>20</v>
+      </c>
+      <c r="K9" s="36">
+        <v>18</v>
+      </c>
+      <c r="L9" s="36">
+        <v>14</v>
+      </c>
+      <c r="M9" s="36">
+        <v>14</v>
+      </c>
+      <c r="N9" s="36">
+        <v>11</v>
+      </c>
+      <c r="O9" s="36">
+        <v>10</v>
+      </c>
+      <c r="P9" s="36">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="36">
         <v>9</v>
       </c>
-      <c r="C9" s="36">
-        <v>7</v>
-      </c>
-      <c r="D9" s="36">
+      <c r="R9" s="36">
+        <v>7</v>
+      </c>
+      <c r="S9" s="36">
+        <v>5</v>
+      </c>
+      <c r="T9" s="36">
+        <v>8</v>
+      </c>
+      <c r="U9" s="36">
+        <v>3</v>
+      </c>
+      <c r="V9" s="36">
+        <v>4</v>
+      </c>
+      <c r="W9" s="36">
+        <v>7</v>
+      </c>
+      <c r="X9" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y9" s="36">
+        <v>7</v>
+      </c>
+      <c r="Z9" s="36">
+        <v>4</v>
+      </c>
+      <c r="AA9" s="36">
+        <v>5</v>
+      </c>
+      <c r="AB9" s="36">
+        <v>8</v>
+      </c>
+      <c r="AC9" s="36">
+        <v>10</v>
+      </c>
+      <c r="AD9" s="36">
         <v>9</v>
       </c>
-      <c r="E9" s="36">
-        <v>12</v>
-      </c>
-      <c r="F9" s="36">
-        <v>13</v>
-      </c>
-      <c r="G9" s="36">
-        <v>9</v>
-      </c>
-      <c r="H9" s="36">
-        <v>11</v>
-      </c>
-      <c r="I9" s="36">
-        <v>7</v>
-      </c>
-      <c r="J9" s="36">
-        <v>6</v>
-      </c>
-      <c r="K9" s="36">
-        <v>6</v>
-      </c>
-      <c r="L9" s="36">
-        <v>7</v>
-      </c>
-      <c r="M9" s="36">
-        <v>7</v>
-      </c>
-      <c r="N9" s="36">
-        <v>13</v>
-      </c>
-      <c r="O9" s="36">
-        <v>13</v>
-      </c>
-      <c r="P9" s="36">
-        <v>13</v>
-      </c>
-      <c r="Q9" s="36">
-        <v>10</v>
-      </c>
-      <c r="R9" s="36">
-        <v>13</v>
-      </c>
-      <c r="S9" s="36">
-        <v>10</v>
-      </c>
-      <c r="T9" s="36">
-        <v>10</v>
-      </c>
-      <c r="U9" s="36">
-        <v>7</v>
-      </c>
-      <c r="V9" s="36">
-        <v>6</v>
-      </c>
-      <c r="W9" s="36">
-        <v>5</v>
-      </c>
-      <c r="X9" s="36">
-        <v>3</v>
-      </c>
-      <c r="Y9" s="36">
-        <v>3</v>
-      </c>
-      <c r="Z9" s="36">
-        <v>2</v>
-      </c>
-      <c r="AA9" s="36">
-        <v>2</v>
-      </c>
-      <c r="AB9" s="36">
-        <v>2</v>
-      </c>
-      <c r="AC9" s="36">
-        <v>3</v>
-      </c>
-      <c r="AD9" s="37">
-        <v>4</v>
-      </c>
-      <c r="AE9" s="34">
-        <f>AD9-AC9</f>
+      <c r="AE9" s="37">
+        <v>4</v>
       </c>
       <c r="AF9" s="35">
-        <f>AD9-B9</f>
+        <f>AE9-AD9</f>
+      </c>
+      <c r="AG9" s="35">
+        <f>AE9-B9</f>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO OESTE</t>
+          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
         </is>
       </c>
       <c r="B10" s="36">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C10" s="36">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="D10" s="36">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E10" s="36">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="F10" s="36">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G10" s="36">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H10" s="36">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I10" s="36">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="J10" s="36">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="K10" s="36">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L10" s="36">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M10" s="36">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="N10" s="36">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="O10" s="36">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="P10" s="36">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="36">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="R10" s="36">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="S10" s="36">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="T10" s="36">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="U10" s="36">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V10" s="36">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="W10" s="36">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="X10" s="36">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Y10" s="36">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="Z10" s="36">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AA10" s="36">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AB10" s="36">
+        <v>2</v>
+      </c>
+      <c r="AC10" s="36">
+        <v>1</v>
+      </c>
+      <c r="AD10" s="36">
+        <v>1</v>
+      </c>
+      <c r="AE10" s="37">
         <v>3</v>
       </c>
-      <c r="AC10" s="36">
-        <v>4</v>
-      </c>
-      <c r="AD10" s="37">
-        <v>3</v>
-      </c>
-      <c r="AE10" s="35">
-        <f>AD10-AC10</f>
-      </c>
-      <c r="AF10" s="35">
-        <f>AD10-B10</f>
+      <c r="AF10" s="34">
+        <f>AE10-AD10</f>
+      </c>
+      <c r="AG10" s="35">
+        <f>AE10-B10</f>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP INTERIOR SUL</t>
+          <t xml:space="preserve">SP SUL</t>
         </is>
       </c>
       <c r="B11" s="36">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C11" s="36">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D11" s="36">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E11" s="36">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F11" s="36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G11" s="36">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H11" s="36">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="I11" s="36">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="J11" s="36">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="K11" s="36">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="L11" s="36">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M11" s="36">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="N11" s="36">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O11" s="36">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P11" s="36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="36">
         <v>6</v>
       </c>
       <c r="R11" s="36">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S11" s="36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T11" s="36">
         <v>8</v>
       </c>
       <c r="U11" s="36">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="V11" s="36">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="W11" s="36">
         <v>4</v>
       </c>
       <c r="X11" s="36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Y11" s="36">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="36">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB11" s="36">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC11" s="36">
-        <v>6</v>
-      </c>
-      <c r="AD11" s="37">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="36">
         <v>2</v>
       </c>
-      <c r="AE11" s="35">
-        <f>AD11-AC11</f>
-      </c>
-      <c r="AF11" s="35">
-        <f>AD11-B11</f>
+      <c r="AE11" s="37">
+        <v>3</v>
+      </c>
+      <c r="AF11" s="34">
+        <f>AE11-AD11</f>
+      </c>
+      <c r="AG11" s="35">
+        <f>AE11-B11</f>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SP SUL</t>
+          <t xml:space="preserve">SP INTERIOR NORTE</t>
         </is>
       </c>
       <c r="B12" s="36">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C12" s="36">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D12" s="36">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E12" s="36">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="F12" s="36">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="G12" s="36">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H12" s="36">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="I12" s="36">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="J12" s="36">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="K12" s="36">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="L12" s="36">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M12" s="36">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="N12" s="36">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O12" s="36">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="P12" s="36">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="36">
+        <v>5</v>
+      </c>
+      <c r="R12" s="36">
+        <v>5</v>
+      </c>
+      <c r="S12" s="36">
         <v>6</v>
       </c>
-      <c r="R12" s="36">
-        <v>5</v>
-      </c>
-      <c r="S12" s="36">
-        <v>7</v>
-      </c>
       <c r="T12" s="36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U12" s="36">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="V12" s="36">
         <v>3</v>
       </c>
       <c r="W12" s="36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X12" s="36">
+        <v>4</v>
+      </c>
+      <c r="Y12" s="36">
+        <v>4</v>
+      </c>
+      <c r="Z12" s="36">
+        <v>4</v>
+      </c>
+      <c r="AA12" s="36">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="36">
+        <v>5</v>
+      </c>
+      <c r="AC12" s="36">
+        <v>5</v>
+      </c>
+      <c r="AD12" s="36">
+        <v>5</v>
+      </c>
+      <c r="AE12" s="37">
         <v>2</v>
       </c>
-      <c r="Y12" s="36">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="36">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="36">
-        <v>2</v>
-      </c>
-      <c r="AB12" s="36">
-        <v>1</v>
-      </c>
-      <c r="AC12" s="36">
-        <v>1</v>
-      </c>
-      <c r="AD12" s="37">
-        <v>2</v>
-      </c>
-      <c r="AE12" s="34">
-        <f>AD12-AC12</f>
-      </c>
       <c r="AF12" s="35">
-        <f>AD12-B12</f>
+        <f>AE12-AD12</f>
+      </c>
+      <c r="AG12" s="35">
+        <f>AE12-B12</f>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO CENTRO LITORAL</t>
+          <t xml:space="preserve">BK É FOGO NORTE</t>
         </is>
       </c>
       <c r="B13" s="36">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C13" s="36">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D13" s="36">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E13" s="36">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F13" s="36">
+        <v>7</v>
+      </c>
+      <c r="G13" s="36">
+        <v>6</v>
+      </c>
+      <c r="H13" s="36">
+        <v>8</v>
+      </c>
+      <c r="I13" s="36">
+        <v>11</v>
+      </c>
+      <c r="J13" s="36">
+        <v>11</v>
+      </c>
+      <c r="K13" s="36">
+        <v>12</v>
+      </c>
+      <c r="L13" s="36">
+        <v>4</v>
+      </c>
+      <c r="M13" s="36">
+        <v>4</v>
+      </c>
+      <c r="N13" s="36">
         <v>2</v>
-      </c>
-      <c r="G13" s="36">
-        <v>4</v>
-      </c>
-      <c r="H13" s="36">
-        <v>2</v>
-      </c>
-      <c r="I13" s="36">
-        <v>4</v>
-      </c>
-      <c r="J13" s="36">
-        <v>3</v>
-      </c>
-      <c r="K13" s="36">
-        <v>0</v>
-      </c>
-      <c r="L13" s="36">
-        <v>0</v>
-      </c>
-      <c r="M13" s="36">
-        <v>0</v>
-      </c>
-      <c r="N13" s="36">
-        <v>1</v>
       </c>
       <c r="O13" s="36">
         <v>3</v>
       </c>
       <c r="P13" s="36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="36">
         <v>2</v>
       </c>
       <c r="R13" s="36">
+        <v>1</v>
+      </c>
+      <c r="S13" s="36">
+        <v>1</v>
+      </c>
+      <c r="T13" s="36">
+        <v>1</v>
+      </c>
+      <c r="U13" s="36">
+        <v>1</v>
+      </c>
+      <c r="V13" s="36">
+        <v>4</v>
+      </c>
+      <c r="W13" s="36">
         <v>2</v>
       </c>
-      <c r="S13" s="36">
+      <c r="X13" s="36">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="36">
         <v>3</v>
-      </c>
-      <c r="T13" s="36">
-        <v>2</v>
-      </c>
-      <c r="U13" s="36">
-        <v>4</v>
-      </c>
-      <c r="V13" s="36">
-        <v>4</v>
-      </c>
-      <c r="W13" s="36">
-        <v>3</v>
-      </c>
-      <c r="X13" s="36">
-        <v>4</v>
-      </c>
-      <c r="Y13" s="36">
-        <v>4</v>
       </c>
       <c r="Z13" s="36">
         <v>3</v>
@@ -1457,119 +1490,125 @@
         <v>2</v>
       </c>
       <c r="AB13" s="36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC13" s="36">
-        <v>1</v>
-      </c>
-      <c r="AD13" s="37">
-        <v>1</v>
-      </c>
-      <c r="AE13" s="36">
-        <f>AD13-AC13</f>
-      </c>
-      <c r="AF13" s="35">
-        <f>AD13-B13</f>
+        <v>0</v>
+      </c>
+      <c r="AD13" s="36">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="37">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="36">
+        <f>AE13-AD13</f>
+      </c>
+      <c r="AG13" s="35">
+        <f>AE13-B13</f>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BK É FOGO NORTE</t>
+          <t xml:space="preserve">SP INTERIOR SUL</t>
         </is>
       </c>
       <c r="B14" s="36">
+        <v>12</v>
+      </c>
+      <c r="C14" s="36">
+        <v>11</v>
+      </c>
+      <c r="D14" s="36">
+        <v>10</v>
+      </c>
+      <c r="E14" s="36">
+        <v>10</v>
+      </c>
+      <c r="F14" s="36">
+        <v>12</v>
+      </c>
+      <c r="G14" s="36">
+        <v>11</v>
+      </c>
+      <c r="H14" s="36">
+        <v>12</v>
+      </c>
+      <c r="I14" s="36">
+        <v>7</v>
+      </c>
+      <c r="J14" s="36">
+        <v>6</v>
+      </c>
+      <c r="K14" s="36">
+        <v>7</v>
+      </c>
+      <c r="L14" s="36">
+        <v>7</v>
+      </c>
+      <c r="M14" s="36">
+        <v>7</v>
+      </c>
+      <c r="N14" s="36">
+        <v>10</v>
+      </c>
+      <c r="O14" s="36">
+        <v>7</v>
+      </c>
+      <c r="P14" s="36">
         <v>8</v>
       </c>
-      <c r="C14" s="36">
-        <v>7</v>
-      </c>
-      <c r="D14" s="36">
-        <v>9</v>
-      </c>
-      <c r="E14" s="36">
-        <v>14</v>
-      </c>
-      <c r="F14" s="36">
-        <v>7</v>
-      </c>
-      <c r="G14" s="36">
+      <c r="Q14" s="36">
         <v>6</v>
       </c>
-      <c r="H14" s="36">
+      <c r="R14" s="36">
+        <v>6</v>
+      </c>
+      <c r="S14" s="36">
+        <v>5</v>
+      </c>
+      <c r="T14" s="36">
         <v>8</v>
       </c>
-      <c r="I14" s="36">
+      <c r="U14" s="36">
         <v>11</v>
       </c>
-      <c r="J14" s="36">
-        <v>11</v>
-      </c>
-      <c r="K14" s="36">
-        <v>12</v>
-      </c>
-      <c r="L14" s="36">
-        <v>4</v>
-      </c>
-      <c r="M14" s="36">
-        <v>4</v>
-      </c>
-      <c r="N14" s="36">
+      <c r="V14" s="36">
+        <v>8</v>
+      </c>
+      <c r="W14" s="36">
+        <v>4</v>
+      </c>
+      <c r="X14" s="36">
+        <v>5</v>
+      </c>
+      <c r="Y14" s="36">
+        <v>6</v>
+      </c>
+      <c r="Z14" s="36">
+        <v>5</v>
+      </c>
+      <c r="AA14" s="36">
+        <v>4</v>
+      </c>
+      <c r="AB14" s="36">
+        <v>6</v>
+      </c>
+      <c r="AC14" s="36">
+        <v>6</v>
+      </c>
+      <c r="AD14" s="36">
         <v>2</v>
       </c>
-      <c r="O14" s="36">
-        <v>3</v>
-      </c>
-      <c r="P14" s="36">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="36">
-        <v>2</v>
-      </c>
-      <c r="R14" s="36">
-        <v>1</v>
-      </c>
-      <c r="S14" s="36">
-        <v>1</v>
-      </c>
-      <c r="T14" s="36">
-        <v>1</v>
-      </c>
-      <c r="U14" s="36">
-        <v>1</v>
-      </c>
-      <c r="V14" s="36">
-        <v>4</v>
-      </c>
-      <c r="W14" s="36">
-        <v>2</v>
-      </c>
-      <c r="X14" s="36">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="36">
-        <v>3</v>
-      </c>
-      <c r="Z14" s="36">
-        <v>3</v>
-      </c>
-      <c r="AA14" s="36">
-        <v>2</v>
-      </c>
-      <c r="AB14" s="36">
-        <v>1</v>
-      </c>
-      <c r="AC14" s="36">
-        <v>0</v>
-      </c>
-      <c r="AD14" s="37">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="36">
-        <f>AD14-AC14</f>
+      <c r="AE14" s="37">
+        <v>0</v>
       </c>
       <c r="AF14" s="35">
-        <f>AD14-B14</f>
+        <f>AE14-AD14</f>
+      </c>
+      <c r="AG14" s="35">
+        <f>AE14-B14</f>
       </c>
     </row>
     <row r="15">
@@ -1665,11 +1704,14 @@
       <c r="AD15" s="38">
         <f>SUM(AD4:AD14)</f>
       </c>
-      <c r="AE15" s="41">
-        <f>AD15-AC15</f>
+      <c r="AE15" s="38">
+        <f>SUM(AE4:AE14)</f>
       </c>
       <c r="AF15" s="41">
-        <f>AD15-B15</f>
+        <f>AE15-AD15</f>
+      </c>
+      <c r="AG15" s="41">
+        <f>AE15-B15</f>
       </c>
     </row>
     <row r="16">
@@ -1833,6 +1875,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="AG16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1924,15 +1971,18 @@
       <c r="AC17" s="36">
         <v>14</v>
       </c>
-      <c r="AD17" s="37">
+      <c r="AD17" s="36">
         <v>39</v>
       </c>
-      <c r="AE17" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AE17" s="37">
+        <v>38</v>
       </c>
       <c r="AF17" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AG17" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2028,15 +2078,18 @@
       <c r="AC18" s="36">
         <v>19</v>
       </c>
-      <c r="AD18" s="37">
+      <c r="AD18" s="36">
         <v>26</v>
       </c>
-      <c r="AE18" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AE18" s="37">
+        <v>32</v>
       </c>
       <c r="AF18" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AG18" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2132,15 +2185,18 @@
       <c r="AC19" s="36">
         <f>AC18-AC17</f>
       </c>
-      <c r="AD19" s="37">
+      <c r="AD19" s="36">
         <f>AD18-AD17</f>
       </c>
-      <c r="AE19" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AE19" s="37">
+        <f>AE18-AE17</f>
       </c>
       <c r="AF19" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AG19" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -2236,15 +2292,18 @@
       <c r="AC20" s="36">
         <v>7</v>
       </c>
-      <c r="AD20" s="37">
+      <c r="AD20" s="36">
         <v>6</v>
       </c>
-      <c r="AE20" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="AE20" s="37">
+        <v>4</v>
       </c>
       <c r="AF20" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AG20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>